<commit_message>
Updated GRN Functions and added 10 new PO with Free of cost scenarios
Updated GRN Functions and added 10 new PO with Free of cost scenarios
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\GitHub - Repos\roadmap\testdata\"/>
     </mc:Choice>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2447" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2421" uniqueCount="196">
   <si>
     <t>Purchase Order &amp; GRN</t>
   </si>
@@ -643,9 +643,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.00_);[Red]\(0.00\)"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -1082,7 +1083,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1325,6 +1326,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1604,12 +1606,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="9.85546875"/>
-    <col min="2" max="2" customWidth="true" style="97" width="25.5703125"/>
-    <col min="3" max="3" customWidth="true" style="97" width="26.0"/>
-    <col min="4" max="19" style="97" width="9.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="9.85546875"/>
+    <col min="1" max="1" width="9.85546875" style="97"/>
+    <col min="2" max="2" width="25.5703125" style="97" customWidth="1"/>
+    <col min="3" max="3" width="26" style="97" customWidth="1"/>
+    <col min="4" max="19" width="9.85546875" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.85546875" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -2346,7 +2348,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -4716,7 +4718,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -7086,8 +7088,8 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="16.0"/>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -9461,7 +9463,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -11489,14 +11491,14 @@
       <c r="F23" s="26">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>174</v>
       </c>
       <c r="H23" s="26">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>167</v>
       </c>
       <c r="J23" s="26">
@@ -11835,8 +11837,8 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.5703125"/>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="2" max="2" width="26.5703125" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -13864,14 +13866,14 @@
       <c r="F23" s="26">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>174</v>
       </c>
       <c r="H23" s="26">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>167</v>
       </c>
       <c r="J23" s="26">
@@ -14210,7 +14212,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -16238,14 +16240,14 @@
       <c r="F23" s="26">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>174</v>
       </c>
       <c r="H23" s="26">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>167</v>
       </c>
       <c r="J23" s="26">
@@ -16578,7 +16580,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -18606,14 +18608,14 @@
       <c r="F23" s="26">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>174</v>
       </c>
       <c r="H23" s="26">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>167</v>
       </c>
       <c r="J23" s="26">
@@ -18952,7 +18954,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" customWidth="true" width="9.42578125"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
@@ -20980,14 +20982,14 @@
       <c r="F23" s="26">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>174</v>
       </c>
       <c r="H23" s="26">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>167</v>
       </c>
       <c r="J23" s="26">
@@ -23351,14 +23353,14 @@
       <c r="F23" s="26">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>174</v>
       </c>
       <c r="H23" s="26">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>167</v>
       </c>
       <c r="J23" s="26">
@@ -23697,12 +23699,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="9.85546875"/>
-    <col min="2" max="2" customWidth="true" style="97" width="25.5703125"/>
-    <col min="3" max="3" customWidth="true" style="97" width="26.0"/>
-    <col min="4" max="19" style="97" width="9.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="9.85546875"/>
+    <col min="1" max="1" width="9.85546875" style="97"/>
+    <col min="2" max="2" width="25.5703125" style="97" customWidth="1"/>
+    <col min="3" max="3" width="26" style="97" customWidth="1"/>
+    <col min="4" max="19" width="9.85546875" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.85546875" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -24439,12 +24441,12 @@
   <dimension ref="A1:BQ17"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="8.7109375"/>
-    <col min="2" max="2" customWidth="true" style="97" width="19.140625"/>
-    <col min="3" max="3" customWidth="true" style="97" width="25.85546875"/>
-    <col min="4" max="19" style="97" width="8.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="8.7109375"/>
+    <col min="1" max="1" width="8.7109375" style="97"/>
+    <col min="2" max="2" width="19.140625" style="97" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" style="97" customWidth="1"/>
+    <col min="4" max="19" width="8.7109375" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.7109375" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -26141,12 +26143,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="8.7109375"/>
-    <col min="2" max="2" customWidth="true" style="97" width="21.140625"/>
-    <col min="3" max="3" customWidth="true" style="97" width="21.28515625"/>
-    <col min="4" max="19" style="97" width="8.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="8.7109375"/>
+    <col min="1" max="1" width="8.7109375" style="97"/>
+    <col min="2" max="2" width="21.140625" style="97" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" style="97" customWidth="1"/>
+    <col min="4" max="19" width="8.7109375" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.7109375" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -26552,8 +26554,8 @@
         <f>F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" s="55" t="s">
-        <v>102</v>
+      <c r="I4" s="55">
+        <v>0</v>
       </c>
       <c r="J4" s="62">
         <v>8</v>
@@ -26563,35 +26565,35 @@
       </c>
       <c r="L4" s="62">
         <f>IF(OR(I4=0,I4="0"),0,H4)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="M4" s="62">
         <f>ROUND(L4*I4%,3)</f>
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="N4" s="62">
         <f>H4-M4</f>
-        <v>237.5</v>
+        <v>250</v>
       </c>
       <c r="O4" s="62">
         <f>ROUND(N4*J4%,3)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P4" s="62">
         <f>ROUND(N4-O4,2)</f>
-        <v>218.5</v>
+        <v>230</v>
       </c>
       <c r="Q4" s="62">
         <f>ROUND(P4*K4%,2)</f>
-        <v>10.93</v>
+        <v>11.5</v>
       </c>
       <c r="R4" s="73">
         <f>ROUND(M4+O4+Q4,3)</f>
-        <v>42.43</v>
-      </c>
-      <c r="S4" s="73">
+        <v>31.5</v>
+      </c>
+      <c r="S4" s="122">
         <f>(H4-R4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T4" s="62">
         <v>88363222</v>
@@ -26628,7 +26630,7 @@
       </c>
       <c r="AC4" s="78">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD4" s="73">
         <v>120</v>
@@ -26648,7 +26650,7 @@
       </c>
       <c r="AI4" s="73">
         <f>S4*$M2</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ4" s="73">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -26667,7 +26669,7 @@
       </c>
       <c r="AN4" s="73">
         <f>ROUND(AI4/AM4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AO4" s="73">
         <f>AJ4/AM4</f>
@@ -26682,7 +26684,7 @@
       </c>
       <c r="AR4" s="73">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AS4" s="85" t="s">
         <v>98</v>
@@ -26702,7 +26704,7 @@
       </c>
       <c r="AX4" s="89">
         <f>AR4</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AY4" s="86">
         <f>AU4+AW4</f>
@@ -26710,7 +26712,7 @@
       </c>
       <c r="AZ4" s="86">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),3)</f>
-        <v>41.515000000000001</v>
+        <v>42.061</v>
       </c>
       <c r="BA4" s="91"/>
       <c r="BB4" s="91" t="s">
@@ -26742,7 +26744,7 @@
       </c>
       <c r="BO4" s="86">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>41.515000000000001</v>
+        <v>41.787999999999997</v>
       </c>
       <c r="BP4" s="95">
         <f>ROUND(BN4+AW4,3)</f>
@@ -26777,11 +26779,11 @@
       <c r="Q5" s="61"/>
       <c r="R5" s="74">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>42.43</v>
+        <v>31.5</v>
       </c>
       <c r="S5" s="67">
         <f t="shared" si="0"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T5" s="74"/>
       <c r="U5" s="74"/>
@@ -26806,7 +26808,7 @@
       </c>
       <c r="AC5" s="79">
         <f t="shared" si="1"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD5" s="80">
         <f t="shared" si="1"/>
@@ -26827,7 +26829,7 @@
       </c>
       <c r="AI5" s="80">
         <f t="shared" si="2"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ5" s="80">
         <f t="shared" si="2"/>
@@ -26878,6 +26880,7 @@
     <hyperlink ref="AS4" r:id="rId1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -26886,12 +26889,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="8.7109375"/>
-    <col min="2" max="2" customWidth="true" style="97" width="21.140625"/>
-    <col min="3" max="3" customWidth="true" style="97" width="21.28515625"/>
-    <col min="4" max="19" style="97" width="8.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="8.7109375"/>
+    <col min="1" max="1" width="8.7109375" style="97"/>
+    <col min="2" max="2" width="21.140625" style="97" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" style="97" customWidth="1"/>
+    <col min="4" max="19" width="8.7109375" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.7109375" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -27297,8 +27300,8 @@
         <f>F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" s="55" t="s">
-        <v>102</v>
+      <c r="I4" s="55">
+        <v>0</v>
       </c>
       <c r="J4" s="62">
         <v>8</v>
@@ -27308,35 +27311,35 @@
       </c>
       <c r="L4" s="62">
         <f>IF(OR(I4=0,I4="0"),0,H4)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="M4" s="62">
         <f>ROUND(L4*I4%,3)</f>
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="N4" s="62">
         <f>H4-M4</f>
-        <v>237.5</v>
+        <v>250</v>
       </c>
       <c r="O4" s="62">
         <f>ROUND(N4*J4%,3)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P4" s="62">
         <f>ROUND(N4-O4,2)</f>
-        <v>218.5</v>
+        <v>230</v>
       </c>
       <c r="Q4" s="62">
         <f>ROUND(P4*K4%,2)</f>
-        <v>10.93</v>
+        <v>11.5</v>
       </c>
       <c r="R4" s="73">
         <f>ROUND(M4+O4+Q4,3)</f>
-        <v>42.43</v>
-      </c>
-      <c r="S4" s="73">
+        <v>31.5</v>
+      </c>
+      <c r="S4" s="122">
         <f>(H4-R4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T4" s="62">
         <v>88363222</v>
@@ -27373,7 +27376,7 @@
       </c>
       <c r="AC4" s="78">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD4" s="73">
         <v>120</v>
@@ -27393,7 +27396,7 @@
       </c>
       <c r="AI4" s="73">
         <f>S4*$M2</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ4" s="73">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -27412,7 +27415,7 @@
       </c>
       <c r="AN4" s="73">
         <f>ROUND(AI4/AM4,5)</f>
-        <v>124.542</v>
+        <v>131.1</v>
       </c>
       <c r="AO4" s="73">
         <f>AJ4/AM4</f>
@@ -27427,7 +27430,7 @@
       </c>
       <c r="AR4" s="73">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>124.542</v>
+        <v>131.1</v>
       </c>
       <c r="AS4" s="85" t="s">
         <v>98</v>
@@ -27447,7 +27450,7 @@
       </c>
       <c r="AX4" s="89">
         <f>AR4</f>
-        <v>124.542</v>
+        <v>131.1</v>
       </c>
       <c r="AY4" s="86">
         <f>AU4+AW4</f>
@@ -27455,7 +27458,7 @@
       </c>
       <c r="AZ4" s="86">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),3)</f>
-        <v>49.817999999999998</v>
+        <v>50.473999999999997</v>
       </c>
       <c r="BA4" s="91"/>
       <c r="BB4" s="91" t="s">
@@ -27487,7 +27490,7 @@
       </c>
       <c r="BO4" s="86">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>43.59075</v>
+        <v>43.754750000000001</v>
       </c>
       <c r="BP4" s="95">
         <f>ROUND(BN4+AW4,3)</f>
@@ -27522,11 +27525,11 @@
       <c r="Q5" s="61"/>
       <c r="R5" s="74">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>42.43</v>
+        <v>31.5</v>
       </c>
       <c r="S5" s="67">
         <f t="shared" si="0"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T5" s="74"/>
       <c r="U5" s="74"/>
@@ -27551,7 +27554,7 @@
       </c>
       <c r="AC5" s="79">
         <f t="shared" si="1"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD5" s="80">
         <f t="shared" si="1"/>
@@ -27572,7 +27575,7 @@
       </c>
       <c r="AI5" s="80">
         <f t="shared" si="2"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ5" s="80">
         <f t="shared" si="2"/>
@@ -27631,12 +27634,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="8.7109375"/>
-    <col min="2" max="2" customWidth="true" style="97" width="23.42578125"/>
-    <col min="3" max="3" customWidth="true" style="97" width="29.42578125"/>
-    <col min="4" max="19" style="97" width="8.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="8.7109375"/>
+    <col min="1" max="1" width="8.7109375" style="97"/>
+    <col min="2" max="2" width="23.42578125" style="97" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" style="97" customWidth="1"/>
+    <col min="4" max="19" width="8.7109375" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.7109375" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -28042,8 +28045,8 @@
         <f>F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" s="55" t="s">
-        <v>102</v>
+      <c r="I4" s="55">
+        <v>0</v>
       </c>
       <c r="J4" s="62">
         <v>8</v>
@@ -28053,35 +28056,35 @@
       </c>
       <c r="L4" s="62">
         <f>IF(OR(I4=0,I4="0"),0,H4)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="M4" s="62">
         <f>ROUND(L4*I4%,3)</f>
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="N4" s="62">
         <f>H4-M4</f>
-        <v>237.5</v>
+        <v>250</v>
       </c>
       <c r="O4" s="62">
         <f>ROUND(N4*J4%,3)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P4" s="62">
         <f>ROUND(N4-O4,2)</f>
-        <v>218.5</v>
+        <v>230</v>
       </c>
       <c r="Q4" s="62">
         <f>ROUND(P4*K4%,2)</f>
-        <v>10.93</v>
+        <v>11.5</v>
       </c>
       <c r="R4" s="73">
         <f>ROUND(M4+O4+Q4,3)</f>
-        <v>42.43</v>
-      </c>
-      <c r="S4" s="73">
+        <v>31.5</v>
+      </c>
+      <c r="S4" s="122">
         <f>(H4-R4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T4" s="62">
         <v>88363222</v>
@@ -28118,7 +28121,7 @@
       </c>
       <c r="AC4" s="78">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD4" s="73">
         <v>120</v>
@@ -28138,7 +28141,7 @@
       </c>
       <c r="AI4" s="73">
         <f>S4*$M2</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ4" s="73">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -28157,7 +28160,7 @@
       </c>
       <c r="AN4" s="73">
         <f>ROUND(AI4/AM4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AO4" s="73">
         <f>AJ4/AM4</f>
@@ -28172,7 +28175,7 @@
       </c>
       <c r="AR4" s="73">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AS4" s="85" t="s">
         <v>98</v>
@@ -28192,7 +28195,7 @@
       </c>
       <c r="AX4" s="89">
         <f>AR4</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AY4" s="86">
         <f>AU4+AW4</f>
@@ -28200,7 +28203,7 @@
       </c>
       <c r="AZ4" s="86">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),3)</f>
-        <v>41.515000000000001</v>
+        <v>42.061</v>
       </c>
       <c r="BA4" s="91"/>
       <c r="BB4" s="91" t="s">
@@ -28232,7 +28235,7 @@
       </c>
       <c r="BO4" s="86">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>41.515000000000001</v>
+        <v>41.787999999999997</v>
       </c>
       <c r="BP4" s="95">
         <f>ROUND(BN4+AW4,3)</f>
@@ -28267,11 +28270,11 @@
       <c r="Q5" s="61"/>
       <c r="R5" s="74">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>42.43</v>
+        <v>31.5</v>
       </c>
       <c r="S5" s="67">
         <f t="shared" si="0"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T5" s="74"/>
       <c r="U5" s="74"/>
@@ -28296,7 +28299,7 @@
       </c>
       <c r="AC5" s="79">
         <f t="shared" si="1"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD5" s="80">
         <f t="shared" si="1"/>
@@ -28317,7 +28320,7 @@
       </c>
       <c r="AI5" s="80">
         <f t="shared" si="2"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ5" s="80">
         <f t="shared" si="2"/>
@@ -28376,12 +28379,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="8.7109375"/>
-    <col min="2" max="2" customWidth="true" style="97" width="27.28515625"/>
-    <col min="3" max="3" customWidth="true" style="97" width="25.42578125"/>
-    <col min="4" max="19" style="97" width="8.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="8.7109375"/>
+    <col min="1" max="1" width="8.7109375" style="97"/>
+    <col min="2" max="2" width="27.28515625" style="97" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" style="97" customWidth="1"/>
+    <col min="4" max="19" width="8.7109375" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.7109375" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -28787,8 +28790,8 @@
         <f>F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" s="55" t="s">
-        <v>102</v>
+      <c r="I4" s="55">
+        <v>0</v>
       </c>
       <c r="J4" s="62">
         <v>8</v>
@@ -28798,35 +28801,35 @@
       </c>
       <c r="L4" s="62">
         <f>IF(OR(I4=0,I4="0"),0,H4)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="M4" s="62">
         <f>ROUND(L4*I4%,3)</f>
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="N4" s="62">
         <f>H4-M4</f>
-        <v>237.5</v>
+        <v>250</v>
       </c>
       <c r="O4" s="62">
         <f>ROUND(N4*J4%,3)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P4" s="62">
         <f>ROUND(N4-O4,2)</f>
-        <v>218.5</v>
+        <v>230</v>
       </c>
       <c r="Q4" s="62">
         <f>ROUND(P4*K4%,2)</f>
-        <v>10.93</v>
+        <v>11.5</v>
       </c>
       <c r="R4" s="73">
         <f>ROUND(M4+O4+Q4,3)</f>
-        <v>42.43</v>
-      </c>
-      <c r="S4" s="73">
+        <v>31.5</v>
+      </c>
+      <c r="S4" s="122">
         <f>(H4-R4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T4" s="62">
         <v>88363222</v>
@@ -28863,7 +28866,7 @@
       </c>
       <c r="AC4" s="78">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD4" s="73">
         <v>120</v>
@@ -28883,7 +28886,7 @@
       </c>
       <c r="AI4" s="73">
         <f>S4*$M2</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ4" s="73">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -28902,7 +28905,7 @@
       </c>
       <c r="AN4" s="73">
         <f>ROUND(AI4/AM4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AO4" s="73">
         <f>AJ4/AM4</f>
@@ -28917,7 +28920,7 @@
       </c>
       <c r="AR4" s="73">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AS4" s="85" t="s">
         <v>98</v>
@@ -28937,7 +28940,7 @@
       </c>
       <c r="AX4" s="89">
         <f>AR4</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AY4" s="86">
         <f>AU4+AW4</f>
@@ -28945,7 +28948,7 @@
       </c>
       <c r="AZ4" s="90">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),3)</f>
-        <v>41.515000000000001</v>
+        <v>42.243000000000002</v>
       </c>
       <c r="BA4" s="91"/>
       <c r="BB4" s="91" t="s">
@@ -28977,7 +28980,7 @@
       </c>
       <c r="BO4" s="86">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>41.515000000000001</v>
+        <v>41.878999999999998</v>
       </c>
       <c r="BP4" s="95">
         <f>ROUND(BN4+AW4,3)</f>
@@ -29012,11 +29015,11 @@
       <c r="Q5" s="61"/>
       <c r="R5" s="74">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>42.43</v>
+        <v>31.5</v>
       </c>
       <c r="S5" s="67">
         <f t="shared" si="0"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T5" s="74"/>
       <c r="U5" s="74"/>
@@ -29041,7 +29044,7 @@
       </c>
       <c r="AC5" s="79">
         <f t="shared" si="1"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD5" s="80">
         <f t="shared" si="1"/>
@@ -29062,7 +29065,7 @@
       </c>
       <c r="AI5" s="80">
         <f t="shared" si="2"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ5" s="80">
         <f t="shared" si="2"/>
@@ -29121,12 +29124,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="97" width="8.7109375"/>
-    <col min="2" max="2" customWidth="true" style="97" width="27.28515625"/>
-    <col min="3" max="3" customWidth="true" style="97" width="25.42578125"/>
-    <col min="4" max="19" style="97" width="8.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="97" width="10.140625"/>
-    <col min="21" max="16384" style="97" width="8.7109375"/>
+    <col min="1" max="1" width="8.7109375" style="97"/>
+    <col min="2" max="2" width="27.28515625" style="97" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" style="97" customWidth="1"/>
+    <col min="4" max="19" width="8.7109375" style="97"/>
+    <col min="20" max="20" width="10.140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.7109375" style="97"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -29532,8 +29535,8 @@
         <f>F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" s="55" t="s">
-        <v>102</v>
+      <c r="I4" s="55">
+        <v>0</v>
       </c>
       <c r="J4" s="62">
         <v>8</v>
@@ -29543,35 +29546,35 @@
       </c>
       <c r="L4" s="62">
         <f>IF(OR(I4=0,I4="0"),0,H4)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="M4" s="62">
         <f>ROUND(L4*I4%,3)</f>
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="N4" s="62">
         <f>H4-M4</f>
-        <v>237.5</v>
+        <v>250</v>
       </c>
       <c r="O4" s="62">
         <f>ROUND(N4*J4%,3)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P4" s="62">
         <f>ROUND(N4-O4,2)</f>
-        <v>218.5</v>
+        <v>230</v>
       </c>
       <c r="Q4" s="62">
         <f>ROUND(P4*K4%,2)</f>
-        <v>10.93</v>
+        <v>11.5</v>
       </c>
       <c r="R4" s="73">
         <f>ROUND(M4+O4+Q4,3)</f>
-        <v>42.43</v>
-      </c>
-      <c r="S4" s="73">
+        <v>31.5</v>
+      </c>
+      <c r="S4" s="122">
         <f>(H4-R4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T4" s="62">
         <v>88363222</v>
@@ -29608,7 +29611,7 @@
       </c>
       <c r="AC4" s="78">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD4" s="73">
         <v>120</v>
@@ -29628,7 +29631,7 @@
       </c>
       <c r="AI4" s="73">
         <f>S4*$M2</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ4" s="73">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -29647,7 +29650,7 @@
       </c>
       <c r="AN4" s="73">
         <f>ROUND(AI4/AM4,5)</f>
-        <v>124.542</v>
+        <v>131.1</v>
       </c>
       <c r="AO4" s="73">
         <f>AJ4/AM4</f>
@@ -29662,7 +29665,7 @@
       </c>
       <c r="AR4" s="73">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>124.542</v>
+        <v>131.1</v>
       </c>
       <c r="AS4" s="85" t="s">
         <v>98</v>
@@ -29682,7 +29685,7 @@
       </c>
       <c r="AX4" s="89">
         <f>AR4</f>
-        <v>124.542</v>
+        <v>131.1</v>
       </c>
       <c r="AY4" s="86">
         <f>AU4+AW4</f>
@@ -29690,7 +29693,7 @@
       </c>
       <c r="AZ4" s="90">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),3)</f>
-        <v>53.375999999999998</v>
+        <v>54.313000000000002</v>
       </c>
       <c r="BA4" s="91"/>
       <c r="BB4" s="91" t="s">
@@ -29722,7 +29725,7 @@
       </c>
       <c r="BO4" s="86">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>44.480249999999998</v>
+        <v>44.714500000000001</v>
       </c>
       <c r="BP4" s="95">
         <f>ROUND(BN4+AW4,3)</f>
@@ -29757,11 +29760,11 @@
       <c r="Q5" s="61"/>
       <c r="R5" s="74">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>42.43</v>
+        <v>31.5</v>
       </c>
       <c r="S5" s="67">
         <f t="shared" si="0"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T5" s="74"/>
       <c r="U5" s="74"/>
@@ -29786,7 +29789,7 @@
       </c>
       <c r="AC5" s="79">
         <f t="shared" si="1"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AD5" s="80">
         <f t="shared" si="1"/>
@@ -29807,7 +29810,7 @@
       </c>
       <c r="AI5" s="80">
         <f t="shared" si="2"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ5" s="80">
         <f t="shared" si="2"/>
@@ -29866,17 +29869,17 @@
   <dimension ref="A1:BQ18"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="55" width="8.85546875"/>
-    <col min="2" max="2" customWidth="true" style="55" width="28.0"/>
-    <col min="3" max="3" customWidth="true" style="55" width="23.0"/>
-    <col min="4" max="12" style="55" width="8.85546875"/>
-    <col min="13" max="13" customWidth="true" style="55" width="9.140625"/>
-    <col min="14" max="14" customWidth="true" style="55" width="13.85546875"/>
-    <col min="15" max="19" style="55" width="8.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" style="55" width="10.140625"/>
-    <col min="21" max="63" style="55" width="8.85546875"/>
-    <col min="64" max="64" customWidth="true" style="55" width="11.0"/>
-    <col min="65" max="16384" style="55" width="8.85546875"/>
+    <col min="1" max="1" width="8.85546875" style="55"/>
+    <col min="2" max="2" width="28" style="55" customWidth="1"/>
+    <col min="3" max="3" width="23" style="55" customWidth="1"/>
+    <col min="4" max="12" width="8.85546875" style="55"/>
+    <col min="13" max="13" width="9.140625" style="55" customWidth="1"/>
+    <col min="14" max="14" width="13.85546875" style="55" customWidth="1"/>
+    <col min="15" max="19" width="8.85546875" style="55"/>
+    <col min="20" max="20" width="10.140625" style="55" bestFit="1" customWidth="1"/>
+    <col min="21" max="63" width="8.85546875" style="55"/>
+    <col min="64" max="64" width="11" style="55" customWidth="1"/>
+    <col min="65" max="16384" width="8.85546875" style="55"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -30282,8 +30285,8 @@
         <f>F4*G4</f>
         <v>250</v>
       </c>
-      <c r="I4" s="55" t="s">
-        <v>102</v>
+      <c r="I4" s="55">
+        <v>0</v>
       </c>
       <c r="J4" s="62">
         <v>8</v>
@@ -30293,35 +30296,35 @@
       </c>
       <c r="L4" s="62">
         <f>IF(OR(I4=0,I4="0"),0,H4)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="M4" s="62">
         <f>ROUND(L4*I4%,3)</f>
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="N4" s="62">
         <f>H4-M4</f>
-        <v>237.5</v>
+        <v>250</v>
       </c>
       <c r="O4" s="62">
         <f>ROUND(N4*J4%,3)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P4" s="62">
         <f>ROUND(N4-O4,2)</f>
-        <v>218.5</v>
+        <v>230</v>
       </c>
       <c r="Q4" s="62">
         <f>ROUND(P4*K4%,2)</f>
-        <v>10.93</v>
+        <v>11.5</v>
       </c>
       <c r="R4" s="73">
         <f>ROUND(M4+O4+Q4,3)</f>
-        <v>42.43</v>
-      </c>
-      <c r="S4" s="73">
+        <v>31.5</v>
+      </c>
+      <c r="S4" s="122">
         <f>(H4-R4)</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T4" s="62">
         <v>88363222</v>
@@ -30331,11 +30334,11 @@
       </c>
       <c r="V4" s="62">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
-        <v>18.68</v>
+        <v>19.670000000000002</v>
       </c>
       <c r="W4" s="62">
         <f>IF($C$2=1,ROUND((((S4*U4)/100)/2),2),0)</f>
-        <v>18.68</v>
+        <v>19.670000000000002</v>
       </c>
       <c r="X4" s="62">
         <f>IF($C$2=2,ROUND(((S4*U4)/100),2),0)</f>
@@ -30354,11 +30357,11 @@
       </c>
       <c r="AB4" s="62">
         <f>V4+W4+X4+Y4+AA4</f>
-        <v>37.36</v>
+        <v>39.340000000000003</v>
       </c>
       <c r="AC4" s="78">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>244.93</v>
+        <v>257.84000000000003</v>
       </c>
       <c r="AD4" s="73">
         <v>120</v>
@@ -30378,7 +30381,7 @@
       </c>
       <c r="AI4" s="73">
         <f>S4*$M2</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ4" s="73">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -30397,7 +30400,7 @@
       </c>
       <c r="AN4" s="73">
         <f>ROUND(AI4/AM4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AO4" s="73">
         <f>AJ4/AM4</f>
@@ -30412,7 +30415,7 @@
       </c>
       <c r="AR4" s="73">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AS4" s="85" t="s">
         <v>98</v>
@@ -30432,7 +30435,7 @@
       </c>
       <c r="AX4" s="89">
         <f>AR4</f>
-        <v>41.514000000000003</v>
+        <v>43.7</v>
       </c>
       <c r="AY4" s="86">
         <f>AU4+AW4</f>
@@ -30440,7 +30443,7 @@
       </c>
       <c r="AZ4" s="90">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),3)</f>
-        <v>41.515000000000001</v>
+        <v>42.243000000000002</v>
       </c>
       <c r="BA4" s="91"/>
       <c r="BB4" s="91" t="s">
@@ -30472,7 +30475,7 @@
       </c>
       <c r="BO4" s="86">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>41.515000000000001</v>
+        <v>41.878999999999998</v>
       </c>
       <c r="BP4" s="95">
         <f>ROUND(BN4+AW4,3)</f>
@@ -30507,21 +30510,21 @@
       <c r="Q5" s="61"/>
       <c r="R5" s="74">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>42.43</v>
+        <v>31.5</v>
       </c>
       <c r="S5" s="67">
         <f t="shared" si="0"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="T5" s="74"/>
       <c r="U5" s="74"/>
       <c r="V5" s="75">
         <f t="shared" si="0"/>
-        <v>18.68</v>
+        <v>19.670000000000002</v>
       </c>
       <c r="W5" s="75">
         <f t="shared" si="0"/>
-        <v>18.68</v>
+        <v>19.670000000000002</v>
       </c>
       <c r="X5" s="75">
         <f t="shared" si="0"/>
@@ -30532,11 +30535,11 @@
       <c r="AA5" s="75"/>
       <c r="AB5" s="74">
         <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
-        <v>37.36</v>
+        <v>39.340000000000003</v>
       </c>
       <c r="AC5" s="79">
         <f t="shared" si="1"/>
-        <v>244.93</v>
+        <v>257.84000000000003</v>
       </c>
       <c r="AD5" s="80">
         <f t="shared" si="1"/>
@@ -30557,7 +30560,7 @@
       </c>
       <c r="AI5" s="80">
         <f t="shared" si="2"/>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="AJ5" s="80">
         <f t="shared" si="2"/>
@@ -30766,7 +30769,7 @@
       <c r="H8" s="110"/>
       <c r="I8" s="111">
         <f>R5</f>
-        <v>42.43</v>
+        <v>31.5</v>
       </c>
       <c r="J8" s="111"/>
       <c r="K8" s="63"/>
@@ -30854,7 +30857,7 @@
       <c r="H9" s="110"/>
       <c r="I9" s="111">
         <f>S5</f>
-        <v>207.57</v>
+        <v>218.5</v>
       </c>
       <c r="J9" s="111"/>
       <c r="K9" s="63"/>
@@ -30938,7 +30941,7 @@
       <c r="H10" s="110"/>
       <c r="I10" s="111">
         <f>AB5</f>
-        <v>37.36</v>
+        <v>39.340000000000003</v>
       </c>
       <c r="J10" s="111"/>
       <c r="K10" s="63"/>
@@ -31022,7 +31025,7 @@
       <c r="H11" s="110"/>
       <c r="I11" s="112">
         <f>I9+I10</f>
-        <v>244.93</v>
+        <v>257.84000000000003</v>
       </c>
       <c r="J11" s="112"/>
       <c r="K11" s="63"/>

</xml_diff>

<commit_message>
Added New Test scenarios "From PR to PO with FOC"
Added New Test scenarios "From PR to PO with FOC"
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="2" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="ImportPoToGRNUDGeneralSameUOM" sheetId="11" r:id="rId1"/>
@@ -1284,6 +1284,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1296,9 +1297,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1307,6 +1305,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1326,7 +1327,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1688,10 +1688,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -2352,37 +2352,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -3906,14 +3906,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -4054,10 +4054,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -4722,37 +4722,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -6276,14 +6276,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -6424,10 +6424,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -7093,37 +7093,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -8647,14 +8647,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -8795,10 +8795,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -9467,37 +9467,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -11021,14 +11021,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -11169,10 +11169,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -11842,37 +11842,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -13396,14 +13396,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -13544,10 +13544,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -14216,37 +14216,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -15770,14 +15770,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="119" t="s">
+      <c r="B19" s="120" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="120"/>
-      <c r="D19" s="120"/>
-      <c r="E19" s="120"/>
-      <c r="F19" s="120"/>
-      <c r="G19" s="121"/>
+      <c r="C19" s="121"/>
+      <c r="D19" s="121"/>
+      <c r="E19" s="121"/>
+      <c r="F19" s="121"/>
+      <c r="G19" s="122"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -15918,10 +15918,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -16584,37 +16584,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -18138,14 +18138,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -18286,10 +18286,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -18958,37 +18958,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -20512,14 +20512,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -20660,10 +20660,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -21329,37 +21329,37 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:69" ht="18.75">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="117" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+      <c r="G1" s="117"/>
+      <c r="H1" s="117"/>
+      <c r="I1" s="117"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="117"/>
+      <c r="L1" s="117"/>
+      <c r="M1" s="117"/>
+      <c r="N1" s="117"/>
+      <c r="O1" s="117"/>
+      <c r="P1" s="117"/>
+      <c r="Q1" s="117"/>
+      <c r="R1" s="117"/>
+      <c r="S1" s="117"/>
+      <c r="T1" s="117"/>
+      <c r="U1" s="117"/>
+      <c r="V1" s="117"/>
+      <c r="W1" s="117"/>
+      <c r="X1" s="117"/>
+      <c r="Y1" s="117"/>
+      <c r="Z1" s="117"/>
+      <c r="AA1" s="117"/>
+      <c r="AB1" s="117"/>
+      <c r="AC1" s="117"/>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
@@ -22883,14 +22883,14 @@
     </row>
     <row r="19" spans="1:69">
       <c r="A19" s="16"/>
-      <c r="B19" s="117" t="s">
+      <c r="B19" s="118" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="117"/>
-      <c r="G19" s="117"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="17">
         <f>SUM(H4:H18)</f>
         <v>71856.759999999995</v>
@@ -23031,10 +23031,10 @@
       <c r="BQ20" s="27"/>
     </row>
     <row r="21" spans="1:69">
-      <c r="A21" s="118" t="s">
+      <c r="A21" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="118"/>
+      <c r="B21" s="119"/>
       <c r="C21" s="20">
         <v>3</v>
       </c>
@@ -23781,10 +23781,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -24523,10 +24523,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -25248,15 +25248,15 @@
       <c r="D7" s="63"/>
       <c r="E7" s="63"/>
       <c r="F7" s="63"/>
-      <c r="G7" s="109" t="s">
+      <c r="G7" s="110" t="s">
         <v>103</v>
       </c>
-      <c r="H7" s="110"/>
-      <c r="I7" s="111">
+      <c r="H7" s="111"/>
+      <c r="I7" s="112">
         <f>H5</f>
         <v>750</v>
       </c>
-      <c r="J7" s="111"/>
+      <c r="J7" s="112"/>
       <c r="K7" s="63"/>
       <c r="L7" s="63"/>
       <c r="M7" s="113" t="s">
@@ -25330,15 +25330,15 @@
       <c r="D8" s="63"/>
       <c r="E8" s="63"/>
       <c r="F8" s="63"/>
-      <c r="G8" s="109" t="s">
+      <c r="G8" s="110" t="s">
         <v>107</v>
       </c>
-      <c r="H8" s="110"/>
-      <c r="I8" s="111">
+      <c r="H8" s="111"/>
+      <c r="I8" s="112">
         <f>R5</f>
         <v>127.28</v>
       </c>
-      <c r="J8" s="111"/>
+      <c r="J8" s="112"/>
       <c r="K8" s="63"/>
       <c r="L8" s="63"/>
       <c r="M8" s="71">
@@ -25418,15 +25418,15 @@
       <c r="D9" s="63"/>
       <c r="E9" s="63"/>
       <c r="F9" s="63"/>
-      <c r="G9" s="109" t="s">
+      <c r="G9" s="110" t="s">
         <v>110</v>
       </c>
-      <c r="H9" s="110"/>
-      <c r="I9" s="111">
+      <c r="H9" s="111"/>
+      <c r="I9" s="112">
         <f>S5</f>
         <v>622.72</v>
       </c>
-      <c r="J9" s="111"/>
+      <c r="J9" s="112"/>
       <c r="K9" s="63"/>
       <c r="L9" s="63"/>
       <c r="M9" s="61">
@@ -25502,15 +25502,15 @@
       <c r="D10" s="63"/>
       <c r="E10" s="63"/>
       <c r="F10" s="63"/>
-      <c r="G10" s="109" t="s">
+      <c r="G10" s="110" t="s">
         <v>112</v>
       </c>
-      <c r="H10" s="110"/>
-      <c r="I10" s="111">
+      <c r="H10" s="111"/>
+      <c r="I10" s="112">
         <f>AB5</f>
         <v>0</v>
       </c>
-      <c r="J10" s="111"/>
+      <c r="J10" s="112"/>
       <c r="K10" s="63"/>
       <c r="L10" s="63"/>
       <c r="M10" s="61">
@@ -25586,15 +25586,15 @@
       <c r="D11" s="63"/>
       <c r="E11" s="63"/>
       <c r="F11" s="63"/>
-      <c r="G11" s="109" t="s">
+      <c r="G11" s="110" t="s">
         <v>114</v>
       </c>
-      <c r="H11" s="110"/>
-      <c r="I11" s="112">
+      <c r="H11" s="111"/>
+      <c r="I11" s="116">
         <f>I9+I10</f>
         <v>622.72</v>
       </c>
-      <c r="J11" s="112"/>
+      <c r="J11" s="116"/>
       <c r="K11" s="63"/>
       <c r="L11" s="63"/>
       <c r="M11" s="63"/>
@@ -26118,18 +26118,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:J11"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="M7:P7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="I8:J8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:J11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="AS4" r:id="rId1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
@@ -26225,10 +26225,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -26591,7 +26591,7 @@
         <f>ROUND(M4+O4+Q4,3)</f>
         <v>31.5</v>
       </c>
-      <c r="S4" s="122">
+      <c r="S4" s="108">
         <f>(H4-R4)</f>
         <v>218.5</v>
       </c>
@@ -26599,7 +26599,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="62">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="62">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -26971,10 +26971,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -27337,7 +27337,7 @@
         <f>ROUND(M4+O4+Q4,3)</f>
         <v>31.5</v>
       </c>
-      <c r="S4" s="122">
+      <c r="S4" s="108">
         <f>(H4-R4)</f>
         <v>218.5</v>
       </c>
@@ -27716,10 +27716,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -28082,7 +28082,7 @@
         <f>ROUND(M4+O4+Q4,3)</f>
         <v>31.5</v>
       </c>
-      <c r="S4" s="122">
+      <c r="S4" s="108">
         <f>(H4-R4)</f>
         <v>218.5</v>
       </c>
@@ -28461,10 +28461,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -28827,7 +28827,7 @@
         <f>ROUND(M4+O4+Q4,3)</f>
         <v>31.5</v>
       </c>
-      <c r="S4" s="122">
+      <c r="S4" s="108">
         <f>(H4-R4)</f>
         <v>218.5</v>
       </c>
@@ -29206,10 +29206,10 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
         <v>3</v>
       </c>
@@ -29572,7 +29572,7 @@
         <f>ROUND(M4+O4+Q4,3)</f>
         <v>31.5</v>
       </c>
-      <c r="S4" s="122">
+      <c r="S4" s="108">
         <f>(H4-R4)</f>
         <v>218.5</v>
       </c>
@@ -29872,10 +29872,13 @@
     <col min="1" max="1" width="8.85546875" style="55"/>
     <col min="2" max="2" width="28" style="55" customWidth="1"/>
     <col min="3" max="3" width="23" style="55" customWidth="1"/>
-    <col min="4" max="12" width="8.85546875" style="55"/>
+    <col min="4" max="11" width="8.85546875" style="55"/>
+    <col min="12" max="12" width="15.7109375" style="55" customWidth="1"/>
     <col min="13" max="13" width="9.140625" style="55" customWidth="1"/>
     <col min="14" max="14" width="13.85546875" style="55" customWidth="1"/>
-    <col min="15" max="19" width="8.85546875" style="55"/>
+    <col min="15" max="15" width="11.28515625" style="55" customWidth="1"/>
+    <col min="16" max="16" width="17.85546875" style="55" customWidth="1"/>
+    <col min="17" max="19" width="8.85546875" style="55"/>
     <col min="20" max="20" width="10.140625" style="55" bestFit="1" customWidth="1"/>
     <col min="21" max="63" width="8.85546875" style="55"/>
     <col min="64" max="64" width="11" style="55" customWidth="1"/>
@@ -29956,12 +29959,12 @@
       <c r="BQ1" s="87"/>
     </row>
     <row r="2" spans="1:69">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="108"/>
+      <c r="B2" s="109"/>
       <c r="C2" s="58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" s="59" t="s">
         <v>2</v>
@@ -30322,7 +30325,7 @@
         <f>ROUND(M4+O4+Q4,3)</f>
         <v>31.5</v>
       </c>
-      <c r="S4" s="122">
+      <c r="S4" s="108">
         <f>(H4-R4)</f>
         <v>218.5</v>
       </c>
@@ -30330,15 +30333,15 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="62">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="62">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
-        <v>19.670000000000002</v>
+        <v>0</v>
       </c>
       <c r="W4" s="62">
         <f>IF($C$2=1,ROUND((((S4*U4)/100)/2),2),0)</f>
-        <v>19.670000000000002</v>
+        <v>0</v>
       </c>
       <c r="X4" s="62">
         <f>IF($C$2=2,ROUND(((S4*U4)/100),2),0)</f>
@@ -30357,11 +30360,11 @@
       </c>
       <c r="AB4" s="62">
         <f>V4+W4+X4+Y4+AA4</f>
-        <v>39.340000000000003</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="78">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>257.84000000000003</v>
+        <v>218.5</v>
       </c>
       <c r="AD4" s="73">
         <v>120</v>
@@ -30520,11 +30523,11 @@
       <c r="U5" s="74"/>
       <c r="V5" s="75">
         <f t="shared" si="0"/>
-        <v>19.670000000000002</v>
+        <v>0</v>
       </c>
       <c r="W5" s="75">
         <f t="shared" si="0"/>
-        <v>19.670000000000002</v>
+        <v>0</v>
       </c>
       <c r="X5" s="75">
         <f t="shared" si="0"/>
@@ -30535,11 +30538,11 @@
       <c r="AA5" s="75"/>
       <c r="AB5" s="74">
         <f t="shared" ref="AB5:AE5" si="1">SUM(AB4:AB4)</f>
-        <v>39.340000000000003</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="79">
         <f t="shared" si="1"/>
-        <v>257.84000000000003</v>
+        <v>218.5</v>
       </c>
       <c r="AD5" s="80">
         <f t="shared" si="1"/>
@@ -30681,15 +30684,15 @@
       <c r="D7" s="63"/>
       <c r="E7" s="63"/>
       <c r="F7" s="63"/>
-      <c r="G7" s="109" t="s">
+      <c r="G7" s="110" t="s">
         <v>103</v>
       </c>
-      <c r="H7" s="110"/>
-      <c r="I7" s="111">
+      <c r="H7" s="111"/>
+      <c r="I7" s="112">
         <f>H5</f>
         <v>250</v>
       </c>
-      <c r="J7" s="111"/>
+      <c r="J7" s="112"/>
       <c r="K7" s="63"/>
       <c r="L7" s="63"/>
       <c r="M7" s="113" t="s">
@@ -30763,15 +30766,15 @@
       <c r="D8" s="63"/>
       <c r="E8" s="63"/>
       <c r="F8" s="63"/>
-      <c r="G8" s="109" t="s">
+      <c r="G8" s="110" t="s">
         <v>107</v>
       </c>
-      <c r="H8" s="110"/>
-      <c r="I8" s="111">
+      <c r="H8" s="111"/>
+      <c r="I8" s="112">
         <f>R5</f>
         <v>31.5</v>
       </c>
-      <c r="J8" s="111"/>
+      <c r="J8" s="112"/>
       <c r="K8" s="63"/>
       <c r="L8" s="63"/>
       <c r="M8" s="71">
@@ -30851,15 +30854,15 @@
       <c r="D9" s="63"/>
       <c r="E9" s="63"/>
       <c r="F9" s="63"/>
-      <c r="G9" s="109" t="s">
+      <c r="G9" s="110" t="s">
         <v>110</v>
       </c>
-      <c r="H9" s="110"/>
-      <c r="I9" s="111">
+      <c r="H9" s="111"/>
+      <c r="I9" s="112">
         <f>S5</f>
         <v>218.5</v>
       </c>
-      <c r="J9" s="111"/>
+      <c r="J9" s="112"/>
       <c r="K9" s="63"/>
       <c r="L9" s="63"/>
       <c r="M9" s="61">
@@ -30935,15 +30938,15 @@
       <c r="D10" s="63"/>
       <c r="E10" s="63"/>
       <c r="F10" s="63"/>
-      <c r="G10" s="109" t="s">
+      <c r="G10" s="110" t="s">
         <v>112</v>
       </c>
-      <c r="H10" s="110"/>
-      <c r="I10" s="111">
+      <c r="H10" s="111"/>
+      <c r="I10" s="112">
         <f>AB5</f>
-        <v>39.340000000000003</v>
-      </c>
-      <c r="J10" s="111"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="112"/>
       <c r="K10" s="63"/>
       <c r="L10" s="63"/>
       <c r="M10" s="61">
@@ -31019,15 +31022,15 @@
       <c r="D11" s="63"/>
       <c r="E11" s="63"/>
       <c r="F11" s="63"/>
-      <c r="G11" s="109" t="s">
+      <c r="G11" s="110" t="s">
         <v>114</v>
       </c>
-      <c r="H11" s="110"/>
-      <c r="I11" s="112">
+      <c r="H11" s="111"/>
+      <c r="I11" s="116">
         <f>I9+I10</f>
-        <v>257.84000000000003</v>
-      </c>
-      <c r="J11" s="112"/>
+        <v>218.5</v>
+      </c>
+      <c r="J11" s="116"/>
       <c r="K11" s="63"/>
       <c r="L11" s="63"/>
       <c r="M11" s="63"/>
@@ -31622,18 +31625,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:J11"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="M7:P7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="I8:J8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:J11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="AS4" r:id="rId1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>

</xml_diff>

<commit_message>
Fixes in purchase module scenarios test data
Fixes in purchase module scenarios test data
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2417" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2777" uniqueCount="219">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -665,6 +665,42 @@
   </si>
   <si>
     <t>209.665</t>
+  </si>
+  <si>
+    <t>1035</t>
+  </si>
+  <si>
+    <t>1338.31746</t>
+  </si>
+  <si>
+    <t>1085</t>
+  </si>
+  <si>
+    <t>1133.33646</t>
+  </si>
+  <si>
+    <t>1095</t>
+  </si>
+  <si>
+    <t>1124.12375</t>
+  </si>
+  <si>
+    <t>1150</t>
+  </si>
+  <si>
+    <t>1216.94021</t>
+  </si>
+  <si>
+    <t>1105</t>
+  </si>
+  <si>
+    <t>1115.07779</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>8156.97779</t>
   </si>
 </sst>
 </file>
@@ -5270,6 +5306,8 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
+      <c r="AU4" s="1"/>
+      <c r="AV4" s="1"/>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>5</v>
@@ -5308,10 +5346,10 @@
       <c r="BL4" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="BM4" s="1" t="s">
+      <c r="BM4" t="s" s="1">
         <v>114</v>
       </c>
-      <c r="BN4" s="1" t="s">
+      <c r="BN4" t="s" s="1">
         <v>114</v>
       </c>
       <c r="BO4" s="28">
@@ -7720,11 +7758,11 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AU4" t="s" s="1">
         <v>114</v>
       </c>
-      <c r="AV4" s="1" t="s">
-        <v>188</v>
+      <c r="AV4" t="s" s="1">
+        <v>164</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -7764,11 +7802,11 @@
       <c r="BL4" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="BM4" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>190</v>
+      <c r="BM4" t="s" s="1">
+        <v>214</v>
+      </c>
+      <c r="BN4" t="s" s="1">
+        <v>213</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -9221,11 +9259,11 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AU4" t="s" s="1">
         <v>114</v>
       </c>
-      <c r="AV4" s="1" t="s">
-        <v>188</v>
+      <c r="AV4" t="s" s="1">
+        <v>164</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -9265,11 +9303,11 @@
       <c r="BL4" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="BM4" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>196</v>
+      <c r="BM4" t="s" s="1">
+        <v>216</v>
+      </c>
+      <c r="BN4" t="s" s="1">
+        <v>215</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -11755,6 +11793,8 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
+      <c r="AU4" s="1"/>
+      <c r="AV4" s="1"/>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>1</v>
@@ -11793,10 +11833,10 @@
       <c r="BL4" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="BM4" s="1" t="s">
+      <c r="BM4" t="s" s="1">
         <v>114</v>
       </c>
-      <c r="BN4" s="1" t="s">
+      <c r="BN4" t="s" s="1">
         <v>114</v>
       </c>
       <c r="BO4" s="28">
@@ -12496,10 +12536,10 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AU4" t="s" s="1">
         <v>114</v>
       </c>
-      <c r="AV4" s="1" t="s">
+      <c r="AV4" t="s" s="1">
         <v>201</v>
       </c>
       <c r="AW4" s="28">
@@ -12540,10 +12580,10 @@
       <c r="BL4" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="BM4" s="1" t="s">
+      <c r="BM4" t="s" s="1">
         <v>202</v>
       </c>
-      <c r="BN4" s="1" t="s">
+      <c r="BN4" t="s" s="1">
         <v>203</v>
       </c>
       <c r="BO4" s="28">
@@ -13247,10 +13287,10 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AU4" t="s" s="1">
         <v>114</v>
       </c>
-      <c r="AV4" s="1" t="s">
+      <c r="AV4" t="s" s="1">
         <v>201</v>
       </c>
       <c r="AW4" s="28">
@@ -13291,10 +13331,10 @@
       <c r="BL4" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="BM4" s="1" t="s">
+      <c r="BM4" t="s" s="1">
         <v>205</v>
       </c>
-      <c r="BN4" s="1" t="s">
+      <c r="BN4" t="s" s="1">
         <v>206</v>
       </c>
       <c r="BO4" s="28">
@@ -18129,7 +18169,7 @@
         <v>114</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="AW23" s="103">
         <f>AM23</f>
@@ -18170,10 +18210,10 @@
         <v>120</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>137</v>
+        <v>218</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>138</v>
+        <v>217</v>
       </c>
       <c r="BO23" s="103">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
Updated Import GRN File
Updated Import GRN File
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="16" activeTab="17"/>
+    <workbookView windowWidth="20490" windowHeight="7620" firstSheet="7" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="ImportDirectGRNUDGeneralSameUOM" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2392" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="214">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -403,13 +403,13 @@
     <t>RMS</t>
   </si>
   <si>
-    <t>RM WH</t>
+    <t>RM KD</t>
   </si>
   <si>
-    <t>6454.29073</t>
+    <t>8230.87693</t>
   </si>
   <si>
-    <t>106</t>
+    <t>26</t>
   </si>
   <si>
     <t>VD Asbl. Val.</t>
@@ -425,9 +425,6 @@
   </si>
   <si>
     <t>ITEM-GWL-SERVICE-02</t>
-  </si>
-  <si>
-    <t>INS WH-1</t>
   </si>
   <si>
     <t>116.334</t>
@@ -467,9 +464,6 @@
   </si>
   <si>
     <t>8415</t>
-  </si>
-  <si>
-    <t>RM KD</t>
   </si>
   <si>
     <t>8213.55001</t>
@@ -521,6 +515,9 @@
   </si>
   <si>
     <t>Item Desc</t>
+  </si>
+  <si>
+    <t>INS WH-1</t>
   </si>
   <si>
     <t>110</t>
@@ -626,6 +623,69 @@
   </si>
   <si>
     <t>209.665</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>8208.45001</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>8189.01334</t>
+  </si>
+  <si>
+    <t>19792.25</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>8500</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>8186.02307</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>8166.79999</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>8150.13999</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>8135.56249</t>
+  </si>
+  <si>
+    <t>19791.96667</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>36</t>
   </si>
 </sst>
 </file>
@@ -1667,7 +1727,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="148">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49">
       <alignment vertical="center"/>
@@ -1933,6 +1993,9 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1991,9 +2054,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2334,79 +2394,79 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BR24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.5727272727273" customWidth="1"/>
-    <col min="2" max="2" width="21.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="27.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5727272727273" customWidth="1"/>
-    <col min="48" max="48" width="21.1454545454545" customWidth="1"/>
-    <col min="49" max="49" width="11.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="16.7181818181818" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4272727272727" customWidth="1"/>
-    <col min="53" max="53" width="18.8545454545455" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="15.5727272727273" customWidth="1"/>
-    <col min="56" max="56" width="14.2818181818182" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2818181818182" customWidth="1"/>
-    <col min="59" max="59" width="13.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="12.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="21.8545454545455" customWidth="1"/>
-    <col min="63" max="63" width="30.5727272727273" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="9.57272727272727" customWidth="1"/>
-    <col min="70" max="70" width="5.42727272727273" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="25.5714285714286"/>
+    <col min="2" max="2" customWidth="true" width="21.8571428571429"/>
+    <col min="3" max="3" customWidth="true" width="27.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5714285714286"/>
+    <col min="48" max="48" customWidth="true" width="21.1428571428571"/>
+    <col min="49" max="49" customWidth="true" width="11.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="16.7142857142857"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="53" max="53" customWidth="true" width="18.8571428571429"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="15.5714285714286"/>
+    <col min="56" max="56" customWidth="true" width="14.2857142857143"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2857142857143"/>
+    <col min="59" max="59" customWidth="true" width="13.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="12.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="21.8571428571429"/>
+    <col min="63" max="63" customWidth="true" width="30.5714285714286"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="9.57142857142857"/>
+    <col min="70" max="70" customWidth="true" width="5.42857142857143"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -2479,7 +2539,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -2552,7 +2612,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -3815,7 +3875,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:70">
+    <row r="18" ht="15.75" spans="1:70">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -3899,7 +3959,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:70">
+    <row r="19" ht="15.75" spans="1:70">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -3971,56 +4031,56 @@
       <c r="BP19" s="65"/>
       <c r="BQ19" s="65"/>
     </row>
-    <row r="20" s="131" customFormat="1" spans="1:70">
-      <c r="A20" s="133" t="s">
+    <row r="20" s="132" customFormat="1" spans="1:70">
+      <c r="A20" s="134" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="133"/>
-      <c r="C20" s="133"/>
-      <c r="D20" s="133"/>
-      <c r="E20" s="133"/>
-      <c r="F20" s="133"/>
-      <c r="G20" s="133"/>
-      <c r="H20" s="133"/>
-      <c r="I20" s="134"/>
-      <c r="J20" s="134"/>
-      <c r="K20" s="134"/>
-      <c r="L20" s="134"/>
-      <c r="M20" s="134"/>
-      <c r="N20" s="134"/>
-      <c r="O20" s="134"/>
-      <c r="P20" s="134"/>
-      <c r="Q20" s="134"/>
-      <c r="R20" s="133"/>
-      <c r="S20" s="133"/>
-      <c r="T20" s="133"/>
-      <c r="U20" s="133"/>
-      <c r="V20" s="133"/>
-      <c r="W20" s="133"/>
-      <c r="X20" s="133"/>
-      <c r="Y20" s="133"/>
-      <c r="Z20" s="133"/>
-      <c r="AA20" s="133"/>
-      <c r="AB20" s="133"/>
-      <c r="AC20" s="133"/>
-      <c r="AD20" s="133"/>
-      <c r="AE20" s="133"/>
-      <c r="AF20" s="133"/>
-      <c r="AG20" s="133"/>
-      <c r="AH20" s="133"/>
-      <c r="AI20" s="133"/>
-      <c r="AJ20" s="133"/>
-      <c r="AK20" s="133"/>
-      <c r="AL20" s="133"/>
-      <c r="AM20" s="133"/>
-      <c r="AN20" s="133"/>
-      <c r="AO20" s="133"/>
-      <c r="AP20" s="133"/>
-      <c r="AQ20" s="133"/>
-      <c r="AR20" s="133"/>
-      <c r="AS20" s="135"/>
+      <c r="B20" s="134"/>
+      <c r="C20" s="134"/>
+      <c r="D20" s="134"/>
+      <c r="E20" s="134"/>
+      <c r="F20" s="134"/>
+      <c r="G20" s="134"/>
+      <c r="H20" s="134"/>
+      <c r="I20" s="135"/>
+      <c r="J20" s="135"/>
+      <c r="K20" s="135"/>
+      <c r="L20" s="135"/>
+      <c r="M20" s="135"/>
+      <c r="N20" s="135"/>
+      <c r="O20" s="135"/>
+      <c r="P20" s="135"/>
+      <c r="Q20" s="135"/>
+      <c r="R20" s="134"/>
+      <c r="S20" s="134"/>
+      <c r="T20" s="134"/>
+      <c r="U20" s="134"/>
+      <c r="V20" s="134"/>
+      <c r="W20" s="134"/>
+      <c r="X20" s="134"/>
+      <c r="Y20" s="134"/>
+      <c r="Z20" s="134"/>
+      <c r="AA20" s="134"/>
+      <c r="AB20" s="134"/>
+      <c r="AC20" s="134"/>
+      <c r="AD20" s="134"/>
+      <c r="AE20" s="134"/>
+      <c r="AF20" s="134"/>
+      <c r="AG20" s="134"/>
+      <c r="AH20" s="134"/>
+      <c r="AI20" s="134"/>
+      <c r="AJ20" s="134"/>
+      <c r="AK20" s="134"/>
+      <c r="AL20" s="134"/>
+      <c r="AM20" s="134"/>
+      <c r="AN20" s="134"/>
+      <c r="AO20" s="134"/>
+      <c r="AP20" s="134"/>
+      <c r="AQ20" s="134"/>
+      <c r="AR20" s="134"/>
+      <c r="AS20" s="136"/>
     </row>
-    <row r="21" s="131" customFormat="1" spans="1:70">
+    <row r="21" s="132" customFormat="1" spans="1:70">
       <c r="A21" s="89" t="s">
         <v>43</v>
       </c>
@@ -4089,33 +4149,33 @@
       <c r="AP21" s="91"/>
       <c r="AQ21" s="91"/>
       <c r="AR21" s="91"/>
-      <c r="AS21" s="136"/>
-      <c r="AT21" s="137"/>
-      <c r="AU21" s="137"/>
-      <c r="AV21" s="137"/>
-      <c r="AW21" s="137"/>
-      <c r="AX21" s="137"/>
-      <c r="AY21" s="137"/>
-      <c r="AZ21" s="137"/>
-      <c r="BA21" s="137"/>
-      <c r="BB21" s="137"/>
-      <c r="BC21" s="137"/>
-      <c r="BD21" s="137"/>
-      <c r="BE21" s="137"/>
-      <c r="BF21" s="137"/>
-      <c r="BG21" s="137"/>
-      <c r="BH21" s="137"/>
-      <c r="BI21" s="137"/>
-      <c r="BJ21" s="137"/>
-      <c r="BK21" s="137"/>
-      <c r="BL21" s="137"/>
-      <c r="BM21" s="137"/>
-      <c r="BN21" s="137"/>
-      <c r="BO21" s="137"/>
-      <c r="BP21" s="137"/>
-      <c r="BQ21" s="137"/>
+      <c r="AS21" s="137"/>
+      <c r="AT21" s="138"/>
+      <c r="AU21" s="138"/>
+      <c r="AV21" s="138"/>
+      <c r="AW21" s="138"/>
+      <c r="AX21" s="138"/>
+      <c r="AY21" s="138"/>
+      <c r="AZ21" s="138"/>
+      <c r="BA21" s="138"/>
+      <c r="BB21" s="138"/>
+      <c r="BC21" s="138"/>
+      <c r="BD21" s="138"/>
+      <c r="BE21" s="138"/>
+      <c r="BF21" s="138"/>
+      <c r="BG21" s="138"/>
+      <c r="BH21" s="138"/>
+      <c r="BI21" s="138"/>
+      <c r="BJ21" s="138"/>
+      <c r="BK21" s="138"/>
+      <c r="BL21" s="138"/>
+      <c r="BM21" s="138"/>
+      <c r="BN21" s="138"/>
+      <c r="BO21" s="138"/>
+      <c r="BP21" s="138"/>
+      <c r="BQ21" s="138"/>
     </row>
-    <row r="22" s="132" customFormat="1" ht="15.25" spans="1:70">
+    <row r="22" s="133" customFormat="1" ht="15.75" spans="1:70">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -4149,22 +4209,22 @@
       <c r="K22" s="96" t="s">
         <v>54</v>
       </c>
-      <c r="L22" s="138" t="s">
+      <c r="L22" s="139" t="s">
         <v>55</v>
       </c>
-      <c r="M22" s="138" t="s">
+      <c r="M22" s="139" t="s">
         <v>56</v>
       </c>
-      <c r="N22" s="138" t="s">
+      <c r="N22" s="139" t="s">
         <v>57</v>
       </c>
-      <c r="O22" s="138" t="s">
+      <c r="O22" s="139" t="s">
         <v>58</v>
       </c>
-      <c r="P22" s="138" t="s">
+      <c r="P22" s="139" t="s">
         <v>59</v>
       </c>
-      <c r="Q22" s="138" t="s">
+      <c r="Q22" s="139" t="s">
         <v>60</v>
       </c>
       <c r="R22" s="96" t="s">
@@ -4248,10 +4308,10 @@
       <c r="AR22" s="100" t="s">
         <v>87</v>
       </c>
-      <c r="AS22" s="139" t="s">
+      <c r="AS22" s="140" t="s">
         <v>88</v>
       </c>
-      <c r="AT22" s="139" t="s">
+      <c r="AT22" s="140" t="s">
         <v>86</v>
       </c>
       <c r="AU22" s="102" t="s">
@@ -4323,9 +4383,9 @@
       <c r="BQ22" s="102" t="s">
         <v>63</v>
       </c>
-      <c r="BR22" s="140"/>
+      <c r="BR22" s="141"/>
     </row>
-    <row r="23" s="131" customFormat="1" ht="15.25" spans="1:70">
+    <row r="23" s="132" customFormat="1" ht="15.75" spans="1:70">
       <c r="A23" s="89">
         <v>1</v>
       </c>
@@ -4347,52 +4407,52 @@
       <c r="G23" s="104">
         <v>100</v>
       </c>
-      <c r="H23" s="141">
+      <c r="H23" s="121">
         <f>F23*G23</f>
         <v>200</v>
       </c>
-      <c r="I23" s="137">
+      <c r="I23" s="138">
         <v>1</v>
       </c>
-      <c r="J23" s="141">
+      <c r="J23" s="121">
         <v>2</v>
       </c>
-      <c r="K23" s="141">
+      <c r="K23" s="121">
         <v>4</v>
       </c>
-      <c r="L23" s="141">
+      <c r="L23" s="121">
         <f>H23</f>
         <v>200</v>
       </c>
-      <c r="M23" s="141">
+      <c r="M23" s="121">
         <f>ROUND(L23*I23%,2)</f>
         <v>2</v>
       </c>
-      <c r="N23" s="141">
+      <c r="N23" s="121">
         <f>H23-M23</f>
         <v>198</v>
       </c>
-      <c r="O23" s="141">
+      <c r="O23" s="121">
         <f>ROUND(N23*J23%,2)</f>
         <v>3.96</v>
       </c>
-      <c r="P23" s="141">
+      <c r="P23" s="121">
         <f>ROUND(N23-O23,2)</f>
         <v>194.04</v>
       </c>
-      <c r="Q23" s="141">
+      <c r="Q23" s="121">
         <f>ROUND(P23*K23%,2)</f>
         <v>7.76</v>
       </c>
-      <c r="R23" s="141">
+      <c r="R23" s="121">
         <f>M23+O23+Q23</f>
         <v>13.72</v>
       </c>
-      <c r="S23" s="141">
+      <c r="S23" s="121">
         <f>(H23-R23)</f>
         <v>186.28</v>
       </c>
-      <c r="T23" s="141" t="s">
+      <c r="T23" s="121" t="s">
         <v>111</v>
       </c>
       <c r="U23" s="106">
@@ -4425,89 +4485,89 @@
         <f>V23+W23+X23+Y23+AA23</f>
         <v>0</v>
       </c>
-      <c r="AC23" s="141">
+      <c r="AC23" s="121">
         <f>IF($V21=1,S23+AB23,S23)</f>
         <v>186.28</v>
       </c>
-      <c r="AD23" s="141">
+      <c r="AD23" s="121">
         <v>120</v>
       </c>
-      <c r="AE23" s="141">
+      <c r="AE23" s="121">
         <f>IF($P$21=1,(S23/$S$24)*$E$35,AD23/$AD$24*$E$35)</f>
         <v>0</v>
       </c>
-      <c r="AF23" s="141"/>
-      <c r="AG23" s="141">
+      <c r="AF23" s="121"/>
+      <c r="AG23" s="121">
         <f>IF($P$21=1,(S23/$S$24)*$E$37,AD23/$AD$24*$E$37)</f>
         <v>0</v>
       </c>
-      <c r="AH23" s="141">
+      <c r="AH23" s="121">
         <f>IF($P$21=1,(S23/$S$24)*$E$37,AD23/$AD$24*$E$37)</f>
         <v>0</v>
       </c>
-      <c r="AI23" s="141">
+      <c r="AI23" s="121">
         <f>S23*$M$21</f>
         <v>15833.8</v>
       </c>
-      <c r="AJ23" s="141">
+      <c r="AJ23" s="121">
         <f>IF($C$21=3,0,AG23+AH23)</f>
         <v>0</v>
       </c>
-      <c r="AK23" s="141">
+      <c r="AK23" s="121">
         <f>IF($C$21=3,AE23+AG23+AH23,0)</f>
         <v>0</v>
       </c>
-      <c r="AL23" s="141">
+      <c r="AL23" s="121">
         <v>1</v>
       </c>
-      <c r="AM23" s="141">
+      <c r="AM23" s="121">
         <f>F23/AL23</f>
         <v>2</v>
       </c>
-      <c r="AN23" s="141">
+      <c r="AN23" s="121">
         <f>AI23/AM23</f>
         <v>7916.9</v>
       </c>
-      <c r="AO23" s="141">
+      <c r="AO23" s="121">
         <f>AJ23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AP23" s="141">
+      <c r="AP23" s="121">
         <f>AK23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AQ23" s="141" t="s">
-        <v>12</v>
-      </c>
-      <c r="AR23" s="141">
+      <c r="AQ23" s="121" t="s">
+        <v>12</v>
+      </c>
+      <c r="AR23" s="121">
         <f>AN23+AO23+AP23</f>
         <v>7916.9</v>
       </c>
-      <c r="AS23" s="141" t="s">
+      <c r="AS23" s="121" t="s">
         <v>112</v>
       </c>
-      <c r="AT23" s="141" t="s">
-        <v>12</v>
-      </c>
-      <c r="AU23" t="s">
+      <c r="AT23" s="121" t="s">
+        <v>12</v>
+      </c>
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>114</v>
       </c>
-      <c r="AW23" s="141">
+      <c r="AW23" s="121">
         <f>AM23</f>
         <v>2</v>
       </c>
-      <c r="AX23" s="141">
+      <c r="AX23" s="121">
         <f>AR23</f>
         <v>7916.9</v>
       </c>
-      <c r="AY23" s="141">
+      <c r="AY23" s="121">
         <f>AU23+AW23</f>
         <v>2</v>
       </c>
-      <c r="AZ23" s="141">
+      <c r="AZ23" s="121">
         <f>ROUND(((AU23*AV23)+(AW23*AX23))/(AU23+AW23),5)</f>
         <v>7916.9</v>
       </c>
@@ -4527,19 +4587,19 @@
       <c r="BF23" s="142"/>
       <c r="BG23" s="142"/>
       <c r="BH23" s="142"/>
-      <c r="BI23" s="141"/>
-      <c r="BJ23" s="141"/>
-      <c r="BK23" s="141"/>
-      <c r="BL23" s="141" t="s">
+      <c r="BI23" s="121"/>
+      <c r="BJ23" s="121"/>
+      <c r="BK23" s="121"/>
+      <c r="BL23" s="121" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
-        <v>120</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>121</v>
-      </c>
-      <c r="BO23" s="141">
+      <c r="BM23" t="s" s="0">
+        <v>196</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="BO23" s="121">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>5978.94273</v>
       </c>
@@ -4551,10 +4611,10 @@
         <v>88363222</v>
       </c>
     </row>
-    <row r="24" s="131" customFormat="1" spans="1:70">
-      <c r="A24" s="136"/>
-      <c r="B24" s="137"/>
-      <c r="C24" s="137"/>
+    <row r="24" s="132" customFormat="1" spans="1:70">
+      <c r="A24" s="137"/>
+      <c r="B24" s="138"/>
+      <c r="C24" s="138"/>
       <c r="D24" s="144" t="s">
         <v>41</v>
       </c>
@@ -4565,15 +4625,15 @@
         <f>SUM(H23:H23)</f>
         <v>200</v>
       </c>
-      <c r="I24" s="136"/>
-      <c r="J24" s="136"/>
-      <c r="K24" s="136"/>
-      <c r="L24" s="136"/>
-      <c r="M24" s="136"/>
-      <c r="N24" s="136"/>
-      <c r="O24" s="136"/>
-      <c r="P24" s="136"/>
-      <c r="Q24" s="136"/>
+      <c r="I24" s="137"/>
+      <c r="J24" s="137"/>
+      <c r="K24" s="137"/>
+      <c r="L24" s="137"/>
+      <c r="M24" s="137"/>
+      <c r="N24" s="137"/>
+      <c r="O24" s="137"/>
+      <c r="P24" s="137"/>
+      <c r="Q24" s="137"/>
       <c r="R24" s="144">
         <f t="shared" ref="R24:Y24" si="1">SUM(R23:R23)</f>
         <v>13.72</v>
@@ -4649,31 +4709,31 @@
       <c r="AP24" s="99"/>
       <c r="AQ24" s="99"/>
       <c r="AR24" s="99"/>
-      <c r="AS24" s="136"/>
-      <c r="AT24" s="137"/>
-      <c r="AU24" s="137"/>
-      <c r="AV24" s="137"/>
-      <c r="AW24" s="137"/>
-      <c r="AX24" s="137"/>
-      <c r="AY24" s="137"/>
-      <c r="AZ24" s="137"/>
-      <c r="BA24" s="137"/>
-      <c r="BB24" s="137"/>
-      <c r="BC24" s="137"/>
-      <c r="BD24" s="137"/>
-      <c r="BE24" s="137"/>
-      <c r="BF24" s="137"/>
-      <c r="BG24" s="137"/>
-      <c r="BH24" s="137"/>
-      <c r="BI24" s="137"/>
-      <c r="BJ24" s="137"/>
-      <c r="BK24" s="137"/>
-      <c r="BL24" s="137"/>
-      <c r="BM24" s="137"/>
-      <c r="BN24" s="137"/>
-      <c r="BO24" s="137"/>
-      <c r="BP24" s="137"/>
-      <c r="BQ24" s="137"/>
+      <c r="AS24" s="137"/>
+      <c r="AT24" s="138"/>
+      <c r="AU24" s="138"/>
+      <c r="AV24" s="138"/>
+      <c r="AW24" s="138"/>
+      <c r="AX24" s="138"/>
+      <c r="AY24" s="138"/>
+      <c r="AZ24" s="138"/>
+      <c r="BA24" s="138"/>
+      <c r="BB24" s="138"/>
+      <c r="BC24" s="138"/>
+      <c r="BD24" s="138"/>
+      <c r="BE24" s="138"/>
+      <c r="BF24" s="138"/>
+      <c r="BG24" s="138"/>
+      <c r="BH24" s="138"/>
+      <c r="BI24" s="138"/>
+      <c r="BJ24" s="138"/>
+      <c r="BK24" s="138"/>
+      <c r="BL24" s="138"/>
+      <c r="BM24" s="138"/>
+      <c r="BN24" s="138"/>
+      <c r="BO24" s="138"/>
+      <c r="BP24" s="138"/>
+      <c r="BQ24" s="138"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4690,18 +4750,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
-  <sheetFormatPr defaultColWidth="9.85454545454546" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="9.85714285714286" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="9.85454545454546" style="1"/>
-    <col min="2" max="2" width="25.5727272727273" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="19" width="9.85454545454546" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="51" width="9.85454545454546" style="1"/>
-    <col min="52" max="52" width="11.5727272727273" style="1" customWidth="1"/>
-    <col min="53" max="66" width="9.85454545454546" style="1"/>
-    <col min="67" max="67" width="12" style="1"/>
-    <col min="68" max="16384" width="9.85454545454546" style="1"/>
+    <col min="1" max="1" style="1" width="9.85714285714286"/>
+    <col min="2" max="2" customWidth="true" style="1" width="25.5714285714286"/>
+    <col min="3" max="3" customWidth="true" style="1" width="26.0"/>
+    <col min="4" max="19" style="1" width="9.85714285714286"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="9.85714285714286"/>
+    <col min="52" max="52" customWidth="true" style="1" width="11.5714285714286"/>
+    <col min="53" max="66" style="1" width="9.85714285714286"/>
+    <col min="67" max="67" style="1" width="12.0"/>
+    <col min="68" max="16384" style="1" width="9.85714285714286"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -4777,7 +4837,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -4872,7 +4932,7 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="46" t="s">
         <v>2</v>
       </c>
@@ -5081,7 +5141,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
@@ -5240,7 +5300,7 @@
         <v>129.788</v>
       </c>
       <c r="AS4" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -5281,7 +5341,7 @@
       <c r="BJ4" s="6"/>
       <c r="BK4" s="6"/>
       <c r="BL4" s="29" t="s">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="BM4" s="1" t="s">
         <v>113</v>
@@ -5301,7 +5361,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -5432,18 +5492,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ17"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.71818181818182" style="1"/>
-    <col min="2" max="2" width="19.1454545454545" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.8545454545455" style="1" customWidth="1"/>
-    <col min="4" max="19" width="8.71818181818182" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="51" width="8.71818181818182" style="1"/>
-    <col min="52" max="52" width="12" style="1"/>
-    <col min="53" max="66" width="8.71818181818182" style="1"/>
-    <col min="67" max="67" width="12" style="1"/>
-    <col min="68" max="16384" width="8.71818181818182" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="19.1428571428571"/>
+    <col min="3" max="3" customWidth="true" style="1" width="25.8571428571429"/>
+    <col min="4" max="19" style="1" width="8.71428571428571"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="12.0"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="12.0"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -5519,7 +5579,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -5614,15 +5674,15 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -5823,7 +5883,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
@@ -5982,16 +6042,16 @@
         <v>129.79</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="AV4" s="23" t="s">
         <v>159</v>
-      </c>
-      <c r="AV4" s="23" t="s">
-        <v>160</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -6029,13 +6089,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="BM4" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="BN4" s="23" t="s">
         <v>161</v>
-      </c>
-      <c r="BM4" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="BN4" s="23" t="s">
-        <v>162</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -6049,7 +6109,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -6167,7 +6227,7 @@
       <c r="BP5" s="6"/>
       <c r="BQ5" s="6"/>
     </row>
-    <row r="6" ht="15.25" spans="1:69">
+    <row r="6" ht="15.75" spans="1:69">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -6238,7 +6298,7 @@
       <c r="BP6" s="6"/>
       <c r="BQ6" s="6"/>
     </row>
-    <row r="7" ht="15.25" spans="1:69">
+    <row r="7" ht="15.75" spans="1:69">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -6246,7 +6306,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H7" s="56"/>
       <c r="I7" s="57">
@@ -6257,7 +6317,7 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="58" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N7" s="59"/>
       <c r="O7" s="59"/>
@@ -6306,10 +6366,10 @@
       <c r="BF7" s="5"/>
       <c r="BG7" s="5"/>
       <c r="BH7" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="BI7" s="148" t="s">
         <v>165</v>
-      </c>
-      <c r="BI7" s="148" t="s">
-        <v>166</v>
       </c>
       <c r="BJ7" s="5"/>
       <c r="BK7" s="5"/>
@@ -6320,7 +6380,7 @@
       <c r="BP7" s="6"/>
       <c r="BQ7" s="6"/>
     </row>
-    <row r="8" ht="15.25" spans="1:69">
+    <row r="8" ht="15.75" spans="1:69">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -6328,7 +6388,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="55" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H8" s="56"/>
       <c r="I8" s="57">
@@ -6348,7 +6408,7 @@
         <v>2</v>
       </c>
       <c r="P8" s="61" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
@@ -6394,10 +6454,10 @@
       <c r="BF8" s="5"/>
       <c r="BG8" s="5"/>
       <c r="BH8" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="BI8" s="148" t="s">
         <v>169</v>
-      </c>
-      <c r="BI8" s="148" t="s">
-        <v>170</v>
       </c>
       <c r="BJ8" s="5"/>
       <c r="BK8" s="5"/>
@@ -6408,7 +6468,7 @@
       <c r="BP8" s="6"/>
       <c r="BQ8" s="6"/>
     </row>
-    <row r="9" ht="15.25" spans="1:69">
+    <row r="9" ht="15.75" spans="1:69">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -6416,7 +6476,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="55" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H9" s="56"/>
       <c r="I9" s="57">
@@ -6436,7 +6496,7 @@
         <v>2.5</v>
       </c>
       <c r="P9" s="20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
@@ -6492,7 +6552,7 @@
       <c r="BP9" s="6"/>
       <c r="BQ9" s="6"/>
     </row>
-    <row r="10" ht="15.25" spans="1:69">
+    <row r="10" ht="15.75" spans="1:69">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -6500,7 +6560,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H10" s="56"/>
       <c r="I10" s="57">
@@ -6514,13 +6574,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O10" s="20">
         <v>0.001</v>
       </c>
       <c r="P10" s="20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Q10" s="5"/>
       <c r="R10" s="5"/>
@@ -6576,7 +6636,7 @@
       <c r="BP10" s="6"/>
       <c r="BQ10" s="6"/>
     </row>
-    <row r="11" ht="15.25" spans="1:69">
+    <row r="11" ht="15.75" spans="1:69">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -6584,7 +6644,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H11" s="56"/>
       <c r="I11" s="62">
@@ -6718,10 +6778,10 @@
       <c r="BK12" s="5"/>
       <c r="BL12" s="5"/>
       <c r="BM12" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="BN12" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="BN12" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="BO12" s="5"/>
       <c r="BP12" s="6"/>
@@ -6791,7 +6851,7 @@
       <c r="BI13" s="5"/>
       <c r="BJ13" s="5"/>
       <c r="BK13" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="BL13" s="5">
         <v>12.5</v>
@@ -6872,7 +6932,7 @@
       <c r="BI14" s="5"/>
       <c r="BJ14" s="5"/>
       <c r="BK14" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BL14" s="5">
         <v>487.4072</v>
@@ -6950,7 +7010,7 @@
       <c r="BI15" s="5"/>
       <c r="BJ15" s="5"/>
       <c r="BK15" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="BL15" s="5">
         <v>37.5</v>
@@ -7025,7 +7085,7 @@
       <c r="BI16" s="5"/>
       <c r="BJ16" s="5"/>
       <c r="BK16" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BL16" s="5">
         <v>487.4072</v>
@@ -7140,18 +7200,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71818181818182" style="1"/>
-    <col min="2" max="2" width="21.1454545454545" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.2818181818182" style="1" customWidth="1"/>
-    <col min="4" max="19" width="8.71818181818182" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="51" width="8.71818181818182" style="1"/>
-    <col min="52" max="52" width="10.5727272727273" style="1"/>
-    <col min="53" max="66" width="8.71818181818182" style="1"/>
-    <col min="67" max="67" width="13.2818181818182" style="1"/>
-    <col min="68" max="16384" width="8.71818181818182" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="21.1428571428571"/>
+    <col min="3" max="3" customWidth="true" style="1" width="21.2857142857143"/>
+    <col min="4" max="19" style="1" width="8.71428571428571"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="10.5714285714286"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="13.2857142857143"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7227,7 +7287,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -7322,15 +7382,15 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -7531,15 +7591,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -7690,7 +7750,7 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -7699,7 +7759,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -7737,13 +7797,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="BM4" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="BN4" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>183</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -7757,7 +7817,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -7892,18 +7952,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71818181818182" style="1"/>
-    <col min="2" max="2" width="23.4272727272727" style="1" customWidth="1"/>
-    <col min="3" max="3" width="29.4272727272727" style="1" customWidth="1"/>
-    <col min="4" max="19" width="8.71818181818182" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="51" width="8.71818181818182" style="1"/>
-    <col min="52" max="52" width="10.7181818181818" style="1"/>
-    <col min="53" max="66" width="8.71818181818182" style="1"/>
-    <col min="67" max="67" width="10.5727272727273" style="1"/>
-    <col min="68" max="16384" width="8.71818181818182" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="23.4285714285714"/>
+    <col min="3" max="3" customWidth="true" style="1" width="29.4285714285714"/>
+    <col min="4" max="19" style="1" width="8.71428571428571"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="10.7142857142857"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="10.5714285714286"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7979,7 +8039,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -8074,15 +8134,15 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -8283,15 +8343,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -8442,16 +8502,16 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="AV4" s="23" t="s">
         <v>184</v>
-      </c>
-      <c r="AV4" s="23" t="s">
-        <v>185</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -8489,13 +8549,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="BM4" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="BN4" s="23" t="s">
         <v>161</v>
-      </c>
-      <c r="BM4" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="BN4" s="23" t="s">
-        <v>162</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -8509,7 +8569,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -8643,16 +8703,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71818181818182" style="1"/>
-    <col min="2" max="2" width="27.2818181818182" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.4272727272727" style="1" customWidth="1"/>
-    <col min="4" max="19" width="8.71818181818182" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="66" width="8.71818181818182" style="1"/>
-    <col min="67" max="67" width="12" style="1"/>
-    <col min="68" max="16384" width="8.71818181818182" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="27.2857142857143"/>
+    <col min="3" max="3" customWidth="true" style="1" width="25.4285714285714"/>
+    <col min="4" max="19" style="1" width="8.71428571428571"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="12.0"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -8728,7 +8788,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -8823,15 +8883,15 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -9032,15 +9092,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -9191,7 +9251,7 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -9200,7 +9260,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -9238,13 +9298,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="BM4" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="BN4" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>187</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -9258,7 +9318,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -9392,26 +9452,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ18"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85714285714286" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.85454545454546" style="23"/>
-    <col min="2" max="2" width="28" style="23" customWidth="1"/>
-    <col min="3" max="3" width="23" style="23" customWidth="1"/>
-    <col min="4" max="11" width="8.85454545454546" style="23"/>
-    <col min="12" max="12" width="15.7181818181818" style="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14545454545454" style="23" customWidth="1"/>
-    <col min="14" max="14" width="13.8545454545455" style="23" customWidth="1"/>
-    <col min="15" max="15" width="11.2818181818182" style="23" customWidth="1"/>
-    <col min="16" max="16" width="17.8545454545455" style="23" customWidth="1"/>
-    <col min="17" max="19" width="8.85454545454546" style="23"/>
-    <col min="20" max="20" width="10.1454545454545" style="23" customWidth="1"/>
-    <col min="21" max="51" width="8.85454545454546" style="23"/>
-    <col min="52" max="52" width="10.7181818181818" style="23"/>
-    <col min="53" max="63" width="8.85454545454546" style="23"/>
-    <col min="64" max="64" width="11" style="23" customWidth="1"/>
-    <col min="65" max="66" width="8.85454545454546" style="23"/>
-    <col min="67" max="67" width="10.7181818181818" style="23"/>
-    <col min="68" max="16384" width="8.85454545454546" style="23"/>
+    <col min="1" max="1" style="23" width="8.85714285714286"/>
+    <col min="2" max="2" customWidth="true" style="23" width="28.0"/>
+    <col min="3" max="3" customWidth="true" style="23" width="23.0"/>
+    <col min="4" max="11" style="23" width="8.85714285714286"/>
+    <col min="12" max="12" customWidth="true" style="23" width="15.7142857142857"/>
+    <col min="13" max="13" customWidth="true" style="23" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" style="23" width="13.8571428571429"/>
+    <col min="15" max="15" customWidth="true" style="23" width="11.2857142857143"/>
+    <col min="16" max="16" customWidth="true" style="23" width="17.8571428571429"/>
+    <col min="17" max="19" style="23" width="8.85714285714286"/>
+    <col min="20" max="20" customWidth="true" style="23" width="10.1428571428571"/>
+    <col min="21" max="51" style="23" width="8.85714285714286"/>
+    <col min="52" max="52" style="23" width="10.7142857142857"/>
+    <col min="53" max="63" style="23" width="8.85714285714286"/>
+    <col min="64" max="64" customWidth="true" style="23" width="11.0"/>
+    <col min="65" max="66" style="23" width="8.85714285714286"/>
+    <col min="67" max="67" style="23" width="10.7142857142857"/>
+    <col min="68" max="16384" style="23" width="8.85714285714286"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -9487,7 +9547,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -9582,15 +9642,15 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -9791,15 +9851,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -9950,16 +10010,16 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AV4" s="23" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -9997,13 +10057,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="BM4" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="BN4" s="23" t="s">
         <v>161</v>
-      </c>
-      <c r="BM4" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="BN4" s="23" t="s">
-        <v>162</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -10017,7 +10077,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -10135,7 +10195,7 @@
       <c r="BP5" s="6"/>
       <c r="BQ5" s="6"/>
     </row>
-    <row r="6" ht="15.25" spans="1:69">
+    <row r="6" ht="15.75" spans="1:69">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -10206,7 +10266,7 @@
       <c r="BP6" s="6"/>
       <c r="BQ6" s="6"/>
     </row>
-    <row r="7" ht="15.25" spans="1:69">
+    <row r="7" ht="15.75" spans="1:69">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -10214,7 +10274,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H7" s="56"/>
       <c r="I7" s="57">
@@ -10225,7 +10285,7 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="58" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N7" s="59"/>
       <c r="O7" s="59"/>
@@ -10274,10 +10334,10 @@
       <c r="BF7" s="5"/>
       <c r="BG7" s="5"/>
       <c r="BH7" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="BI7" s="148" t="s">
         <v>165</v>
-      </c>
-      <c r="BI7" s="148" t="s">
-        <v>166</v>
       </c>
       <c r="BJ7" s="5"/>
       <c r="BK7" s="5"/>
@@ -10288,7 +10348,7 @@
       <c r="BP7" s="6"/>
       <c r="BQ7" s="6"/>
     </row>
-    <row r="8" ht="15.25" spans="1:69">
+    <row r="8" ht="15.75" spans="1:69">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -10296,7 +10356,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="55" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H8" s="56"/>
       <c r="I8" s="57">
@@ -10316,7 +10376,7 @@
         <v>2</v>
       </c>
       <c r="P8" s="61" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
@@ -10362,10 +10422,10 @@
       <c r="BF8" s="5"/>
       <c r="BG8" s="5"/>
       <c r="BH8" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="BI8" s="148" t="s">
         <v>169</v>
-      </c>
-      <c r="BI8" s="148" t="s">
-        <v>170</v>
       </c>
       <c r="BJ8" s="5"/>
       <c r="BK8" s="5"/>
@@ -10376,7 +10436,7 @@
       <c r="BP8" s="6"/>
       <c r="BQ8" s="6"/>
     </row>
-    <row r="9" ht="15.25" spans="1:69">
+    <row r="9" ht="15.75" spans="1:69">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -10384,7 +10444,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="55" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H9" s="56"/>
       <c r="I9" s="57">
@@ -10404,7 +10464,7 @@
         <v>2.5</v>
       </c>
       <c r="P9" s="20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
@@ -10460,7 +10520,7 @@
       <c r="BP9" s="6"/>
       <c r="BQ9" s="6"/>
     </row>
-    <row r="10" ht="15.25" spans="1:69">
+    <row r="10" ht="15.75" spans="1:69">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -10468,7 +10528,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H10" s="56"/>
       <c r="I10" s="57">
@@ -10482,13 +10542,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O10" s="20">
         <v>0.001</v>
       </c>
       <c r="P10" s="20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Q10" s="5"/>
       <c r="R10" s="5"/>
@@ -10544,7 +10604,7 @@
       <c r="BP10" s="6"/>
       <c r="BQ10" s="6"/>
     </row>
-    <row r="11" ht="15.25" spans="1:69">
+    <row r="11" ht="15.75" spans="1:69">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -10552,7 +10612,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H11" s="56"/>
       <c r="I11" s="62">
@@ -10686,10 +10746,10 @@
       <c r="BK12" s="5"/>
       <c r="BL12" s="5"/>
       <c r="BM12" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="BN12" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="BN12" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="BO12" s="5"/>
       <c r="BP12" s="6"/>
@@ -10759,7 +10819,7 @@
       <c r="BI13" s="5"/>
       <c r="BJ13" s="5"/>
       <c r="BK13" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="BL13" s="5">
         <v>12.5</v>
@@ -10840,7 +10900,7 @@
       <c r="BI14" s="5"/>
       <c r="BJ14" s="5"/>
       <c r="BK14" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BL14" s="5">
         <v>487.4072</v>
@@ -10918,7 +10978,7 @@
       <c r="BI15" s="5"/>
       <c r="BJ15" s="5"/>
       <c r="BK15" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="BL15" s="5">
         <v>37.5</v>
@@ -10993,7 +11053,7 @@
       <c r="BI16" s="5"/>
       <c r="BJ16" s="5"/>
       <c r="BK16" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BL16" s="5">
         <v>487.4072</v>
@@ -11179,14 +11239,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
-  <sheetFormatPr defaultColWidth="9.85454545454546" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="9.85714285714286" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="9.85454545454546" style="1"/>
-    <col min="2" max="2" width="25.5727272727273" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="19" width="9.85454545454546" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.85454545454546" style="1"/>
+    <col min="1" max="1" style="1" width="9.85714285714286"/>
+    <col min="2" max="2" customWidth="true" style="1" width="25.5714285714286"/>
+    <col min="3" max="3" customWidth="true" style="1" width="26.0"/>
+    <col min="4" max="19" style="1" width="9.85714285714286"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="16384" style="1" width="9.85714285714286"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -11262,7 +11322,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -11357,7 +11417,7 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="46" t="s">
         <v>2</v>
       </c>
@@ -11566,21 +11626,21 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -11725,7 +11785,7 @@
         <v>648.94</v>
       </c>
       <c r="AS4" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -11766,7 +11826,7 @@
       <c r="BJ4" s="6"/>
       <c r="BK4" s="6"/>
       <c r="BL4" s="29" t="s">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="BM4" s="1" t="s">
         <v>113</v>
@@ -11786,7 +11846,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -11917,16 +11977,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71818181818182" style="1"/>
-    <col min="2" max="3" width="26.5454545454545" style="1" customWidth="1"/>
-    <col min="4" max="19" width="8.71818181818182" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="66" width="8.71818181818182" style="1"/>
-    <col min="67" max="67" width="13.2818181818182" style="1"/>
-    <col min="68" max="68" width="12.8545454545455" style="1"/>
-    <col min="69" max="16384" width="8.71818181818182" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="3" customWidth="true" style="1" width="26.5428571428571"/>
+    <col min="4" max="19" style="1" width="8.71428571428571"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="13.2857142857143"/>
+    <col min="68" max="68" style="1" width="12.8571428571429"/>
+    <col min="69" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -12002,7 +12062,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -12097,15 +12157,15 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -12306,21 +12366,21 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -12465,7 +12525,7 @@
         <v>648.94</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -12474,7 +12534,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -12512,13 +12572,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="BM4" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="BN4" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>191</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -12532,7 +12592,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -12666,18 +12726,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ5"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71818181818182" style="1"/>
-    <col min="2" max="2" width="27.2818181818182" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.4272727272727" style="1" customWidth="1"/>
-    <col min="4" max="19" width="8.71818181818182" style="1"/>
-    <col min="20" max="20" width="10.1454545454545" style="1" customWidth="1"/>
-    <col min="21" max="51" width="8.71818181818182" style="1"/>
-    <col min="52" max="52" width="9" style="1"/>
-    <col min="53" max="66" width="8.71818181818182" style="1"/>
-    <col min="67" max="67" width="13.2818181818182" style="1"/>
-    <col min="68" max="16384" width="8.71818181818182" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="27.2857142857143"/>
+    <col min="3" max="3" customWidth="true" style="1" width="25.4285714285714"/>
+    <col min="4" max="19" style="1" width="8.71428571428571"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="9.0"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="13.2857142857143"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -12753,7 +12813,7 @@
       <c r="BP1" s="6"/>
       <c r="BQ1" s="6"/>
     </row>
-    <row r="2" ht="15.25" spans="1:69">
+    <row r="2" ht="15.75" spans="1:69">
       <c r="A2" s="7" t="s">
         <v>43</v>
       </c>
@@ -12848,15 +12908,15 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="45" spans="1:69">
+    <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -13057,21 +13117,21 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.25" spans="1:69">
+    <row r="4" ht="15.75" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -13216,7 +13276,7 @@
         <v>648.94</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -13225,7 +13285,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -13263,13 +13323,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="BM4" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="BN4" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>193</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -13283,7 +13343,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.25" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -13417,76 +13477,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="9" width="5.85454545454545" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85454545454545" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.4272727272727" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="11.8545454545455" customWidth="1"/>
-    <col min="20" max="20" width="10.7181818181818" customWidth="1"/>
-    <col min="21" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="18" customWidth="1"/>
-    <col min="48" max="48" width="24.4272727272727" customWidth="1"/>
-    <col min="49" max="49" width="14.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="9.42727272727273" customWidth="1"/>
-    <col min="65" max="65" width="49.1454545454545" customWidth="1"/>
-    <col min="66" max="66" width="43.8545454545455" customWidth="1"/>
-    <col min="67" max="67" width="22.7181818181818" customWidth="1"/>
-    <col min="68" max="68" width="40.8545454545455" customWidth="1"/>
-    <col min="69" max="69" width="7.57272727272727" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="22.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="9" customWidth="true" width="5.85714285714286"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85714285714286"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.4285714285714"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="11.8571428571429"/>
+    <col min="20" max="20" customWidth="true" width="10.7142857142857"/>
+    <col min="21" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="18.0"/>
+    <col min="48" max="48" customWidth="true" width="24.4285714285714"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="9.42857142857143"/>
+    <col min="65" max="65" customWidth="true" width="49.1428571428571"/>
+    <col min="66" max="66" customWidth="true" width="43.8571428571429"/>
+    <col min="67" max="67" customWidth="true" width="22.7142857142857"/>
+    <col min="68" max="68" customWidth="true" width="40.8571428571429"/>
+    <col min="69" max="69" customWidth="true" width="7.57142857142857"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -13559,7 +13619,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -13632,7 +13692,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -14951,7 +15011,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -15039,7 +15099,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -15283,7 +15343,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -15317,22 +15377,22 @@
       <c r="K22" s="96" t="s">
         <v>53</v>
       </c>
-      <c r="L22" s="121" t="s">
+      <c r="L22" s="122" t="s">
         <v>55</v>
       </c>
-      <c r="M22" s="121" t="s">
+      <c r="M22" s="122" t="s">
         <v>56</v>
       </c>
-      <c r="N22" s="121" t="s">
+      <c r="N22" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="O22" s="121" t="s">
+      <c r="O22" s="122" t="s">
         <v>60</v>
       </c>
-      <c r="P22" s="121" t="s">
+      <c r="P22" s="122" t="s">
         <v>122</v>
       </c>
-      <c r="Q22" s="121" t="s">
+      <c r="Q22" s="122" t="s">
         <v>58</v>
       </c>
       <c r="R22" s="96" t="s">
@@ -15492,7 +15552,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.25" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
@@ -15551,7 +15611,7 @@
         <f>ROUND(P23*K23%,2)</f>
         <v>7.76</v>
       </c>
-      <c r="R23" s="122">
+      <c r="R23" s="123">
         <f>ROUND(M23+O23+Q23,3)</f>
         <v>13.72</v>
       </c>
@@ -15592,81 +15652,81 @@
         <f>V23+W23+X23+Y23+AA23</f>
         <v>0</v>
       </c>
-      <c r="AC23" s="123">
+      <c r="AC23" s="124">
         <f>IF($V21=1,S23+AB23,S23)</f>
         <v>186.28</v>
       </c>
-      <c r="AD23" s="122">
+      <c r="AD23" s="123">
         <v>120</v>
       </c>
-      <c r="AE23" s="122">
+      <c r="AE23" s="123">
         <f>IF($P$21=1,(S23/$S$23)*$E$30,AD23/$AD$4*$E$30)</f>
         <v>0</v>
       </c>
-      <c r="AF23" s="122"/>
-      <c r="AG23" s="122">
+      <c r="AF23" s="123"/>
+      <c r="AG23" s="123">
         <f>IF($P$21=1,(S23/$S$23)*$E$20,AD23/$AD$23*$E$20)</f>
         <v>0</v>
       </c>
-      <c r="AH23" s="122">
+      <c r="AH23" s="123">
         <f>IF($P$21=1,(S23/$S$23)*$E$21,AD23/$AD$23*$E$21)</f>
         <v>0</v>
       </c>
-      <c r="AI23" s="122">
+      <c r="AI23" s="123">
         <f>S23*$M21</f>
         <v>15833.8</v>
       </c>
-      <c r="AJ23" s="122">
+      <c r="AJ23" s="123">
         <f>IF($C$2=3,0,AG23+AH23)</f>
         <v>0</v>
       </c>
-      <c r="AK23" s="122">
+      <c r="AK23" s="123">
         <f>IF($C$2=3,AE23+AG23+AH23,0)</f>
         <v>0</v>
       </c>
-      <c r="AL23" s="124">
+      <c r="AL23" s="125">
         <v>3</v>
       </c>
-      <c r="AM23" s="122">
+      <c r="AM23" s="123">
         <f>F23/AL23</f>
         <v>0.666666666666667</v>
       </c>
-      <c r="AN23" s="122">
+      <c r="AN23" s="123">
         <f>ROUND(AI23/AM23,5)</f>
         <v>23750.7</v>
       </c>
-      <c r="AO23" s="122">
+      <c r="AO23" s="123">
         <f>AJ23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AP23" s="122">
+      <c r="AP23" s="123">
         <f>AK23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AQ23" s="122" t="s">
-        <v>12</v>
-      </c>
-      <c r="AR23" s="122">
+      <c r="AQ23" s="123" t="s">
+        <v>12</v>
+      </c>
+      <c r="AR23" s="123">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>23750.7</v>
       </c>
-      <c r="AS23" s="125" t="s">
+      <c r="AS23" s="126" t="s">
+        <v>112</v>
+      </c>
+      <c r="AT23" s="116" t="s">
+        <v>12</v>
+      </c>
+      <c r="AU23" s="117" t="s">
         <v>127</v>
       </c>
-      <c r="AT23" s="116" t="s">
-        <v>12</v>
-      </c>
-      <c r="AU23" s="117" t="s">
+      <c r="AV23" s="117" t="s">
         <v>128</v>
-      </c>
-      <c r="AV23" s="117" t="s">
-        <v>129</v>
       </c>
       <c r="AW23" s="116">
         <f>AM23</f>
         <v>0.666666666666667</v>
       </c>
-      <c r="AX23" s="122">
+      <c r="AX23" s="123">
         <f>AR23</f>
         <v>23750.7</v>
       </c>
@@ -15674,47 +15734,47 @@
         <f>AU23+AW23</f>
         <v>117.000666666667</v>
       </c>
-      <c r="AZ23" s="126">
+      <c r="AZ23" s="127">
         <f>ROUND(((AU23*AV23)+(AW23*AX23))/(AU23+AW23),5)</f>
         <v>6394.32854</v>
       </c>
-      <c r="BA23" s="127"/>
-      <c r="BB23" s="127" t="s">
+      <c r="BA23" s="128"/>
+      <c r="BB23" s="128" t="s">
         <v>115</v>
       </c>
-      <c r="BC23" s="127" t="s">
+      <c r="BC23" s="128" t="s">
         <v>116</v>
       </c>
-      <c r="BD23" s="128" t="s">
+      <c r="BD23" s="129" t="s">
         <v>117</v>
       </c>
-      <c r="BE23" s="128" t="s">
+      <c r="BE23" s="129" t="s">
         <v>118</v>
       </c>
-      <c r="BF23" s="127"/>
-      <c r="BG23" s="127"/>
-      <c r="BH23" s="127"/>
+      <c r="BF23" s="128"/>
+      <c r="BG23" s="128"/>
+      <c r="BH23" s="128"/>
       <c r="BI23" s="116"/>
       <c r="BJ23" s="116"/>
       <c r="BK23" s="116"/>
-      <c r="BL23" s="129" t="s">
+      <c r="BL23" s="130" t="s">
         <v>119</v>
       </c>
       <c r="BM23" s="117" t="s">
+        <v>129</v>
+      </c>
+      <c r="BN23" s="117" t="s">
         <v>130</v>
-      </c>
-      <c r="BN23" s="117" t="s">
-        <v>131</v>
       </c>
       <c r="BO23" s="116">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>280.32668</v>
       </c>
-      <c r="BP23" s="127">
+      <c r="BP23" s="128">
         <f>ROUND(BN23+AW23,3)</f>
         <v>120.667</v>
       </c>
-      <c r="BQ23" s="130">
+      <c r="BQ23" s="131">
         <v>123562</v>
       </c>
     </row>
@@ -15849,7 +15909,7 @@
     <mergeCell ref="A21:B21"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="AS23" r:id="rId1" display="INS WH-1" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
+    <hyperlink ref="AS23" r:id="rId1" display="INS" tooltip="https://webappqc.roadmaperp.com:8765/ords/r/rmqc27/scm-us9011/warehouse1?p367019101_rowid=AAATkUAAHAADnkPAAX&amp;p367019101_store_id=INS WH-1&amp;session=1523407412914"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -15860,76 +15920,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="25.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4272727272727" customWidth="1"/>
-    <col min="48" max="48" width="18.8545454545455" customWidth="1"/>
-    <col min="49" max="49" width="13.4272727272727" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="5.28181818181818" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="25.2857142857143"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -16002,7 +16062,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -16075,7 +16135,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -17394,7 +17454,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -17482,7 +17542,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -17726,7 +17786,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -17866,10 +17926,10 @@
         <v>86</v>
       </c>
       <c r="AU22" s="101" t="s">
+        <v>131</v>
+      </c>
+      <c r="AV22" s="101" t="s">
         <v>132</v>
-      </c>
-      <c r="AV22" s="101" t="s">
-        <v>133</v>
       </c>
       <c r="AW22" s="101" t="s">
         <v>91</v>
@@ -17935,15 +17995,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -18099,11 +18159,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
-        <v>114</v>
+      <c r="AV23" t="s" s="0">
+        <v>197</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -18140,14 +18200,14 @@
       <c r="BI23" s="105"/>
       <c r="BJ23" s="105"/>
       <c r="BK23" s="105"/>
-      <c r="BL23" s="105" t="s">
+      <c r="BL23" s="121" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
-        <v>135</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>136</v>
+      <c r="BM23" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>199</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -18300,76 +18360,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="25.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4272727272727" customWidth="1"/>
-    <col min="48" max="48" width="18.8545454545455" customWidth="1"/>
-    <col min="49" max="49" width="13.4272727272727" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="5.28181818181818" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="25.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -18442,7 +18502,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -18515,7 +18575,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -19834,7 +19894,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -19922,7 +19982,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="118" t="s">
         <v>41</v>
@@ -20166,7 +20226,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -20306,10 +20366,10 @@
         <v>86</v>
       </c>
       <c r="AU22" s="101" t="s">
+        <v>131</v>
+      </c>
+      <c r="AV22" s="101" t="s">
         <v>132</v>
-      </c>
-      <c r="AV22" s="101" t="s">
-        <v>133</v>
       </c>
       <c r="AW22" s="101" t="s">
         <v>91</v>
@@ -20380,10 +20440,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -20726,76 +20786,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="24.7181818181818" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4272727272727" customWidth="1"/>
-    <col min="48" max="48" width="18.8545454545455" customWidth="1"/>
-    <col min="49" max="49" width="13.4272727272727" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="5.28181818181818" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="24.7142857142857"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -20868,7 +20928,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -20941,7 +21001,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -22260,7 +22320,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -22348,7 +22408,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -22592,7 +22652,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -22732,10 +22792,10 @@
         <v>86</v>
       </c>
       <c r="AU22" s="101" t="s">
+        <v>131</v>
+      </c>
+      <c r="AV22" s="101" t="s">
         <v>132</v>
-      </c>
-      <c r="AV22" s="101" t="s">
-        <v>133</v>
       </c>
       <c r="AW22" s="101" t="s">
         <v>91</v>
@@ -22801,15 +22861,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.25" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="89" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C23" s="89" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -22820,15 +22880,15 @@
       <c r="F23" s="104">
         <v>2</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>250</v>
       </c>
       <c r="H23" s="105">
         <f>F23*G23</f>
         <v>500</v>
       </c>
-      <c r="I23" t="s">
-        <v>139</v>
+      <c r="I23" t="s" s="0">
+        <v>138</v>
       </c>
       <c r="J23" s="105">
         <v>2</v>
@@ -22965,11 +23025,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
-        <v>140</v>
+      <c r="AV23" t="s" s="0">
+        <v>197</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -23007,13 +23067,13 @@
       <c r="BJ23" s="105"/>
       <c r="BK23" s="105"/>
       <c r="BL23" s="105" t="s">
-        <v>141</v>
-      </c>
-      <c r="BM23" t="s">
-        <v>142</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>143</v>
+        <v>119</v>
+      </c>
+      <c r="BM23" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>201</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -23166,76 +23226,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="25.1454545454545" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4272727272727" customWidth="1"/>
-    <col min="48" max="48" width="18.8545454545455" customWidth="1"/>
-    <col min="49" max="49" width="13.4272727272727" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="5.28181818181818" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="25.1428571428571"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -23308,7 +23368,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -23381,7 +23441,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -24700,7 +24760,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -24788,7 +24848,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -25032,7 +25092,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -25172,10 +25232,10 @@
         <v>86</v>
       </c>
       <c r="AU22" s="101" t="s">
+        <v>131</v>
+      </c>
+      <c r="AV22" s="101" t="s">
         <v>132</v>
-      </c>
-      <c r="AV22" s="101" t="s">
-        <v>133</v>
       </c>
       <c r="AW22" s="101" t="s">
         <v>91</v>
@@ -25241,15 +25301,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.25" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="89" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C23" s="89" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -25260,15 +25320,15 @@
       <c r="F23" s="104">
         <v>2</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>250</v>
       </c>
       <c r="H23" s="105">
         <f>F23*G23</f>
         <v>500</v>
       </c>
-      <c r="I23" t="s">
-        <v>139</v>
+      <c r="I23" t="s" s="0">
+        <v>138</v>
       </c>
       <c r="J23" s="105">
         <v>2</v>
@@ -25598,76 +25658,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="24.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4272727272727" customWidth="1"/>
-    <col min="48" max="48" width="18.8545454545455" customWidth="1"/>
-    <col min="49" max="49" width="14.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="5.28181818181818" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="24.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -25740,7 +25800,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -25813,7 +25873,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -27132,7 +27192,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -27220,7 +27280,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -27464,7 +27524,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -27604,10 +27664,10 @@
         <v>86</v>
       </c>
       <c r="AU22" s="101" t="s">
+        <v>131</v>
+      </c>
+      <c r="AV22" s="101" t="s">
         <v>132</v>
-      </c>
-      <c r="AV22" s="101" t="s">
-        <v>133</v>
       </c>
       <c r="AW22" s="95" t="s">
         <v>91</v>
@@ -27673,15 +27733,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.25" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -27837,11 +27897,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
-        <v>146</v>
+      <c r="AV23" t="s" s="0">
+        <v>114</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -27881,11 +27941,11 @@
       <c r="BL23" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
-        <v>147</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>148</v>
+      <c r="BM23" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>209</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -28038,76 +28098,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4272727272727" customWidth="1"/>
-    <col min="48" max="48" width="18.8545454545455" customWidth="1"/>
-    <col min="49" max="49" width="14.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="5.28181818181818" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="28.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -28180,7 +28240,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -28253,7 +28313,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -29572,7 +29632,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -29660,7 +29720,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -29904,7 +29964,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -30044,10 +30104,10 @@
         <v>86</v>
       </c>
       <c r="AU22" s="101" t="s">
+        <v>131</v>
+      </c>
+      <c r="AV22" s="101" t="s">
         <v>132</v>
-      </c>
-      <c r="AV22" s="101" t="s">
-        <v>133</v>
       </c>
       <c r="AW22" s="101" t="s">
         <v>91</v>
@@ -30118,10 +30178,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -30277,11 +30337,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
-        <v>150</v>
+      <c r="AV23" t="s" s="0">
+        <v>211</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -30321,11 +30381,11 @@
       <c r="BL23" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
-        <v>151</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>152</v>
+      <c r="BM23" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>213</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -30478,76 +30538,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BQ24"/>
-  <sheetFormatPr defaultColWidth="8.71818181818182" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57272727272727" customWidth="1"/>
-    <col min="2" max="3" width="27.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="79.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="11.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="24.1454545454545" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7181818181818" customWidth="1"/>
-    <col min="9" max="10" width="5.85454545454545" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2818181818182" customWidth="1"/>
-    <col min="13" max="13" width="9.42727272727273" customWidth="1"/>
-    <col min="14" max="14" width="14.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="15.5727272727273" customWidth="1"/>
-    <col min="16" max="16" width="14.4272727272727" customWidth="1"/>
-    <col min="17" max="17" width="39.4272727272727" customWidth="1"/>
-    <col min="18" max="18" width="11.7181818181818" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42727272727273" customWidth="1"/>
-    <col min="21" max="21" width="9.85454545454546" customWidth="1"/>
-    <col min="22" max="22" width="6.57272727272727" customWidth="1"/>
-    <col min="23" max="23" width="37.1454545454545" customWidth="1"/>
-    <col min="24" max="24" width="6.14545454545455" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71818181818182" customWidth="1"/>
-    <col min="27" max="27" width="6.28181818181818" customWidth="1"/>
-    <col min="28" max="28" width="9.28181818181818" customWidth="1"/>
-    <col min="29" max="29" width="9.71818181818182" customWidth="1"/>
-    <col min="30" max="30" width="12.8545454545455" customWidth="1"/>
-    <col min="31" max="31" width="16.1454545454545" customWidth="1"/>
-    <col min="32" max="32" width="15.4272727272727" customWidth="1"/>
-    <col min="33" max="33" width="24.5727272727273" customWidth="1"/>
-    <col min="34" max="34" width="8.57272727272727" customWidth="1"/>
-    <col min="35" max="35" width="14.7181818181818" customWidth="1"/>
-    <col min="36" max="36" width="18.5727272727273" customWidth="1"/>
-    <col min="37" max="37" width="14.1454545454545" customWidth="1"/>
-    <col min="38" max="38" width="14.7181818181818" customWidth="1"/>
-    <col min="39" max="39" width="17.4272727272727" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5727272727273" customWidth="1"/>
-    <col min="42" max="42" width="25.2818181818182" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7181818181818" customWidth="1"/>
-    <col min="45" max="45" width="9.28181818181818" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4272727272727" customWidth="1"/>
-    <col min="48" max="48" width="18.8545454545455" customWidth="1"/>
-    <col min="49" max="49" width="14.5727272727273" customWidth="1"/>
-    <col min="50" max="50" width="19.4272727272727" customWidth="1"/>
-    <col min="51" max="51" width="16.2818181818182" customWidth="1"/>
-    <col min="52" max="52" width="22.7181818181818" customWidth="1"/>
-    <col min="53" max="53" width="21.7181818181818" customWidth="1"/>
-    <col min="54" max="54" width="23.2818181818182" customWidth="1"/>
-    <col min="55" max="55" width="18.2818181818182" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1454545454545" customWidth="1"/>
-    <col min="59" max="59" width="15.5727272727273" customWidth="1"/>
-    <col min="60" max="61" width="14.7181818181818" customWidth="1"/>
-    <col min="62" max="62" width="25.4272727272727" customWidth="1"/>
-    <col min="63" max="63" width="35.4272727272727" customWidth="1"/>
-    <col min="64" max="64" width="8.57272727272727" customWidth="1"/>
-    <col min="65" max="65" width="42.5727272727273" customWidth="1"/>
-    <col min="66" max="66" width="38.1454545454545" customWidth="1"/>
-    <col min="67" max="67" width="19.4272727272727" customWidth="1"/>
-    <col min="68" max="68" width="35.4272727272727" customWidth="1"/>
-    <col min="69" max="69" width="5.28181818181818" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="27.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" spans="1:69">
+    <row r="1" ht="18.75" spans="1:69">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -30620,7 +30680,7 @@
       <c r="BP1" s="65"/>
       <c r="BQ1" s="65"/>
     </row>
-    <row r="2" ht="19.25" spans="1:69">
+    <row r="2" ht="19.5" spans="1:69">
       <c r="A2" s="63" t="s">
         <v>1</v>
       </c>
@@ -30693,7 +30753,7 @@
       <c r="BP2" s="65"/>
       <c r="BQ2" s="65"/>
     </row>
-    <row r="3" ht="15.25" spans="1:69">
+    <row r="3" ht="15.75" spans="1:69">
       <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
@@ -32012,7 +32072,7 @@
       <c r="BP17" s="65"/>
       <c r="BQ17" s="65"/>
     </row>
-    <row r="18" ht="15.25" spans="1:69">
+    <row r="18" ht="15.75" spans="1:69">
       <c r="A18" s="79">
         <v>15</v>
       </c>
@@ -32100,7 +32160,7 @@
       <c r="BP18" s="65"/>
       <c r="BQ18" s="65"/>
     </row>
-    <row r="19" ht="15.25" spans="1:69">
+    <row r="19" ht="15.75" spans="1:69">
       <c r="A19" s="64"/>
       <c r="B19" s="84" t="s">
         <v>41</v>
@@ -32344,7 +32404,7 @@
       <c r="BP21" s="94"/>
       <c r="BQ21" s="94"/>
     </row>
-    <row r="22" ht="15.25" spans="1:69">
+    <row r="22" ht="15.75" spans="1:69">
       <c r="A22" s="95" t="s">
         <v>2</v>
       </c>
@@ -32484,10 +32544,10 @@
         <v>86</v>
       </c>
       <c r="AU22" s="101" t="s">
+        <v>131</v>
+      </c>
+      <c r="AV22" s="101" t="s">
         <v>132</v>
-      </c>
-      <c r="AV22" s="101" t="s">
-        <v>133</v>
       </c>
       <c r="AW22" s="101" t="s">
         <v>91</v>
@@ -32553,15 +32613,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.25" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -32572,15 +32632,15 @@
       <c r="F23" s="104">
         <v>3</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>250</v>
       </c>
       <c r="H23" s="105">
         <f>F23*G23</f>
         <v>750</v>
       </c>
-      <c r="I23" t="s">
-        <v>139</v>
+      <c r="I23" t="s" s="0">
+        <v>138</v>
       </c>
       <c r="J23" s="105">
         <v>2</v>
@@ -32717,11 +32777,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
-        <v>150</v>
+      <c r="AV23" t="s" s="0">
+        <v>148</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -32761,11 +32821,11 @@
       <c r="BL23" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
-        <v>154</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>155</v>
+      <c r="BM23" t="s" s="0">
+        <v>152</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>153</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
Updated inspection WH in testdata
Updated inspection WH in testdata
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" firstSheet="7" activeTab="8"/>
+    <workbookView windowWidth="20490" windowHeight="7620" firstSheet="11" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="ImportDirectGRNUDGeneralSameUOM" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="179">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -406,10 +406,10 @@
     <t>RM KD</t>
   </si>
   <si>
-    <t>8230.87693</t>
+    <t>8111.26667</t>
   </si>
   <si>
-    <t>26</t>
+    <t>42</t>
   </si>
   <si>
     <t>VD Asbl. Val.</t>
@@ -448,10 +448,10 @@
     <t>ITEM-GWL-SIMILAR-RC-02</t>
   </si>
   <si>
-    <t>8156.97779</t>
+    <t>19792.25</t>
   </si>
   <si>
-    <t>54</t>
+    <t>36</t>
   </si>
   <si>
     <t>ITEM-GWL-SERVICE-RC-02</t>
@@ -463,52 +463,40 @@
     <t>1</t>
   </si>
   <si>
-    <t>8415</t>
-  </si>
-  <si>
-    <t>8213.55001</t>
-  </si>
-  <si>
-    <t>84</t>
+    <t>18</t>
   </si>
   <si>
     <t>ITEM-GWL-SERVICE-PL-02</t>
   </si>
   <si>
-    <t>ITEM-GWL-DISSIMILAR-02</t>
+    <t>ITEM-GWL-DISSIMILAR-04</t>
   </si>
   <si>
-    <t>23750.7</t>
+    <t>KGS</t>
   </si>
   <si>
-    <t>21855.47652</t>
+    <t>59375.9</t>
   </si>
   <si>
-    <t>31.344</t>
+    <t>3</t>
   </si>
   <si>
-    <t>ITEM-GWL-DISSIMILAR-RC-02</t>
+    <t>ITEM-GWL-DISSIMILAR-RC-04</t>
   </si>
   <si>
-    <t>25245</t>
+    <t>ITEM-GWL-DISSIMILAR-PL-04</t>
   </si>
   <si>
-    <t>24721.96746</t>
+    <t>INS WH-1</t>
   </si>
   <si>
-    <t>19.674</t>
+    <t>RM WH-49</t>
   </si>
   <si>
-    <t>ITEM-GWL-DISSIMILAR-PL-02</t>
+    <t>11653.51197</t>
   </si>
   <si>
-    <t>24598.03202</t>
-  </si>
-  <si>
-    <t>33.344</t>
-  </si>
-  <si>
-    <t>INS KD</t>
+    <t>71</t>
   </si>
   <si>
     <t>No.</t>
@@ -517,16 +505,10 @@
     <t>Item Desc</t>
   </si>
   <si>
-    <t>INS WH-1</t>
-  </si>
-  <si>
     <t>110</t>
   </si>
   <si>
     <t>124.545</t>
-  </si>
-  <si>
-    <t>RM WH-49</t>
   </si>
   <si>
     <t>5</t>
@@ -545,9 +527,6 @@
   </si>
   <si>
     <t>Disc amt</t>
-  </si>
-  <si>
-    <t>KGS</t>
   </si>
   <si>
     <t>REJ</t>
@@ -589,10 +568,7 @@
     <t>old UnitCost</t>
   </si>
   <si>
-    <t>1216.94021</t>
-  </si>
-  <si>
-    <t>1150</t>
+    <t>250</t>
   </si>
   <si>
     <t>15</t>
@@ -601,91 +577,10 @@
     <t>41.515</t>
   </si>
   <si>
-    <t>1115.07779</t>
-  </si>
-  <si>
-    <t>1105</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
-    <t>11143.5</t>
-  </si>
-  <si>
-    <t>3717.81605</t>
-  </si>
-  <si>
-    <t>248.661</t>
-  </si>
-  <si>
-    <t>4802.16109</t>
-  </si>
-  <si>
-    <t>209.665</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>8208.45001</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>8189.01334</t>
-  </si>
-  <si>
-    <t>19792.25</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>8500</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>8186.02307</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>8166.79999</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>8150.13999</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>8135.56249</t>
-  </si>
-  <si>
-    <t>19791.96667</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>36</t>
+    <t>55159.9</t>
   </si>
 </sst>
 </file>
@@ -1727,7 +1622,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49">
       <alignment vertical="center"/>
@@ -2396,74 +2291,74 @@
   <dimension ref="A1:BR24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="25.5714285714286"/>
-    <col min="2" max="2" customWidth="true" width="21.8571428571429"/>
-    <col min="3" max="3" customWidth="true" width="27.5714285714286"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="15.5714285714286"/>
-    <col min="48" max="48" customWidth="true" width="21.1428571428571"/>
-    <col min="49" max="49" customWidth="true" width="11.5714285714286"/>
-    <col min="50" max="50" customWidth="true" width="16.7142857142857"/>
-    <col min="51" max="51" customWidth="true" width="14.0"/>
-    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
-    <col min="53" max="53" customWidth="true" width="18.8571428571429"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="15.5714285714286"/>
-    <col min="56" max="56" customWidth="true" width="14.2857142857143"/>
-    <col min="57" max="57" customWidth="true" width="17.0"/>
-    <col min="58" max="58" customWidth="true" width="16.2857142857143"/>
-    <col min="59" max="59" customWidth="true" width="13.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="12.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="21.8571428571429"/>
-    <col min="63" max="63" customWidth="true" width="30.5714285714286"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="9.57142857142857"/>
-    <col min="70" max="70" customWidth="true" width="5.42857142857143"/>
+    <col min="1" max="1" width="25.5714285714286" customWidth="1"/>
+    <col min="2" max="2" width="21.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="27.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="15.5714285714286" customWidth="1"/>
+    <col min="48" max="48" width="21.1428571428571" customWidth="1"/>
+    <col min="49" max="49" width="11.5714285714286" customWidth="1"/>
+    <col min="50" max="50" width="16.7142857142857" customWidth="1"/>
+    <col min="51" max="51" width="14" customWidth="1"/>
+    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
+    <col min="53" max="53" width="18.8571428571429" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="15.5714285714286" customWidth="1"/>
+    <col min="56" max="56" width="14.2857142857143" customWidth="1"/>
+    <col min="57" max="57" width="17" customWidth="1"/>
+    <col min="58" max="58" width="16.2857142857143" customWidth="1"/>
+    <col min="59" max="59" width="13.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="12.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="21.8571428571429" customWidth="1"/>
+    <col min="63" max="63" width="30.5714285714286" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="9.57142857142857" customWidth="1"/>
+    <col min="70" max="70" width="5.42857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -4549,10 +4444,10 @@
       <c r="AT23" s="121" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>113</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>114</v>
       </c>
       <c r="AW23" s="121">
@@ -4593,11 +4488,11 @@
       <c r="BL23" s="121" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>196</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>195</v>
+      <c r="BM23" t="s">
+        <v>120</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>121</v>
       </c>
       <c r="BO23" s="121">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -4752,16 +4647,16 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="9.85714285714286" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.85714285714286"/>
-    <col min="2" max="2" customWidth="true" style="1" width="25.5714285714286"/>
-    <col min="3" max="3" customWidth="true" style="1" width="26.0"/>
-    <col min="4" max="19" style="1" width="9.85714285714286"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="51" style="1" width="9.85714285714286"/>
-    <col min="52" max="52" customWidth="true" style="1" width="11.5714285714286"/>
-    <col min="53" max="66" style="1" width="9.85714285714286"/>
-    <col min="67" max="67" style="1" width="12.0"/>
-    <col min="68" max="16384" style="1" width="9.85714285714286"/>
+    <col min="1" max="1" width="9.85714285714286" style="1"/>
+    <col min="2" max="2" width="25.5714285714286" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" customWidth="1"/>
+    <col min="4" max="19" width="9.85714285714286" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="51" width="9.85714285714286" style="1"/>
+    <col min="52" max="52" width="11.5714285714286" style="1" customWidth="1"/>
+    <col min="53" max="66" width="9.85714285714286" style="1"/>
+    <col min="67" max="67" width="12" style="1"/>
+    <col min="68" max="16384" width="9.85714285714286" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -5158,14 +5053,14 @@
         <v>12</v>
       </c>
       <c r="F4" s="22">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G4" s="22">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="H4" s="22">
         <f>F4*G4</f>
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="I4" s="22">
         <v>1</v>
@@ -5178,35 +5073,35 @@
       </c>
       <c r="L4" s="22">
         <f>H4</f>
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="M4" s="22">
         <f>ROUND(L4*I4%,2)</f>
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="N4" s="22">
         <f>H4-M4</f>
-        <v>742.5</v>
+        <v>495</v>
       </c>
       <c r="O4" s="22">
         <f>ROUND(N4*J4%,2)</f>
-        <v>59.4</v>
+        <v>39.6</v>
       </c>
       <c r="P4" s="22">
         <f>ROUND(N4-O4,2)</f>
-        <v>683.1</v>
+        <v>455.4</v>
       </c>
       <c r="Q4" s="22">
         <f>ROUND(P4*K4%,2)</f>
-        <v>34.16</v>
+        <v>22.77</v>
       </c>
       <c r="R4" s="22">
         <f>M4+O4+Q4</f>
-        <v>101.06</v>
+        <v>67.37</v>
       </c>
       <c r="S4" s="22">
         <f>(H4-R4)</f>
-        <v>648.94</v>
+        <v>432.63</v>
       </c>
       <c r="T4" s="22">
         <v>88363222</v>
@@ -5243,7 +5138,7 @@
       </c>
       <c r="AC4" s="22">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>648.94</v>
+        <v>432.63</v>
       </c>
       <c r="AD4" s="22">
         <v>120</v>
@@ -5263,7 +5158,7 @@
       </c>
       <c r="AI4" s="22">
         <f>S4*$M$2</f>
-        <v>648.94</v>
+        <v>432.63</v>
       </c>
       <c r="AJ4" s="22">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -5278,11 +5173,11 @@
       </c>
       <c r="AM4" s="22">
         <f>F4/AL4</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AN4" s="22">
         <f>AI4/AM4</f>
-        <v>129.788</v>
+        <v>216.315</v>
       </c>
       <c r="AO4" s="22">
         <f>AJ4/AM4</f>
@@ -5297,29 +5192,35 @@
       </c>
       <c r="AR4" s="6">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>129.788</v>
+        <v>216.315</v>
       </c>
       <c r="AS4" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
+      </c>
+      <c r="AU4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AX4" s="29">
         <f>AR4</f>
-        <v>129.788</v>
+        <v>216.315</v>
       </c>
       <c r="AY4" s="29">
         <f>AU4+AW4</f>
-        <v>14095</v>
+        <v>2</v>
       </c>
       <c r="AZ4" s="29">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),5)</f>
-        <v>129.788</v>
+        <v>216.315</v>
       </c>
       <c r="BA4" s="31"/>
       <c r="BB4" s="31" t="s">
@@ -5341,21 +5242,21 @@
       <c r="BJ4" s="6"/>
       <c r="BK4" s="6"/>
       <c r="BL4" s="29" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>113</v>
+        <v>150</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>129.788</v>
+        <v>216.315</v>
       </c>
       <c r="BP4" s="35">
         <f>BN4+AW4</f>
-        <v>696</v>
+        <v>2</v>
       </c>
       <c r="BQ4" s="36">
         <v>123562</v>
@@ -5373,7 +5274,7 @@
       <c r="G5" s="39"/>
       <c r="H5" s="40">
         <f>SUM(H4:H4)</f>
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="I5" s="20"/>
       <c r="J5" s="20"/>
@@ -5386,11 +5287,11 @@
       <c r="Q5" s="20"/>
       <c r="R5" s="41">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>101.06</v>
+        <v>67.37</v>
       </c>
       <c r="S5" s="40">
         <f t="shared" si="0"/>
-        <v>648.94</v>
+        <v>432.63</v>
       </c>
       <c r="T5" s="41"/>
       <c r="U5" s="41"/>
@@ -5415,7 +5316,7 @@
       </c>
       <c r="AC5" s="43">
         <f t="shared" si="1"/>
-        <v>648.94</v>
+        <v>432.63</v>
       </c>
       <c r="AD5" s="44">
         <f t="shared" si="1"/>
@@ -5436,7 +5337,7 @@
       </c>
       <c r="AI5" s="44">
         <f t="shared" si="2"/>
-        <v>648.94</v>
+        <v>432.63</v>
       </c>
       <c r="AJ5" s="44">
         <f t="shared" si="2"/>
@@ -5494,16 +5395,16 @@
   <dimension ref="A1:BQ17"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="1" width="8.71428571428571"/>
-    <col min="2" max="2" customWidth="true" style="1" width="19.1428571428571"/>
-    <col min="3" max="3" customWidth="true" style="1" width="25.8571428571429"/>
-    <col min="4" max="19" style="1" width="8.71428571428571"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="51" style="1" width="8.71428571428571"/>
-    <col min="52" max="52" style="1" width="12.0"/>
-    <col min="53" max="66" style="1" width="8.71428571428571"/>
-    <col min="67" max="67" style="1" width="12.0"/>
-    <col min="68" max="16384" style="1" width="8.71428571428571"/>
+    <col min="1" max="1" width="8.71428571428571" style="1"/>
+    <col min="2" max="2" width="19.1428571428571" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.8571428571429" style="1" customWidth="1"/>
+    <col min="4" max="19" width="8.71428571428571" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="51" width="8.71428571428571" style="1"/>
+    <col min="52" max="52" width="12" style="1"/>
+    <col min="53" max="66" width="8.71428571428571" style="1"/>
+    <col min="67" max="67" width="12" style="1"/>
+    <col min="68" max="16384" width="8.71428571428571" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -5676,13 +5577,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -5903,11 +5804,11 @@
         <v>2</v>
       </c>
       <c r="G4" s="22">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="H4" s="22">
         <f>F4*G4</f>
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="I4" s="22">
         <v>1</v>
@@ -5920,35 +5821,35 @@
       </c>
       <c r="L4" s="22">
         <f>H4</f>
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="M4" s="22">
         <f>ROUND(L4*I4%,2)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N4" s="22">
         <f>H4-M4</f>
-        <v>297</v>
+        <v>495</v>
       </c>
       <c r="O4" s="22">
         <f>ROUND(N4*J4%,2)</f>
-        <v>23.76</v>
+        <v>39.6</v>
       </c>
       <c r="P4" s="22">
         <f>ROUND(N4-O4,2)</f>
-        <v>273.24</v>
+        <v>455.4</v>
       </c>
       <c r="Q4" s="22">
         <f>ROUND(P4*K4%,2)</f>
-        <v>13.66</v>
+        <v>22.77</v>
       </c>
       <c r="R4" s="22">
         <f>M4+O4+Q4</f>
-        <v>40.42</v>
+        <v>67.37</v>
       </c>
       <c r="S4" s="22">
         <f>(H4-R4)</f>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="T4" s="22">
         <v>88363222</v>
@@ -5985,7 +5886,7 @@
       </c>
       <c r="AC4" s="26">
         <f>IF($V2=1,S4+AB4,S4)</f>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="AD4" s="24">
         <v>120</v>
@@ -6005,7 +5906,7 @@
       </c>
       <c r="AI4" s="24">
         <f>S4*$M$2</f>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="AJ4" s="24">
         <f>IF($C$2=3,0,AG4+AH4)</f>
@@ -6024,7 +5925,7 @@
       </c>
       <c r="AN4" s="24">
         <f>ROUND(AI4/AM4,5)</f>
-        <v>129.79</v>
+        <v>216.315</v>
       </c>
       <c r="AO4" s="24">
         <f>AJ4/AM4</f>
@@ -6039,19 +5940,19 @@
       </c>
       <c r="AR4" s="24">
         <f>ROUND(AN4+AO4+AP4,5)</f>
-        <v>129.79</v>
+        <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="AV4" s="23" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -6059,7 +5960,7 @@
       </c>
       <c r="AX4" s="29">
         <f>AR4</f>
-        <v>129.79</v>
+        <v>216.315</v>
       </c>
       <c r="AY4" s="29">
         <f>AU4+AW4</f>
@@ -6067,7 +5968,7 @@
       </c>
       <c r="AZ4" s="29">
         <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),5)</f>
-        <v>124.63866</v>
+        <v>126.18375</v>
       </c>
       <c r="BA4" s="31"/>
       <c r="BB4" s="31" t="s">
@@ -6089,17 +5990,17 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="23" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="BN4" s="23" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>124.57176</v>
+        <v>125.01321</v>
       </c>
       <c r="BP4" s="35">
         <f>BN4+AW4</f>
@@ -6121,7 +6022,7 @@
       <c r="G5" s="39"/>
       <c r="H5" s="40">
         <f>SUM(H4:H4)</f>
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="I5" s="20"/>
       <c r="J5" s="20"/>
@@ -6134,11 +6035,11 @@
       <c r="Q5" s="20"/>
       <c r="R5" s="41">
         <f t="shared" ref="R5:X5" si="0">SUM(R4:R4)</f>
-        <v>40.42</v>
+        <v>67.37</v>
       </c>
       <c r="S5" s="40">
         <f t="shared" si="0"/>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="T5" s="41"/>
       <c r="U5" s="41"/>
@@ -6163,7 +6064,7 @@
       </c>
       <c r="AC5" s="43">
         <f t="shared" si="1"/>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="AD5" s="44">
         <f t="shared" si="1"/>
@@ -6184,7 +6085,7 @@
       </c>
       <c r="AI5" s="44">
         <f t="shared" si="2"/>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="AJ5" s="44">
         <f t="shared" si="2"/>
@@ -6306,18 +6207,18 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="55" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="H7" s="56"/>
       <c r="I7" s="57">
         <f>H5</f>
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J7" s="57"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="58" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="N7" s="59"/>
       <c r="O7" s="59"/>
@@ -6366,10 +6267,10 @@
       <c r="BF7" s="5"/>
       <c r="BG7" s="5"/>
       <c r="BH7" s="5" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="BI7" s="148" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="BJ7" s="5"/>
       <c r="BK7" s="5"/>
@@ -6388,12 +6289,12 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="55" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="H8" s="56"/>
       <c r="I8" s="57">
         <f>R5</f>
-        <v>40.42</v>
+        <v>67.37</v>
       </c>
       <c r="J8" s="57"/>
       <c r="K8" s="5"/>
@@ -6408,7 +6309,7 @@
         <v>2</v>
       </c>
       <c r="P8" s="61" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
@@ -6454,10 +6355,10 @@
       <c r="BF8" s="5"/>
       <c r="BG8" s="5"/>
       <c r="BH8" s="5" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="BI8" s="148" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="BJ8" s="5"/>
       <c r="BK8" s="5"/>
@@ -6476,12 +6377,12 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="55" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="H9" s="56"/>
       <c r="I9" s="57">
         <f>S5</f>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="J9" s="57"/>
       <c r="K9" s="5"/>
@@ -6496,7 +6397,7 @@
         <v>2.5</v>
       </c>
       <c r="P9" s="20" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
@@ -6560,7 +6461,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="55" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="H10" s="56"/>
       <c r="I10" s="57">
@@ -6574,13 +6475,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="O10" s="20">
         <v>0.001</v>
       </c>
       <c r="P10" s="20" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="Q10" s="5"/>
       <c r="R10" s="5"/>
@@ -6644,12 +6545,12 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="55" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="H11" s="56"/>
       <c r="I11" s="62">
         <f>I9+I10</f>
-        <v>259.58</v>
+        <v>432.63</v>
       </c>
       <c r="J11" s="62"/>
       <c r="K11" s="5"/>
@@ -6778,10 +6679,10 @@
       <c r="BK12" s="5"/>
       <c r="BL12" s="5"/>
       <c r="BM12" s="5" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="BN12" s="5" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="BO12" s="5"/>
       <c r="BP12" s="6"/>
@@ -6851,7 +6752,7 @@
       <c r="BI13" s="5"/>
       <c r="BJ13" s="5"/>
       <c r="BK13" s="5" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="BL13" s="5">
         <v>12.5</v>
@@ -6932,7 +6833,7 @@
       <c r="BI14" s="5"/>
       <c r="BJ14" s="5"/>
       <c r="BK14" s="5" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="BL14" s="5">
         <v>487.4072</v>
@@ -7010,7 +6911,7 @@
       <c r="BI15" s="5"/>
       <c r="BJ15" s="5"/>
       <c r="BK15" s="5" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="BL15" s="5">
         <v>37.5</v>
@@ -7085,7 +6986,7 @@
       <c r="BI16" s="5"/>
       <c r="BJ16" s="5"/>
       <c r="BK16" s="5" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="BL16" s="5">
         <v>487.4072</v>
@@ -7202,16 +7103,16 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" style="1" width="8.71428571428571"/>
-    <col min="2" max="2" customWidth="true" style="1" width="21.1428571428571"/>
-    <col min="3" max="3" customWidth="true" style="1" width="21.2857142857143"/>
-    <col min="4" max="19" style="1" width="8.71428571428571"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="51" style="1" width="8.71428571428571"/>
-    <col min="52" max="52" style="1" width="10.5714285714286"/>
-    <col min="53" max="66" style="1" width="8.71428571428571"/>
-    <col min="67" max="67" style="1" width="13.2857142857143"/>
-    <col min="68" max="16384" style="1" width="8.71428571428571"/>
+    <col min="1" max="1" width="8.71428571428571" style="1"/>
+    <col min="2" max="2" width="21.1428571428571" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.2857142857143" style="1" customWidth="1"/>
+    <col min="4" max="19" width="8.71428571428571" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="51" width="8.71428571428571" style="1"/>
+    <col min="52" max="52" width="10.5714285714286" style="1"/>
+    <col min="53" max="66" width="8.71428571428571" style="1"/>
+    <col min="67" max="67" width="13.2857142857143" style="1"/>
+    <col min="68" max="16384" width="8.71428571428571" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7384,13 +7285,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -7610,15 +7511,15 @@
       <c r="F4" s="22">
         <v>2</v>
       </c>
-      <c r="G4" s="23">
-        <v>250</v>
+      <c r="G4" s="1" t="s">
+        <v>174</v>
       </c>
       <c r="H4" s="22">
         <f>F4*G4</f>
         <v>500</v>
       </c>
-      <c r="I4" s="23">
-        <v>1</v>
+      <c r="I4" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="J4" s="22">
         <v>8</v>
@@ -7750,16 +7651,10 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
-      </c>
-      <c r="AU4" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="AV4" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -7797,13 +7692,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>181</v>
+        <v>113</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>182</v>
+        <v>113</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -7954,16 +7849,16 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" style="1" width="8.71428571428571"/>
-    <col min="2" max="2" customWidth="true" style="1" width="23.4285714285714"/>
-    <col min="3" max="3" customWidth="true" style="1" width="29.4285714285714"/>
-    <col min="4" max="19" style="1" width="8.71428571428571"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="51" style="1" width="8.71428571428571"/>
-    <col min="52" max="52" style="1" width="10.7142857142857"/>
-    <col min="53" max="66" style="1" width="8.71428571428571"/>
-    <col min="67" max="67" style="1" width="10.5714285714286"/>
-    <col min="68" max="16384" style="1" width="8.71428571428571"/>
+    <col min="1" max="1" width="8.71428571428571" style="1"/>
+    <col min="2" max="2" width="23.4285714285714" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.4285714285714" style="1" customWidth="1"/>
+    <col min="4" max="19" width="8.71428571428571" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="51" width="8.71428571428571" style="1"/>
+    <col min="52" max="52" width="10.7142857142857" style="1"/>
+    <col min="53" max="66" width="8.71428571428571" style="1"/>
+    <col min="67" max="67" width="10.5714285714286" style="1"/>
+    <col min="68" max="16384" width="8.71428571428571" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -8136,13 +8031,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -8502,16 +8397,16 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="AV4" s="23" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -8549,13 +8444,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="23" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="BN4" s="23" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -8705,14 +8600,14 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" style="1" width="8.71428571428571"/>
-    <col min="2" max="2" customWidth="true" style="1" width="27.2857142857143"/>
-    <col min="3" max="3" customWidth="true" style="1" width="25.4285714285714"/>
-    <col min="4" max="19" style="1" width="8.71428571428571"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="66" style="1" width="8.71428571428571"/>
-    <col min="67" max="67" style="1" width="12.0"/>
-    <col min="68" max="16384" style="1" width="8.71428571428571"/>
+    <col min="1" max="1" width="8.71428571428571" style="1"/>
+    <col min="2" max="2" width="27.2857142857143" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.4285714285714" style="1" customWidth="1"/>
+    <col min="4" max="19" width="8.71428571428571" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="66" width="8.71428571428571" style="1"/>
+    <col min="67" max="67" width="12" style="1"/>
+    <col min="68" max="16384" width="8.71428571428571" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -8885,13 +8780,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -9251,7 +9146,7 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -9260,7 +9155,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>159</v>
+        <v>134</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -9274,10 +9169,7 @@
         <f>AU4+AW4</f>
         <v>2</v>
       </c>
-      <c r="AZ4" s="29">
-        <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),5)</f>
-        <v>216.315</v>
-      </c>
+      <c r="AZ4" s="29"/>
       <c r="BA4" s="31"/>
       <c r="BB4" s="31" t="s">
         <v>115</v>
@@ -9298,17 +9190,17 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>185</v>
+        <v>113</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>186</v>
+        <v>113</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>1113.45401</v>
+        <v>1113.0632</v>
       </c>
       <c r="BP4" s="35">
         <f>BN4+AW4</f>
@@ -9454,24 +9346,24 @@
   <dimension ref="A1:BQ18"/>
   <sheetFormatPr defaultColWidth="8.85714285714286" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="23" width="8.85714285714286"/>
-    <col min="2" max="2" customWidth="true" style="23" width="28.0"/>
-    <col min="3" max="3" customWidth="true" style="23" width="23.0"/>
-    <col min="4" max="11" style="23" width="8.85714285714286"/>
-    <col min="12" max="12" customWidth="true" style="23" width="15.7142857142857"/>
-    <col min="13" max="13" customWidth="true" style="23" width="9.14285714285714"/>
-    <col min="14" max="14" customWidth="true" style="23" width="13.8571428571429"/>
-    <col min="15" max="15" customWidth="true" style="23" width="11.2857142857143"/>
-    <col min="16" max="16" customWidth="true" style="23" width="17.8571428571429"/>
-    <col min="17" max="19" style="23" width="8.85714285714286"/>
-    <col min="20" max="20" customWidth="true" style="23" width="10.1428571428571"/>
-    <col min="21" max="51" style="23" width="8.85714285714286"/>
-    <col min="52" max="52" style="23" width="10.7142857142857"/>
-    <col min="53" max="63" style="23" width="8.85714285714286"/>
-    <col min="64" max="64" customWidth="true" style="23" width="11.0"/>
-    <col min="65" max="66" style="23" width="8.85714285714286"/>
-    <col min="67" max="67" style="23" width="10.7142857142857"/>
-    <col min="68" max="16384" style="23" width="8.85714285714286"/>
+    <col min="1" max="1" width="8.85714285714286" style="23"/>
+    <col min="2" max="2" width="28" style="23" customWidth="1"/>
+    <col min="3" max="3" width="23" style="23" customWidth="1"/>
+    <col min="4" max="11" width="8.85714285714286" style="23"/>
+    <col min="12" max="12" width="15.7142857142857" style="23" customWidth="1"/>
+    <col min="13" max="13" width="9.14285714285714" style="23" customWidth="1"/>
+    <col min="14" max="14" width="13.8571428571429" style="23" customWidth="1"/>
+    <col min="15" max="15" width="11.2857142857143" style="23" customWidth="1"/>
+    <col min="16" max="16" width="17.8571428571429" style="23" customWidth="1"/>
+    <col min="17" max="19" width="8.85714285714286" style="23"/>
+    <col min="20" max="20" width="10.1428571428571" style="23" customWidth="1"/>
+    <col min="21" max="51" width="8.85714285714286" style="23"/>
+    <col min="52" max="52" width="10.7142857142857" style="23"/>
+    <col min="53" max="63" width="8.85714285714286" style="23"/>
+    <col min="64" max="64" width="11" style="23" customWidth="1"/>
+    <col min="65" max="66" width="8.85714285714286" style="23"/>
+    <col min="67" max="67" width="10.7142857142857" style="23"/>
+    <col min="68" max="16384" width="8.85714285714286" style="23"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -9644,13 +9536,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -9856,10 +9748,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -10010,16 +9902,16 @@
         <v>216.315</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="AV4" s="23" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -10057,13 +9949,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="23" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="BN4" s="23" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -10274,7 +10166,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="55" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="H7" s="56"/>
       <c r="I7" s="57">
@@ -10285,7 +10177,7 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="58" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="N7" s="59"/>
       <c r="O7" s="59"/>
@@ -10334,10 +10226,10 @@
       <c r="BF7" s="5"/>
       <c r="BG7" s="5"/>
       <c r="BH7" s="5" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="BI7" s="148" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="BJ7" s="5"/>
       <c r="BK7" s="5"/>
@@ -10356,7 +10248,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="55" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="H8" s="56"/>
       <c r="I8" s="57">
@@ -10376,7 +10268,7 @@
         <v>2</v>
       </c>
       <c r="P8" s="61" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
@@ -10422,10 +10314,10 @@
       <c r="BF8" s="5"/>
       <c r="BG8" s="5"/>
       <c r="BH8" s="5" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="BI8" s="148" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="BJ8" s="5"/>
       <c r="BK8" s="5"/>
@@ -10444,7 +10336,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="55" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="H9" s="56"/>
       <c r="I9" s="57">
@@ -10464,7 +10356,7 @@
         <v>2.5</v>
       </c>
       <c r="P9" s="20" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
@@ -10528,7 +10420,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="55" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="H10" s="56"/>
       <c r="I10" s="57">
@@ -10542,13 +10434,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="O10" s="20">
         <v>0.001</v>
       </c>
       <c r="P10" s="20" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="Q10" s="5"/>
       <c r="R10" s="5"/>
@@ -10612,7 +10504,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="55" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="H11" s="56"/>
       <c r="I11" s="62">
@@ -10746,10 +10638,10 @@
       <c r="BK12" s="5"/>
       <c r="BL12" s="5"/>
       <c r="BM12" s="5" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="BN12" s="5" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="BO12" s="5"/>
       <c r="BP12" s="6"/>
@@ -10819,7 +10711,7 @@
       <c r="BI13" s="5"/>
       <c r="BJ13" s="5"/>
       <c r="BK13" s="5" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="BL13" s="5">
         <v>12.5</v>
@@ -10900,7 +10792,7 @@
       <c r="BI14" s="5"/>
       <c r="BJ14" s="5"/>
       <c r="BK14" s="5" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="BL14" s="5">
         <v>487.4072</v>
@@ -10978,7 +10870,7 @@
       <c r="BI15" s="5"/>
       <c r="BJ15" s="5"/>
       <c r="BK15" s="5" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="BL15" s="5">
         <v>37.5</v>
@@ -11053,7 +10945,7 @@
       <c r="BI16" s="5"/>
       <c r="BJ16" s="5"/>
       <c r="BK16" s="5" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="BL16" s="5">
         <v>487.4072</v>
@@ -11241,12 +11133,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="9.85714285714286" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.85714285714286"/>
-    <col min="2" max="2" customWidth="true" style="1" width="25.5714285714286"/>
-    <col min="3" max="3" customWidth="true" style="1" width="26.0"/>
-    <col min="4" max="19" style="1" width="9.85714285714286"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="16384" style="1" width="9.85714285714286"/>
+    <col min="1" max="1" width="9.85714285714286" style="1"/>
+    <col min="2" max="2" width="25.5714285714286" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" customWidth="1"/>
+    <col min="4" max="19" width="9.85714285714286" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.85714285714286" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -11631,16 +11523,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -11785,10 +11677,16 @@
         <v>648.94</v>
       </c>
       <c r="AS4" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
+      </c>
+      <c r="AU4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -11826,13 +11724,13 @@
       <c r="BJ4" s="6"/>
       <c r="BK4" s="6"/>
       <c r="BL4" s="29" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>113</v>
+        <v>178</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>113</v>
+        <v>144</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -11979,14 +11877,14 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" style="1" width="8.71428571428571"/>
-    <col min="2" max="3" customWidth="true" style="1" width="26.5428571428571"/>
-    <col min="4" max="19" style="1" width="8.71428571428571"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="66" style="1" width="8.71428571428571"/>
-    <col min="67" max="67" style="1" width="13.2857142857143"/>
-    <col min="68" max="68" style="1" width="12.8571428571429"/>
-    <col min="69" max="16384" style="1" width="8.71428571428571"/>
+    <col min="1" max="1" width="8.71428571428571" style="1"/>
+    <col min="2" max="3" width="26.5428571428571" style="1" customWidth="1"/>
+    <col min="4" max="19" width="8.71428571428571" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="66" width="8.71428571428571" style="1"/>
+    <col min="67" max="67" width="13.2857142857143" style="1"/>
+    <col min="68" max="68" width="12.8571428571429" style="1"/>
+    <col min="69" max="16384" width="8.71428571428571" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -12159,13 +12057,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -12371,16 +12269,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -12525,7 +12423,7 @@
         <v>648.94</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -12534,7 +12432,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>188</v>
+        <v>143</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -12572,13 +12470,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>189</v>
+        <v>113</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>190</v>
+        <v>113</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -12728,16 +12626,16 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" style="1" width="8.71428571428571"/>
-    <col min="2" max="2" customWidth="true" style="1" width="27.2857142857143"/>
-    <col min="3" max="3" customWidth="true" style="1" width="25.4285714285714"/>
-    <col min="4" max="19" style="1" width="8.71428571428571"/>
-    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
-    <col min="21" max="51" style="1" width="8.71428571428571"/>
-    <col min="52" max="52" style="1" width="9.0"/>
-    <col min="53" max="66" style="1" width="8.71428571428571"/>
-    <col min="67" max="67" style="1" width="13.2857142857143"/>
-    <col min="68" max="16384" style="1" width="8.71428571428571"/>
+    <col min="1" max="1" width="8.71428571428571" style="1"/>
+    <col min="2" max="2" width="27.2857142857143" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.4285714285714" style="1" customWidth="1"/>
+    <col min="4" max="19" width="8.71428571428571" style="1"/>
+    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
+    <col min="21" max="51" width="8.71428571428571" style="1"/>
+    <col min="52" max="52" width="9" style="1"/>
+    <col min="53" max="66" width="8.71428571428571" style="1"/>
+    <col min="67" max="67" width="13.2857142857143" style="1"/>
+    <col min="68" max="16384" width="8.71428571428571" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -12910,13 +12808,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -13122,16 +13020,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -13276,7 +13174,7 @@
         <v>648.94</v>
       </c>
       <c r="AS4" s="28" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AT4" s="29" t="s">
         <v>12</v>
@@ -13285,7 +13183,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>188</v>
+        <v>143</v>
       </c>
       <c r="AW4" s="29">
         <f>AM4</f>
@@ -13323,13 +13221,13 @@
       <c r="BJ4" s="29"/>
       <c r="BK4" s="29"/>
       <c r="BL4" s="34" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>191</v>
+        <v>113</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>192</v>
+        <v>113</v>
       </c>
       <c r="BO4" s="29">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -13479,71 +13377,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="22.0"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="9" customWidth="true" width="5.85714285714286"/>
-    <col min="10" max="10" customWidth="true" width="6.0"/>
-    <col min="11" max="11" customWidth="true" width="5.85714285714286"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.4285714285714"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="11.8571428571429"/>
-    <col min="20" max="20" customWidth="true" width="10.7142857142857"/>
-    <col min="21" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="23.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="18.0"/>
-    <col min="48" max="48" customWidth="true" width="24.4285714285714"/>
-    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="9.42857142857143"/>
-    <col min="65" max="65" customWidth="true" width="49.1428571428571"/>
-    <col min="66" max="66" customWidth="true" width="43.8571428571429"/>
-    <col min="67" max="67" customWidth="true" width="22.7142857142857"/>
-    <col min="68" max="68" customWidth="true" width="40.8571428571429"/>
-    <col min="69" max="69" customWidth="true" width="7.57142857142857"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="9" width="5.85714285714286" customWidth="1"/>
+    <col min="10" max="10" width="6" customWidth="1"/>
+    <col min="11" max="11" width="5.85714285714286" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.4285714285714" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="11.8571428571429" customWidth="1"/>
+    <col min="20" max="20" width="10.7142857142857" customWidth="1"/>
+    <col min="21" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="23.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="18" customWidth="1"/>
+    <col min="48" max="48" width="24.4285714285714" customWidth="1"/>
+    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="9.42857142857143" customWidth="1"/>
+    <col min="65" max="65" width="49.1428571428571" customWidth="1"/>
+    <col min="66" max="66" width="43.8571428571429" customWidth="1"/>
+    <col min="67" max="67" width="22.7142857142857" customWidth="1"/>
+    <col min="68" max="68" width="40.8571428571429" customWidth="1"/>
+    <col min="69" max="69" width="7.57142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -15922,71 +15820,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="25.2857142857143"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
-    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
-    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="25.2857142857143" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
+    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
+    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -18159,11 +18057,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>113</v>
       </c>
-      <c r="AV23" t="s" s="0">
-        <v>197</v>
+      <c r="AV23" t="s">
+        <v>134</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -18203,11 +18101,11 @@
       <c r="BL23" s="121" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>197</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>199</v>
+      <c r="BM23" t="s">
+        <v>134</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>135</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -18362,71 +18260,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="25.5714285714286"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
-    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
-    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="25.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
+    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
+    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -20435,7 +20333,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
@@ -20788,71 +20686,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="24.7142857142857"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
-    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
-    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="24.7142857142857" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
+    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
+    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -22880,14 +22778,14 @@
       <c r="F23" s="104">
         <v>2</v>
       </c>
-      <c r="G23" s="0">
+      <c r="G23">
         <v>250</v>
       </c>
       <c r="H23" s="105">
         <f>F23*G23</f>
         <v>500</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>138</v>
       </c>
       <c r="J23" s="105">
@@ -23025,11 +22923,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>113</v>
       </c>
-      <c r="AV23" t="s" s="0">
-        <v>197</v>
+      <c r="AV23" t="s">
+        <v>134</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -23069,11 +22967,11 @@
       <c r="BL23" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>197</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>201</v>
+      <c r="BM23" t="s">
+        <v>134</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>139</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -23228,71 +23126,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="25.1428571428571"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
-    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
-    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="25.1428571428571" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
+    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
+    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -25301,15 +25199,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="89" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C23" s="89" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -25320,14 +25218,14 @@
       <c r="F23" s="104">
         <v>2</v>
       </c>
-      <c r="G23" s="0">
+      <c r="G23">
         <v>250</v>
       </c>
       <c r="H23" s="105">
         <f>F23*G23</f>
         <v>500</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>138</v>
       </c>
       <c r="J23" s="105">
@@ -25660,71 +25558,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="24.5714285714286"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
-    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
-    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="24.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
+    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
+    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -27733,31 +27631,31 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="89" t="s">
-        <v>12</v>
+        <v>142</v>
       </c>
       <c r="F23" s="104">
         <v>3</v>
       </c>
       <c r="G23" s="104">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="H23" s="105">
         <f>F23*G23</f>
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="I23" s="117">
         <v>1</v>
@@ -27770,35 +27668,35 @@
       </c>
       <c r="L23" s="105">
         <f>H23</f>
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="M23" s="105">
         <f>ROUND(L23*I23%,2)</f>
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="N23" s="105">
         <f>H23-M23</f>
-        <v>297</v>
+        <v>742.5</v>
       </c>
       <c r="O23" s="105">
         <f>ROUND(N23*J23%,2)</f>
-        <v>5.94</v>
+        <v>14.85</v>
       </c>
       <c r="P23" s="105">
         <f>ROUND(N23-O23,2)</f>
-        <v>291.06</v>
+        <v>727.65</v>
       </c>
       <c r="Q23" s="105">
         <f>ROUND(P23*K23%,2)</f>
-        <v>11.64</v>
+        <v>29.11</v>
       </c>
       <c r="R23" s="105">
         <f>M23+O23+Q23</f>
-        <v>20.58</v>
+        <v>51.46</v>
       </c>
       <c r="S23" s="105">
         <f>(H23-R23)</f>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="T23" s="105" t="s">
         <v>111</v>
@@ -27835,7 +27733,7 @@
       </c>
       <c r="AC23" s="105">
         <f>IF($V21=1,S23+AB23,S23)</f>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="AD23" s="105">
         <v>120</v>
@@ -27855,7 +27753,7 @@
       </c>
       <c r="AI23" s="105">
         <f>S23*$M$21</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AJ23" s="105">
         <f>IF($C$21=3,0,AG23+AH23)</f>
@@ -27874,7 +27772,7 @@
       </c>
       <c r="AN23" s="105">
         <f>AI23/AM23</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AO23" s="105">
         <f>AJ23/AM23</f>
@@ -27889,7 +27787,7 @@
       </c>
       <c r="AR23" s="105">
         <f>AN23+AO23+AP23</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AS23" s="105" t="s">
         <v>112</v>
@@ -27897,11 +27795,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>113</v>
       </c>
-      <c r="AV23" t="s" s="0">
-        <v>114</v>
+      <c r="AV23" t="s">
+        <v>143</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -27909,7 +27807,7 @@
       </c>
       <c r="AX23" s="105">
         <f>AR23</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AY23" s="105">
         <f>AU23+AW23</f>
@@ -27917,7 +27815,7 @@
       </c>
       <c r="AZ23" s="105">
         <f>ROUND(((AU23*AV23)+(AW23*AX23))/(AU23+AW23),5)</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="BA23" s="107"/>
       <c r="BB23" s="107" t="s">
@@ -27941,15 +27839,15 @@
       <c r="BL23" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>210</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>209</v>
+      <c r="BM23" t="s">
+        <v>143</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>144</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>21092.09434</v>
+        <v>9181.28366</v>
       </c>
       <c r="BP23" s="109">
         <f>BN23+AW23</f>
@@ -27971,7 +27869,7 @@
       <c r="G24" s="111"/>
       <c r="H24" s="111">
         <f>SUM(H23:H23)</f>
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="I24" s="93"/>
       <c r="J24" s="93"/>
@@ -27984,11 +27882,11 @@
       <c r="Q24" s="93"/>
       <c r="R24" s="111">
         <f t="shared" ref="R24:Y24" si="1">SUM(R23:R23)</f>
-        <v>20.58</v>
+        <v>51.46</v>
       </c>
       <c r="S24" s="112">
         <f t="shared" si="1"/>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="T24" s="111"/>
       <c r="U24" s="111"/>
@@ -28019,7 +27917,7 @@
       </c>
       <c r="AC24" s="114">
         <f t="shared" si="2"/>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="AD24" s="115">
         <f t="shared" si="2"/>
@@ -28040,7 +27938,7 @@
       </c>
       <c r="AI24" s="115">
         <f t="shared" si="3"/>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AJ24" s="115">
         <f t="shared" si="3"/>
@@ -28100,71 +27998,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="28.0"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
-    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
-    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
+    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
+    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -30173,15 +30071,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -30337,11 +30235,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>113</v>
       </c>
-      <c r="AV23" t="s" s="0">
-        <v>211</v>
+      <c r="AV23" t="s">
+        <v>143</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -30381,11 +30279,11 @@
       <c r="BL23" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>211</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>213</v>
+      <c r="BM23" t="s">
+        <v>143</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>144</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -30540,71 +30438,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
-    <col min="2" max="3" customWidth="true" width="27.5714285714286"/>
-    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
-    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
-    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
-    <col min="7" max="7" customWidth="true" width="11.0"/>
-    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
-    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
-    <col min="11" max="11" customWidth="true" width="6.0"/>
-    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
-    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
-    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
-    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
-    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
-    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
-    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
-    <col min="19" max="19" customWidth="true" width="10.0"/>
-    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
-    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
-    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
-    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
-    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
-    <col min="25" max="25" customWidth="true" width="8.0"/>
-    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
-    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
-    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
-    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
-    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
-    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
-    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
-    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
-    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
-    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
-    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
-    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
-    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
-    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
-    <col min="40" max="40" customWidth="true" width="22.0"/>
-    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
-    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
-    <col min="43" max="43" customWidth="true" width="13.0"/>
-    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
-    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
-    <col min="46" max="46" customWidth="true" width="13.0"/>
-    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
-    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
-    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
-    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
-    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
-    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
-    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
-    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
-    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
-    <col min="56" max="56" customWidth="true" width="16.0"/>
-    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
-    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
-    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
-    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
-    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
-    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
-    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
-    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
-    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
-    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
-    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
+    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
+    <col min="2" max="3" width="27.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
+    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
+    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
+    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
+    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
+    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
+    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
+    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
+    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
+    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
+    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
+    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
+    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
+    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
+    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
+    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
+    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
+    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
+    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
+    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
+    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
+    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
+    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
+    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
+    <col min="43" max="43" width="13" customWidth="1"/>
+    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
+    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
+    <col min="46" max="46" width="13" customWidth="1"/>
+    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
+    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
+    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
+    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
+    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
+    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
+    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
+    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
+    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
+    <col min="56" max="56" width="16" customWidth="1"/>
+    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
+    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
+    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
+    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
+    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
+    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
+    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
+    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
+    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
+    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
+    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -32613,15 +32511,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:69">
+    <row r="23" ht="15.75" spans="1:69">
       <c r="A23" s="89">
         <v>1</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D23" s="89" t="s">
         <v>12</v>
@@ -32632,14 +32530,14 @@
       <c r="F23" s="104">
         <v>3</v>
       </c>
-      <c r="G23" s="0">
+      <c r="G23">
         <v>250</v>
       </c>
       <c r="H23" s="105">
         <f>F23*G23</f>
         <v>750</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>138</v>
       </c>
       <c r="J23" s="105">
@@ -32777,11 +32675,11 @@
       <c r="AT23" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>113</v>
       </c>
-      <c r="AV23" t="s" s="0">
-        <v>148</v>
+      <c r="AV23" t="s">
+        <v>143</v>
       </c>
       <c r="AW23" s="105">
         <f>AM23</f>
@@ -32821,11 +32719,11 @@
       <c r="BL23" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>152</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>153</v>
+      <c r="BM23" t="s">
+        <v>143</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>144</v>
       </c>
       <c r="BO23" s="105">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
Phase-4 Purchase module fixes
Phase-4 Purchase module fixes
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2394" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="182">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -581,6 +581,9 @@
   </si>
   <si>
     <t>41.515</t>
+  </si>
+  <si>
+    <t>16</t>
   </si>
   <si>
     <t>10</t>
@@ -7122,8 +7125,14 @@
     <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
     <col min="21" max="28" width="8.71428571428571" style="1"/>
     <col min="29" max="29" width="9.28571428571429" style="1"/>
-    <col min="30" max="51" width="8.71428571428571" style="1"/>
-    <col min="52" max="52" width="10.5714285714286" style="1"/>
+    <col min="30" max="39" width="8.71428571428571" style="1"/>
+    <col min="40" max="40" width="10.1428571428571" style="1"/>
+    <col min="41" max="43" width="8.71428571428571" style="1"/>
+    <col min="44" max="44" width="10.1428571428571" style="1"/>
+    <col min="45" max="49" width="8.71428571428571" style="1"/>
+    <col min="50" max="50" width="10.1428571428571" style="1"/>
+    <col min="51" max="51" width="8.71428571428571" style="1"/>
+    <col min="52" max="52" width="12" style="1"/>
     <col min="53" max="66" width="8.71428571428571" style="1"/>
     <col min="67" max="67" width="13.2857142857143" style="1"/>
     <col min="68" max="16384" width="8.71428571428571" style="1"/>
@@ -7297,7 +7306,7 @@
       <c r="BP2" s="6"/>
       <c r="BQ2" s="6"/>
     </row>
-    <row r="3" ht="61.5" spans="1:69">
+    <row r="3" ht="46.5" spans="1:69">
       <c r="A3" s="10" t="s">
         <v>153</v>
       </c>
@@ -8629,7 +8638,9 @@
     <col min="44" max="44" width="10.1428571428571" style="1"/>
     <col min="45" max="49" width="8.71428571428571" style="1"/>
     <col min="50" max="50" width="10.1428571428571" style="1"/>
-    <col min="51" max="66" width="8.71428571428571" style="1"/>
+    <col min="51" max="51" width="8.71428571428571" style="1"/>
+    <col min="52" max="52" width="12" style="1"/>
+    <col min="53" max="66" width="8.71428571428571" style="1"/>
     <col min="67" max="67" width="12" style="1"/>
     <col min="68" max="16384" width="8.71428571428571" style="1"/>
   </cols>
@@ -9011,7 +9022,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
@@ -9175,6 +9186,12 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
+      <c r="AU4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="1" t="s">
+        <v>149</v>
+      </c>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>2</v>
@@ -9187,7 +9204,10 @@
         <f>AU4+AW4</f>
         <v>2</v>
       </c>
-      <c r="AZ4" s="28"/>
+      <c r="AZ4" s="28">
+        <f>ROUND(((AU4*AV4)+(AW4*AX4))/(AU4+AW4),5)</f>
+        <v>18386.775</v>
+      </c>
       <c r="BA4" s="30"/>
       <c r="BB4" s="30" t="s">
         <v>115</v>
@@ -9211,14 +9231,14 @@
         <v>150</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="BN4" s="1" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>1113.0632</v>
+        <v>18386.775</v>
       </c>
       <c r="BP4" s="34">
         <f>BN4+AW4</f>
@@ -9228,7 +9248,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" ht="15.75" spans="1:69">
+    <row r="5" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="36"/>
       <c r="C5" s="36"/>
@@ -9927,7 +9947,7 @@
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AV4" s="23" t="s">
         <v>178</v>
@@ -11705,7 +11725,7 @@
         <v>113</v>
       </c>
       <c r="AV4" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -11746,7 +11766,7 @@
         <v>150</v>
       </c>
       <c r="BM4" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="BN4" s="1" t="s">
         <v>147</v>

</xml_diff>

<commit_message>
Updated GRN and PO to GRN fixes
Updated GRN and PO to GRN fixes
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2788" uniqueCount="211">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -590,6 +590,93 @@
   </si>
   <si>
     <t>55159.9</t>
+  </si>
+  <si>
+    <t>282</t>
+  </si>
+  <si>
+    <t>7945.84822</t>
+  </si>
+  <si>
+    <t>276</t>
+  </si>
+  <si>
+    <t>254</t>
+  </si>
+  <si>
+    <t>132</t>
+  </si>
+  <si>
+    <t>127</t>
+  </si>
+  <si>
+    <t>124</t>
+  </si>
+  <si>
+    <t>323</t>
+  </si>
+  <si>
+    <t>16906.70787</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>212</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>98</t>
+  </si>
+  <si>
+    <t>96</t>
+  </si>
+  <si>
+    <t>284</t>
+  </si>
+  <si>
+    <t>7945.64436</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>133</t>
+  </si>
+  <si>
+    <t>286</t>
+  </si>
+  <si>
+    <t>7945.44335</t>
+  </si>
+  <si>
+    <t>288</t>
+  </si>
+  <si>
+    <t>7945.24513</t>
+  </si>
+  <si>
+    <t>278</t>
+  </si>
+  <si>
+    <t>258</t>
+  </si>
+  <si>
+    <t>290</t>
+  </si>
+  <si>
+    <t>7945.04965</t>
+  </si>
+  <si>
+    <t>280</t>
+  </si>
+  <si>
+    <t>260</t>
+  </si>
+  <si>
+    <t>134</t>
   </si>
 </sst>
 </file>
@@ -1629,7 +1716,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49">
       <alignment vertical="center"/>
@@ -2297,74 +2384,74 @@
   <dimension ref="A1:BR24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.5714285714286" customWidth="1"/>
-    <col min="2" max="2" width="21.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="27.5714285714286" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="15.5714285714286" customWidth="1"/>
-    <col min="48" max="48" width="21.1428571428571" customWidth="1"/>
-    <col min="49" max="49" width="11.5714285714286" customWidth="1"/>
-    <col min="50" max="50" width="16.7142857142857" customWidth="1"/>
-    <col min="51" max="51" width="14" customWidth="1"/>
-    <col min="52" max="52" width="19.4285714285714" customWidth="1"/>
-    <col min="53" max="53" width="18.8571428571429" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="15.5714285714286" customWidth="1"/>
-    <col min="56" max="56" width="14.2857142857143" customWidth="1"/>
-    <col min="57" max="57" width="17" customWidth="1"/>
-    <col min="58" max="58" width="16.2857142857143" customWidth="1"/>
-    <col min="59" max="59" width="13.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="12.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="21.8571428571429" customWidth="1"/>
-    <col min="63" max="63" width="30.5714285714286" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="9.57142857142857" customWidth="1"/>
-    <col min="70" max="70" width="5.42857142857143" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="25.5714285714286"/>
+    <col min="2" max="2" customWidth="true" width="21.8571428571429"/>
+    <col min="3" max="3" customWidth="true" width="27.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="15.5714285714286"/>
+    <col min="48" max="48" customWidth="true" width="21.1428571428571"/>
+    <col min="49" max="49" customWidth="true" width="11.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="16.7142857142857"/>
+    <col min="51" max="51" customWidth="true" width="14.0"/>
+    <col min="52" max="52" customWidth="true" width="19.4285714285714"/>
+    <col min="53" max="53" customWidth="true" width="18.8571428571429"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="15.5714285714286"/>
+    <col min="56" max="56" customWidth="true" width="14.2857142857143"/>
+    <col min="57" max="57" customWidth="true" width="17.0"/>
+    <col min="58" max="58" customWidth="true" width="16.2857142857143"/>
+    <col min="59" max="59" customWidth="true" width="13.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="12.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="21.8571428571429"/>
+    <col min="63" max="63" customWidth="true" width="30.5714285714286"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="9.57142857142857"/>
+    <col min="70" max="70" customWidth="true" width="5.42857142857143"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -4450,10 +4537,10 @@
       <c r="AT23" s="121" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>114</v>
       </c>
       <c r="AW23" s="121">
@@ -4494,11 +4581,11 @@
       <c r="BL23" s="121" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
-        <v>120</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>121</v>
+      <c r="BM23" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>206</v>
       </c>
       <c r="BO23" s="121">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -4653,24 +4740,24 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="9.85714285714286" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="9.85714285714286" style="1"/>
-    <col min="2" max="2" width="25.5714285714286" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="19" width="9.85714285714286" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="34" width="9.85714285714286" style="1"/>
-    <col min="35" max="35" width="11.4285714285714" style="1"/>
-    <col min="36" max="38" width="9.85714285714286" style="1"/>
-    <col min="39" max="39" width="17.4285714285714" style="1" customWidth="1"/>
-    <col min="40" max="43" width="9.85714285714286" style="1"/>
-    <col min="44" max="44" width="25.7142857142857" style="1" customWidth="1"/>
-    <col min="45" max="49" width="9.85714285714286" style="1"/>
-    <col min="50" max="50" width="16.7142857142857" style="1" customWidth="1"/>
-    <col min="51" max="51" width="9.85714285714286" style="1"/>
-    <col min="52" max="52" width="11.5714285714286" style="1" customWidth="1"/>
-    <col min="53" max="66" width="9.85714285714286" style="1"/>
-    <col min="67" max="67" width="12" style="1"/>
-    <col min="68" max="16384" width="9.85714285714286" style="1"/>
+    <col min="1" max="1" style="1" width="9.85714285714286"/>
+    <col min="2" max="2" customWidth="true" style="1" width="25.5714285714286"/>
+    <col min="3" max="3" customWidth="true" style="1" width="26.0"/>
+    <col min="4" max="19" style="1" width="9.85714285714286"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="34" style="1" width="9.85714285714286"/>
+    <col min="35" max="35" style="1" width="11.4285714285714"/>
+    <col min="36" max="38" style="1" width="9.85714285714286"/>
+    <col min="39" max="39" customWidth="true" style="1" width="17.4285714285714"/>
+    <col min="40" max="43" style="1" width="9.85714285714286"/>
+    <col min="44" max="44" customWidth="true" style="1" width="25.7142857142857"/>
+    <col min="45" max="49" style="1" width="9.85714285714286"/>
+    <col min="50" max="50" customWidth="true" style="1" width="16.7142857142857"/>
+    <col min="51" max="51" style="1" width="9.85714285714286"/>
+    <col min="52" max="52" customWidth="true" style="1" width="11.5714285714286"/>
+    <col min="53" max="66" style="1" width="9.85714285714286"/>
+    <col min="67" max="67" style="1" width="12.0"/>
+    <col min="68" max="16384" style="1" width="9.85714285714286"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -5214,10 +5301,10 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AU4" t="s" s="1">
         <v>113</v>
       </c>
-      <c r="AV4" s="1" t="s">
+      <c r="AV4" t="s" s="1">
         <v>149</v>
       </c>
       <c r="AW4" s="28">
@@ -5258,11 +5345,11 @@
       <c r="BL4" s="28" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>152</v>
+      <c r="BM4" t="s" s="1">
+        <v>190</v>
+      </c>
+      <c r="BN4" t="s" s="1">
+        <v>189</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -5409,16 +5496,16 @@
   <dimension ref="A1:BQ17"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.71428571428571" style="1"/>
-    <col min="2" max="2" width="19.1428571428571" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.8571428571429" style="1" customWidth="1"/>
-    <col min="4" max="19" width="8.71428571428571" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="51" width="8.71428571428571" style="1"/>
-    <col min="52" max="52" width="12" style="1"/>
-    <col min="53" max="66" width="8.71428571428571" style="1"/>
-    <col min="67" max="67" width="12" style="1"/>
-    <col min="68" max="16384" width="8.71428571428571" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="19.1428571428571"/>
+    <col min="3" max="3" customWidth="true" style="1" width="25.8571428571429"/>
+    <col min="4" max="19" style="1" width="8.71428571428571"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="12.0"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="12.0"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7117,25 +7204,25 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71428571428571" style="1"/>
-    <col min="2" max="2" width="21.1428571428571" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.2857142857143" style="1" customWidth="1"/>
-    <col min="4" max="18" width="8.71428571428571" style="1"/>
-    <col min="19" max="19" width="9.28571428571429" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="28" width="8.71428571428571" style="1"/>
-    <col min="29" max="29" width="9.28571428571429" style="1"/>
-    <col min="30" max="39" width="8.71428571428571" style="1"/>
-    <col min="40" max="40" width="10.1428571428571" style="1"/>
-    <col min="41" max="43" width="8.71428571428571" style="1"/>
-    <col min="44" max="44" width="10.1428571428571" style="1"/>
-    <col min="45" max="49" width="8.71428571428571" style="1"/>
-    <col min="50" max="50" width="10.1428571428571" style="1"/>
-    <col min="51" max="51" width="8.71428571428571" style="1"/>
-    <col min="52" max="52" width="12" style="1"/>
-    <col min="53" max="66" width="8.71428571428571" style="1"/>
-    <col min="67" max="67" width="13.2857142857143" style="1"/>
-    <col min="68" max="16384" width="8.71428571428571" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="21.1428571428571"/>
+    <col min="3" max="3" customWidth="true" style="1" width="21.2857142857143"/>
+    <col min="4" max="18" style="1" width="8.71428571428571"/>
+    <col min="19" max="19" style="1" width="9.28571428571429"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="28" style="1" width="8.71428571428571"/>
+    <col min="29" max="29" style="1" width="9.28571428571429"/>
+    <col min="30" max="39" style="1" width="8.71428571428571"/>
+    <col min="40" max="40" style="1" width="10.1428571428571"/>
+    <col min="41" max="43" style="1" width="8.71428571428571"/>
+    <col min="44" max="44" style="1" width="10.1428571428571"/>
+    <col min="45" max="49" style="1" width="8.71428571428571"/>
+    <col min="50" max="50" style="1" width="10.1428571428571"/>
+    <col min="51" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="12.0"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="13.2857142857143"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -7679,6 +7766,12 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
+      <c r="AU4" t="s" s="1">
+        <v>113</v>
+      </c>
+      <c r="AV4" t="s" s="1">
+        <v>149</v>
+      </c>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>2</v>
@@ -7717,11 +7810,11 @@
       <c r="BL4" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>113</v>
+      <c r="BM4" t="s" s="1">
+        <v>149</v>
+      </c>
+      <c r="BN4" t="s" s="1">
+        <v>191</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -7872,17 +7965,17 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71428571428571" style="1"/>
-    <col min="2" max="2" width="23.4285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="29.4285714285714" style="1" customWidth="1"/>
-    <col min="4" max="18" width="8.71428571428571" style="1"/>
-    <col min="19" max="19" width="9.28571428571429" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="51" width="8.71428571428571" style="1"/>
-    <col min="52" max="52" width="10.7142857142857" style="1"/>
-    <col min="53" max="66" width="8.71428571428571" style="1"/>
-    <col min="67" max="67" width="10.5714285714286" style="1"/>
-    <col min="68" max="16384" width="8.71428571428571" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="23.4285714285714"/>
+    <col min="3" max="3" customWidth="true" style="1" width="29.4285714285714"/>
+    <col min="4" max="18" style="1" width="8.71428571428571"/>
+    <col min="19" max="19" style="1" width="9.28571428571429"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="10.7142857142857"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="10.5714285714286"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -8624,25 +8717,25 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71428571428571" style="1"/>
-    <col min="2" max="2" width="27.2857142857143" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.4285714285714" style="1" customWidth="1"/>
-    <col min="4" max="18" width="8.71428571428571" style="1"/>
-    <col min="19" max="19" width="9.28571428571429" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="34" width="8.71428571428571" style="1"/>
-    <col min="35" max="35" width="11.4285714285714" style="1"/>
-    <col min="36" max="39" width="8.71428571428571" style="1"/>
-    <col min="40" max="40" width="10.1428571428571" style="1"/>
-    <col min="41" max="43" width="8.71428571428571" style="1"/>
-    <col min="44" max="44" width="10.1428571428571" style="1"/>
-    <col min="45" max="49" width="8.71428571428571" style="1"/>
-    <col min="50" max="50" width="10.1428571428571" style="1"/>
-    <col min="51" max="51" width="8.71428571428571" style="1"/>
-    <col min="52" max="52" width="12" style="1"/>
-    <col min="53" max="66" width="8.71428571428571" style="1"/>
-    <col min="67" max="67" width="12" style="1"/>
-    <col min="68" max="16384" width="8.71428571428571" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="27.2857142857143"/>
+    <col min="3" max="3" customWidth="true" style="1" width="25.4285714285714"/>
+    <col min="4" max="18" style="1" width="8.71428571428571"/>
+    <col min="19" max="19" style="1" width="9.28571428571429"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="34" style="1" width="8.71428571428571"/>
+    <col min="35" max="35" style="1" width="11.4285714285714"/>
+    <col min="36" max="39" style="1" width="8.71428571428571"/>
+    <col min="40" max="40" style="1" width="10.1428571428571"/>
+    <col min="41" max="43" style="1" width="8.71428571428571"/>
+    <col min="44" max="44" style="1" width="10.1428571428571"/>
+    <col min="45" max="49" style="1" width="8.71428571428571"/>
+    <col min="50" max="50" style="1" width="10.1428571428571"/>
+    <col min="51" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="12.0"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="12.0"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -9186,10 +9279,10 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AU4" t="s" s="1">
         <v>113</v>
       </c>
-      <c r="AV4" s="1" t="s">
+      <c r="AV4" t="s" s="1">
         <v>149</v>
       </c>
       <c r="AW4" s="28">
@@ -9230,11 +9323,11 @@
       <c r="BL4" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" s="1" t="s">
+      <c r="BM4" t="s" s="1">
         <v>149</v>
       </c>
-      <c r="BN4" s="1" t="s">
-        <v>179</v>
+      <c r="BN4" t="s" s="1">
+        <v>192</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -9384,25 +9477,25 @@
   <dimension ref="A1:BQ18"/>
   <sheetFormatPr defaultColWidth="8.85714285714286" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.85714285714286" style="23"/>
-    <col min="2" max="2" width="28" style="23" customWidth="1"/>
-    <col min="3" max="3" width="23" style="23" customWidth="1"/>
-    <col min="4" max="11" width="8.85714285714286" style="23"/>
-    <col min="12" max="12" width="15.7142857142857" style="23" customWidth="1"/>
-    <col min="13" max="13" width="9.14285714285714" style="23" customWidth="1"/>
-    <col min="14" max="14" width="13.8571428571429" style="23" customWidth="1"/>
-    <col min="15" max="15" width="11.2857142857143" style="23" customWidth="1"/>
-    <col min="16" max="16" width="17.8571428571429" style="23" customWidth="1"/>
-    <col min="17" max="18" width="8.85714285714286" style="23"/>
-    <col min="19" max="19" width="9.28571428571429" style="23"/>
-    <col min="20" max="20" width="10.1428571428571" style="23" customWidth="1"/>
-    <col min="21" max="51" width="8.85714285714286" style="23"/>
-    <col min="52" max="52" width="10.7142857142857" style="23"/>
-    <col min="53" max="63" width="8.85714285714286" style="23"/>
-    <col min="64" max="64" width="11" style="23" customWidth="1"/>
-    <col min="65" max="66" width="8.85714285714286" style="23"/>
-    <col min="67" max="67" width="10.7142857142857" style="23"/>
-    <col min="68" max="16384" width="8.85714285714286" style="23"/>
+    <col min="1" max="1" style="23" width="8.85714285714286"/>
+    <col min="2" max="2" customWidth="true" style="23" width="28.0"/>
+    <col min="3" max="3" customWidth="true" style="23" width="23.0"/>
+    <col min="4" max="11" style="23" width="8.85714285714286"/>
+    <col min="12" max="12" customWidth="true" style="23" width="15.7142857142857"/>
+    <col min="13" max="13" customWidth="true" style="23" width="9.14285714285714"/>
+    <col min="14" max="14" customWidth="true" style="23" width="13.8571428571429"/>
+    <col min="15" max="15" customWidth="true" style="23" width="11.2857142857143"/>
+    <col min="16" max="16" customWidth="true" style="23" width="17.8571428571429"/>
+    <col min="17" max="18" style="23" width="8.85714285714286"/>
+    <col min="19" max="19" style="23" width="9.28571428571429"/>
+    <col min="20" max="20" customWidth="true" style="23" width="10.1428571428571"/>
+    <col min="21" max="51" style="23" width="8.85714285714286"/>
+    <col min="52" max="52" style="23" width="10.7142857142857"/>
+    <col min="53" max="63" style="23" width="8.85714285714286"/>
+    <col min="64" max="64" customWidth="true" style="23" width="11.0"/>
+    <col min="65" max="66" style="23" width="8.85714285714286"/>
+    <col min="67" max="67" style="23" width="10.7142857142857"/>
+    <col min="68" max="16384" style="23" width="8.85714285714286"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -11172,12 +11265,12 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="9.85714285714286" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="9.85714285714286" style="1"/>
-    <col min="2" max="2" width="25.5714285714286" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="19" width="9.85714285714286" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.85714285714286" style="1"/>
+    <col min="1" max="1" style="1" width="9.85714285714286"/>
+    <col min="2" max="2" customWidth="true" style="1" width="25.5714285714286"/>
+    <col min="3" max="3" customWidth="true" style="1" width="26.0"/>
+    <col min="4" max="19" style="1" width="9.85714285714286"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="16384" style="1" width="9.85714285714286"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -11721,10 +11814,10 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AU4" t="s" s="1">
         <v>113</v>
       </c>
-      <c r="AV4" s="1" t="s">
+      <c r="AV4" t="s" s="1">
         <v>181</v>
       </c>
       <c r="AW4" s="28">
@@ -11765,11 +11858,11 @@
       <c r="BL4" s="28" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" s="1" t="s">
+      <c r="BM4" t="s" s="1">
         <v>181</v>
       </c>
-      <c r="BN4" s="1" t="s">
-        <v>147</v>
+      <c r="BN4" t="s" s="1">
+        <v>193</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -11916,15 +12009,15 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71428571428571" style="1"/>
-    <col min="2" max="3" width="26.5428571428571" style="1" customWidth="1"/>
-    <col min="4" max="18" width="8.71428571428571" style="1"/>
-    <col min="19" max="19" width="9.28571428571429" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="66" width="8.71428571428571" style="1"/>
-    <col min="67" max="67" width="13.2857142857143" style="1"/>
-    <col min="68" max="68" width="12.8571428571429" style="1"/>
-    <col min="69" max="16384" width="8.71428571428571" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="3" customWidth="true" style="1" width="26.5428571428571"/>
+    <col min="4" max="18" style="1" width="8.71428571428571"/>
+    <col min="19" max="19" style="1" width="9.28571428571429"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="13.2857142857143"/>
+    <col min="68" max="68" style="1" width="12.8571428571429"/>
+    <col min="69" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -12468,6 +12561,12 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
+      <c r="AU4" t="s" s="1">
+        <v>113</v>
+      </c>
+      <c r="AV4" t="s" s="1">
+        <v>181</v>
+      </c>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>1</v>
@@ -12506,11 +12605,11 @@
       <c r="BL4" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>113</v>
+      <c r="BM4" t="s" s="1">
+        <v>181</v>
+      </c>
+      <c r="BN4" t="s" s="1">
+        <v>194</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -12660,17 +12759,17 @@
   <dimension ref="A1:BQ5"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="8.71428571428571" style="1"/>
-    <col min="2" max="2" width="27.2857142857143" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.4285714285714" style="1" customWidth="1"/>
-    <col min="4" max="18" width="8.71428571428571" style="1"/>
-    <col min="19" max="19" width="9.28571428571429" style="1"/>
-    <col min="20" max="20" width="10.1428571428571" style="1" customWidth="1"/>
-    <col min="21" max="51" width="8.71428571428571" style="1"/>
-    <col min="52" max="52" width="9" style="1"/>
-    <col min="53" max="66" width="8.71428571428571" style="1"/>
-    <col min="67" max="67" width="13.2857142857143" style="1"/>
-    <col min="68" max="16384" width="8.71428571428571" style="1"/>
+    <col min="1" max="1" style="1" width="8.71428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="27.2857142857143"/>
+    <col min="3" max="3" customWidth="true" style="1" width="25.4285714285714"/>
+    <col min="4" max="18" style="1" width="8.71428571428571"/>
+    <col min="19" max="19" style="1" width="9.28571428571429"/>
+    <col min="20" max="20" customWidth="true" style="1" width="10.1428571428571"/>
+    <col min="21" max="51" style="1" width="8.71428571428571"/>
+    <col min="52" max="52" style="1" width="9.0"/>
+    <col min="53" max="66" style="1" width="8.71428571428571"/>
+    <col min="67" max="67" style="1" width="13.2857142857143"/>
+    <col min="68" max="16384" style="1" width="8.71428571428571"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69">
@@ -13214,6 +13313,12 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
+      <c r="AU4" t="s" s="1">
+        <v>113</v>
+      </c>
+      <c r="AV4" t="s" s="1">
+        <v>181</v>
+      </c>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>1</v>
@@ -13252,11 +13357,11 @@
       <c r="BL4" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BN4" s="1" t="s">
-        <v>113</v>
+      <c r="BM4" t="s" s="1">
+        <v>181</v>
+      </c>
+      <c r="BN4" t="s" s="1">
+        <v>195</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -13406,71 +13511,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="9" width="5.85714285714286" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5.85714285714286" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.4285714285714" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="11.8571428571429" customWidth="1"/>
-    <col min="20" max="20" width="10.7142857142857" customWidth="1"/>
-    <col min="21" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="23.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="18" customWidth="1"/>
-    <col min="48" max="48" width="24.4285714285714" customWidth="1"/>
-    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="9.42857142857143" customWidth="1"/>
-    <col min="65" max="65" width="49.1428571428571" customWidth="1"/>
-    <col min="66" max="66" width="43.8571428571429" customWidth="1"/>
-    <col min="67" max="67" width="22.7142857142857" customWidth="1"/>
-    <col min="68" max="68" width="40.8571428571429" customWidth="1"/>
-    <col min="69" max="69" width="7.57142857142857" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="22.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="9" customWidth="true" width="5.85714285714286"/>
+    <col min="10" max="10" customWidth="true" width="6.0"/>
+    <col min="11" max="11" customWidth="true" width="5.85714285714286"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.4285714285714"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="11.8571428571429"/>
+    <col min="20" max="20" customWidth="true" width="10.7142857142857"/>
+    <col min="21" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="23.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="18.0"/>
+    <col min="48" max="48" customWidth="true" width="24.4285714285714"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="9.42857142857143"/>
+    <col min="65" max="65" customWidth="true" width="49.1428571428571"/>
+    <col min="66" max="66" customWidth="true" width="43.8571428571429"/>
+    <col min="67" max="67" customWidth="true" width="22.7142857142857"/>
+    <col min="68" max="68" customWidth="true" width="40.8571428571429"/>
+    <col min="69" max="69" customWidth="true" width="7.57142857142857"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -15849,71 +15954,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="25.2857142857143" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
-    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
-    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="25.2857142857143"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -18086,10 +18191,10 @@
       <c r="AT23" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>134</v>
       </c>
       <c r="AW23" s="104">
@@ -18130,11 +18235,11 @@
       <c r="BL23" s="121" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>134</v>
       </c>
-      <c r="BN23" t="s">
-        <v>135</v>
+      <c r="BN23" t="s" s="0">
+        <v>208</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -18289,71 +18394,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="25.5714285714286" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
-    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
-    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="25.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -20715,71 +20820,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="24.7142857142857" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
-    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
-    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="24.7142857142857"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -22807,14 +22912,14 @@
       <c r="F23" s="103">
         <v>2</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>250</v>
       </c>
       <c r="H23" s="104">
         <f>F23*G23</f>
         <v>500</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>138</v>
       </c>
       <c r="J23" s="104">
@@ -22952,10 +23057,10 @@
       <c r="AT23" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>134</v>
       </c>
       <c r="AW23" s="104">
@@ -22996,11 +23101,11 @@
       <c r="BL23" s="104" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>134</v>
       </c>
-      <c r="BN23" t="s">
-        <v>139</v>
+      <c r="BN23" t="s" s="0">
+        <v>209</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -23155,71 +23260,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="25.1428571428571" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
-    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
-    <col min="49" max="49" width="13.4285714285714" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="25.1428571428571"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="13.4285714285714"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -25247,14 +25352,14 @@
       <c r="F23" s="103">
         <v>2</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>250</v>
       </c>
       <c r="H23" s="104">
         <f>F23*G23</f>
         <v>500</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>138</v>
       </c>
       <c r="J23" s="104">
@@ -25587,71 +25692,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="24.5714285714286" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
-    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
-    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="24.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -27824,10 +27929,10 @@
       <c r="AT23" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>143</v>
       </c>
       <c r="AW23" s="104">
@@ -27868,11 +27973,11 @@
       <c r="BL23" s="104" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>143</v>
       </c>
-      <c r="BN23" t="s">
-        <v>144</v>
+      <c r="BN23" t="s" s="0">
+        <v>210</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -28027,71 +28132,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
-    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
-    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="28.0"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -30264,10 +30369,10 @@
       <c r="AT23" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>143</v>
       </c>
       <c r="AW23" s="104">
@@ -30308,11 +30413,11 @@
       <c r="BL23" s="104" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>143</v>
       </c>
-      <c r="BN23" t="s">
-        <v>144</v>
+      <c r="BN23" t="s" s="0">
+        <v>187</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -30467,71 +30572,71 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.71428571428571" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.57142857142857" customWidth="1"/>
-    <col min="2" max="3" width="27.5714285714286" customWidth="1"/>
-    <col min="4" max="4" width="79.4285714285714" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="24.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="12.7142857142857" customWidth="1"/>
-    <col min="9" max="10" width="5.85714285714286" customWidth="1"/>
-    <col min="11" max="11" width="6" customWidth="1"/>
-    <col min="12" max="12" width="14.2857142857143" customWidth="1"/>
-    <col min="13" max="13" width="9.42857142857143" customWidth="1"/>
-    <col min="14" max="14" width="14.2857142857143" customWidth="1"/>
-    <col min="15" max="15" width="15.5714285714286" customWidth="1"/>
-    <col min="16" max="16" width="14.4285714285714" customWidth="1"/>
-    <col min="17" max="17" width="39.4285714285714" customWidth="1"/>
-    <col min="18" max="18" width="11.7142857142857" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="6.42857142857143" customWidth="1"/>
-    <col min="21" max="21" width="9.85714285714286" customWidth="1"/>
-    <col min="22" max="22" width="6.57142857142857" customWidth="1"/>
-    <col min="23" max="23" width="37.1428571428571" customWidth="1"/>
-    <col min="24" max="24" width="6.14285714285714" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.71428571428571" customWidth="1"/>
-    <col min="27" max="27" width="6.28571428571429" customWidth="1"/>
-    <col min="28" max="28" width="9.28571428571429" customWidth="1"/>
-    <col min="29" max="29" width="9.71428571428571" customWidth="1"/>
-    <col min="30" max="30" width="12.8571428571429" customWidth="1"/>
-    <col min="31" max="31" width="16.1428571428571" customWidth="1"/>
-    <col min="32" max="32" width="15.4285714285714" customWidth="1"/>
-    <col min="33" max="33" width="24.5714285714286" customWidth="1"/>
-    <col min="34" max="34" width="8.57142857142857" customWidth="1"/>
-    <col min="35" max="35" width="14.7142857142857" customWidth="1"/>
-    <col min="36" max="36" width="18.5714285714286" customWidth="1"/>
-    <col min="37" max="37" width="14.1428571428571" customWidth="1"/>
-    <col min="38" max="38" width="14.7142857142857" customWidth="1"/>
-    <col min="39" max="39" width="17.4285714285714" customWidth="1"/>
-    <col min="40" max="40" width="22" customWidth="1"/>
-    <col min="41" max="41" width="17.5714285714286" customWidth="1"/>
-    <col min="42" max="42" width="25.2857142857143" customWidth="1"/>
-    <col min="43" max="43" width="13" customWidth="1"/>
-    <col min="44" max="44" width="25.7142857142857" customWidth="1"/>
-    <col min="45" max="45" width="9.28571428571429" customWidth="1"/>
-    <col min="46" max="46" width="13" customWidth="1"/>
-    <col min="47" max="47" width="12.4285714285714" customWidth="1"/>
-    <col min="48" max="48" width="18.8571428571429" customWidth="1"/>
-    <col min="49" max="49" width="14.5714285714286" customWidth="1"/>
-    <col min="50" max="50" width="19.4285714285714" customWidth="1"/>
-    <col min="51" max="51" width="16.2857142857143" customWidth="1"/>
-    <col min="52" max="52" width="22.7142857142857" customWidth="1"/>
-    <col min="53" max="53" width="21.7142857142857" customWidth="1"/>
-    <col min="54" max="54" width="23.2857142857143" customWidth="1"/>
-    <col min="55" max="55" width="18.2857142857143" customWidth="1"/>
-    <col min="56" max="56" width="16" customWidth="1"/>
-    <col min="57" max="58" width="19.1428571428571" customWidth="1"/>
-    <col min="59" max="59" width="15.5714285714286" customWidth="1"/>
-    <col min="60" max="61" width="14.7142857142857" customWidth="1"/>
-    <col min="62" max="62" width="25.4285714285714" customWidth="1"/>
-    <col min="63" max="63" width="35.4285714285714" customWidth="1"/>
-    <col min="64" max="64" width="8.57142857142857" customWidth="1"/>
-    <col min="65" max="65" width="42.5714285714286" customWidth="1"/>
-    <col min="66" max="66" width="38.1428571428571" customWidth="1"/>
-    <col min="67" max="67" width="19.4285714285714" customWidth="1"/>
-    <col min="68" max="68" width="35.4285714285714" customWidth="1"/>
-    <col min="69" max="69" width="5.28571428571429" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="7.57142857142857"/>
+    <col min="2" max="3" customWidth="true" width="27.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="79.4285714285714"/>
+    <col min="5" max="5" customWidth="true" width="11.5714285714286"/>
+    <col min="6" max="6" customWidth="true" width="24.1428571428571"/>
+    <col min="7" max="7" customWidth="true" width="11.0"/>
+    <col min="8" max="8" customWidth="true" width="12.7142857142857"/>
+    <col min="9" max="10" customWidth="true" width="5.85714285714286"/>
+    <col min="11" max="11" customWidth="true" width="6.0"/>
+    <col min="12" max="12" customWidth="true" width="14.2857142857143"/>
+    <col min="13" max="13" customWidth="true" width="9.42857142857143"/>
+    <col min="14" max="14" customWidth="true" width="14.2857142857143"/>
+    <col min="15" max="15" customWidth="true" width="15.5714285714286"/>
+    <col min="16" max="16" customWidth="true" width="14.4285714285714"/>
+    <col min="17" max="17" customWidth="true" width="39.4285714285714"/>
+    <col min="18" max="18" customWidth="true" width="11.7142857142857"/>
+    <col min="19" max="19" customWidth="true" width="10.0"/>
+    <col min="20" max="20" customWidth="true" width="6.42857142857143"/>
+    <col min="21" max="21" customWidth="true" width="9.85714285714286"/>
+    <col min="22" max="22" customWidth="true" width="6.57142857142857"/>
+    <col min="23" max="23" customWidth="true" width="37.1428571428571"/>
+    <col min="24" max="24" customWidth="true" width="6.14285714285714"/>
+    <col min="25" max="25" customWidth="true" width="8.0"/>
+    <col min="26" max="26" customWidth="true" width="7.71428571428571"/>
+    <col min="27" max="27" customWidth="true" width="6.28571428571429"/>
+    <col min="28" max="28" customWidth="true" width="9.28571428571429"/>
+    <col min="29" max="29" customWidth="true" width="9.71428571428571"/>
+    <col min="30" max="30" customWidth="true" width="12.8571428571429"/>
+    <col min="31" max="31" customWidth="true" width="16.1428571428571"/>
+    <col min="32" max="32" customWidth="true" width="15.4285714285714"/>
+    <col min="33" max="33" customWidth="true" width="24.5714285714286"/>
+    <col min="34" max="34" customWidth="true" width="8.57142857142857"/>
+    <col min="35" max="35" customWidth="true" width="14.7142857142857"/>
+    <col min="36" max="36" customWidth="true" width="18.5714285714286"/>
+    <col min="37" max="37" customWidth="true" width="14.1428571428571"/>
+    <col min="38" max="38" customWidth="true" width="14.7142857142857"/>
+    <col min="39" max="39" customWidth="true" width="17.4285714285714"/>
+    <col min="40" max="40" customWidth="true" width="22.0"/>
+    <col min="41" max="41" customWidth="true" width="17.5714285714286"/>
+    <col min="42" max="42" customWidth="true" width="25.2857142857143"/>
+    <col min="43" max="43" customWidth="true" width="13.0"/>
+    <col min="44" max="44" customWidth="true" width="25.7142857142857"/>
+    <col min="45" max="45" customWidth="true" width="9.28571428571429"/>
+    <col min="46" max="46" customWidth="true" width="13.0"/>
+    <col min="47" max="47" customWidth="true" width="12.4285714285714"/>
+    <col min="48" max="48" customWidth="true" width="18.8571428571429"/>
+    <col min="49" max="49" customWidth="true" width="14.5714285714286"/>
+    <col min="50" max="50" customWidth="true" width="19.4285714285714"/>
+    <col min="51" max="51" customWidth="true" width="16.2857142857143"/>
+    <col min="52" max="52" customWidth="true" width="22.7142857142857"/>
+    <col min="53" max="53" customWidth="true" width="21.7142857142857"/>
+    <col min="54" max="54" customWidth="true" width="23.2857142857143"/>
+    <col min="55" max="55" customWidth="true" width="18.2857142857143"/>
+    <col min="56" max="56" customWidth="true" width="16.0"/>
+    <col min="57" max="58" customWidth="true" width="19.1428571428571"/>
+    <col min="59" max="59" customWidth="true" width="15.5714285714286"/>
+    <col min="60" max="61" customWidth="true" width="14.7142857142857"/>
+    <col min="62" max="62" customWidth="true" width="25.4285714285714"/>
+    <col min="63" max="63" customWidth="true" width="35.4285714285714"/>
+    <col min="64" max="64" customWidth="true" width="8.57142857142857"/>
+    <col min="65" max="65" customWidth="true" width="42.5714285714286"/>
+    <col min="66" max="66" customWidth="true" width="38.1428571428571"/>
+    <col min="67" max="67" customWidth="true" width="19.4285714285714"/>
+    <col min="68" max="68" customWidth="true" width="35.4285714285714"/>
+    <col min="69" max="69" customWidth="true" width="5.28571428571429"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:69">
@@ -32559,14 +32664,14 @@
       <c r="F23" s="103">
         <v>3</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>250</v>
       </c>
       <c r="H23" s="104">
         <f>F23*G23</f>
         <v>750</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>138</v>
       </c>
       <c r="J23" s="104">
@@ -32704,10 +32809,10 @@
       <c r="AT23" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>113</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>143</v>
       </c>
       <c r="AW23" s="104">
@@ -32748,11 +32853,11 @@
       <c r="BL23" s="104" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>143</v>
       </c>
-      <c r="BN23" t="s">
-        <v>147</v>
+      <c r="BN23" t="s" s="0">
+        <v>188</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
Fixed Failed Test scenarios in the purchase module
Fixed Failed Test scenarios in the purchase module
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2788" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3004" uniqueCount="239">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -677,6 +677,90 @@
   </si>
   <si>
     <t>134</t>
+  </si>
+  <si>
+    <t>292</t>
+  </si>
+  <si>
+    <t>7944.85684</t>
+  </si>
+  <si>
+    <t>294</t>
+  </si>
+  <si>
+    <t>7944.66666</t>
+  </si>
+  <si>
+    <t>262</t>
+  </si>
+  <si>
+    <t>135</t>
+  </si>
+  <si>
+    <t>136</t>
+  </si>
+  <si>
+    <t>128</t>
+  </si>
+  <si>
+    <t>129</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>126</t>
+  </si>
+  <si>
+    <t>296</t>
+  </si>
+  <si>
+    <t>7944.47905</t>
+  </si>
+  <si>
+    <t>298</t>
+  </si>
+  <si>
+    <t>7944.29396</t>
+  </si>
+  <si>
+    <t>264</t>
+  </si>
+  <si>
+    <t>266</t>
+  </si>
+  <si>
+    <t>137</t>
+  </si>
+  <si>
+    <t>138</t>
+  </si>
+  <si>
+    <t>130</t>
+  </si>
+  <si>
+    <t>131</t>
+  </si>
+  <si>
+    <t>18387.625</t>
+  </si>
+  <si>
+    <t>325</t>
+  </si>
+  <si>
+    <t>16915.82121</t>
+  </si>
+  <si>
+    <t>327</t>
+  </si>
+  <si>
+    <t>16924.82307</t>
+  </si>
+  <si>
+    <t>202</t>
+  </si>
+  <si>
+    <t>18386.78342</t>
   </si>
 </sst>
 </file>
@@ -4582,10 +4666,10 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>207</v>
+        <v>225</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="BO23" s="121">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -5305,7 +5389,7 @@
         <v>113</v>
       </c>
       <c r="AV4" t="s" s="1">
-        <v>149</v>
+        <v>232</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -5346,10 +5430,10 @@
         <v>150</v>
       </c>
       <c r="BM4" t="s" s="1">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="BN4" t="s" s="1">
-        <v>189</v>
+        <v>235</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -7770,7 +7854,7 @@
         <v>113</v>
       </c>
       <c r="AV4" t="s" s="1">
-        <v>149</v>
+        <v>232</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -7811,10 +7895,10 @@
         <v>150</v>
       </c>
       <c r="BM4" t="s" s="1">
-        <v>149</v>
+        <v>238</v>
       </c>
       <c r="BN4" t="s" s="1">
-        <v>191</v>
+        <v>237</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -11814,12 +11898,8 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
-        <v>113</v>
-      </c>
-      <c r="AV4" t="s" s="1">
-        <v>181</v>
-      </c>
+      <c r="AU4" s="1"/>
+      <c r="AV4" s="1"/>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>1</v>
@@ -11858,12 +11938,8 @@
       <c r="BL4" s="28" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" t="s" s="1">
-        <v>181</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>193</v>
-      </c>
+      <c r="BM4" s="1"/>
+      <c r="BN4" s="1"/>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
         <v>55159.9</v>
@@ -12561,12 +12637,8 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
-        <v>113</v>
-      </c>
-      <c r="AV4" t="s" s="1">
-        <v>181</v>
-      </c>
+      <c r="AU4" s="1"/>
+      <c r="AV4" s="1"/>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>1</v>
@@ -12605,12 +12677,8 @@
       <c r="BL4" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" t="s" s="1">
-        <v>181</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>194</v>
-      </c>
+      <c r="BM4" s="1"/>
+      <c r="BN4" s="1"/>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
         <v>55159.9</v>
@@ -13313,12 +13381,8 @@
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
-        <v>113</v>
-      </c>
-      <c r="AV4" t="s" s="1">
-        <v>181</v>
-      </c>
+      <c r="AU4" s="1"/>
+      <c r="AV4" s="1"/>
       <c r="AW4" s="28">
         <f>AM4</f>
         <v>1</v>
@@ -13357,12 +13421,8 @@
       <c r="BL4" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="BM4" t="s" s="1">
-        <v>181</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>195</v>
-      </c>
+      <c r="BM4" s="1"/>
+      <c r="BN4" s="1"/>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
         <v>55159.9</v>
@@ -18239,7 +18299,7 @@
         <v>134</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -23105,7 +23165,7 @@
         <v>134</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -27977,7 +28037,7 @@
         <v>143</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>210</v>
+        <v>229</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -30417,7 +30477,7 @@
         <v>143</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>187</v>
+        <v>231</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -32857,7 +32917,7 @@
         <v>143</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>188</v>
+        <v>218</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
Fixed failed HRM, GRN and Purchase Order test steps
Fixed failed HRM, GRN and Purchase Order test steps
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" firstSheet="12" activeTab="13"/>
+    <workbookView windowWidth="20490" windowHeight="7020" firstSheet="16" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="ImportDirectGRNUDGeneralSameUOM" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3344" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="207">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -406,10 +406,10 @@
     <t>RM KD</t>
   </si>
   <si>
-    <t>8033.52</t>
+    <t>8052.25314</t>
   </si>
   <si>
-    <t>70</t>
+    <t>542</t>
   </si>
   <si>
     <t>VD Asbl. Val.</t>
@@ -451,7 +451,10 @@
     <t>19792.25</t>
   </si>
   <si>
-    <t>62</t>
+    <t>20069.15269</t>
+  </si>
+  <si>
+    <t>518</t>
   </si>
   <si>
     <t>ITEM-GWL-SERVICE-RC-02</t>
@@ -463,7 +466,10 @@
     <t>1</t>
   </si>
   <si>
-    <t>44</t>
+    <t>20047.13933</t>
+  </si>
+  <si>
+    <t>486</t>
   </si>
   <si>
     <t>ITEM-GWL-SERVICE-PL-02</t>
@@ -478,31 +484,43 @@
     <t>59375.9</t>
   </si>
   <si>
-    <t>25</t>
+    <t>60109.36701</t>
+  </si>
+  <si>
+    <t>240</t>
   </si>
   <si>
     <t>ITEM-GWL-DISSIMILAR-RC-04</t>
   </si>
   <si>
+    <t>60311.33617</t>
+  </si>
+  <si>
+    <t>230</t>
+  </si>
+  <si>
     <t>ITEM-GWL-DISSIMILAR-PL-04</t>
   </si>
   <si>
-    <t>20</t>
+    <t>60261.1188</t>
+  </si>
+  <si>
+    <t>232</t>
   </si>
   <si>
     <t>INS WH-1</t>
   </si>
   <si>
-    <t>18386.775</t>
+    <t>18387.625</t>
   </si>
   <si>
     <t>RM WH-49</t>
   </si>
   <si>
-    <t>14156.1407</t>
+    <t>17536.37859</t>
   </si>
   <si>
-    <t>113</t>
+    <t>505</t>
   </si>
   <si>
     <t>No.</t>
@@ -577,289 +595,76 @@
     <t>250</t>
   </si>
   <si>
+    <t>18386.8077</t>
+  </si>
+  <si>
+    <t>208</t>
+  </si>
+  <si>
     <t>15</t>
   </si>
   <si>
     <t>41.515</t>
   </si>
   <si>
-    <t>16</t>
+    <t>18386.79839</t>
+  </si>
+  <si>
+    <t>218</t>
   </si>
   <si>
     <t>10</t>
   </si>
   <si>
-    <t>55159.9</t>
+    <t>55162.875</t>
   </si>
   <si>
-    <t>282</t>
+    <t>55159.94917</t>
   </si>
   <si>
-    <t>7945.84822</t>
+    <t>121</t>
   </si>
   <si>
-    <t>276</t>
+    <t>55159.98837</t>
   </si>
   <si>
-    <t>254</t>
+    <t>101</t>
   </si>
   <si>
-    <t>132</t>
-  </si>
-  <si>
-    <t>127</t>
-  </si>
-  <si>
-    <t>124</t>
-  </si>
-  <si>
-    <t>323</t>
-  </si>
-  <si>
-    <t>16906.70787</t>
-  </si>
-  <si>
-    <t>200</t>
-  </si>
-  <si>
-    <t>212</t>
-  </si>
-  <si>
-    <t>119</t>
+    <t>55159.96071</t>
   </si>
   <si>
     <t>98</t>
   </si>
   <si>
-    <t>96</t>
+    <t>507</t>
   </si>
   <si>
-    <t>284</t>
+    <t>17539.73656</t>
   </si>
   <si>
-    <t>7945.64436</t>
+    <t>544</t>
   </si>
   <si>
-    <t>256</t>
+    <t>8051.75552</t>
   </si>
   <si>
-    <t>133</t>
+    <t>520</t>
   </si>
   <si>
-    <t>286</t>
+    <t>20068.08768</t>
   </si>
   <si>
-    <t>7945.44335</t>
+    <t>488</t>
   </si>
   <si>
-    <t>288</t>
+    <t>20046.0947</t>
   </si>
   <si>
-    <t>7945.24513</t>
+    <t>241</t>
   </si>
   <si>
-    <t>278</t>
-  </si>
-  <si>
-    <t>258</t>
-  </si>
-  <si>
-    <t>290</t>
-  </si>
-  <si>
-    <t>7945.04965</t>
-  </si>
-  <si>
-    <t>280</t>
-  </si>
-  <si>
-    <t>260</t>
-  </si>
-  <si>
-    <t>134</t>
-  </si>
-  <si>
-    <t>292</t>
-  </si>
-  <si>
-    <t>7944.85684</t>
-  </si>
-  <si>
-    <t>294</t>
-  </si>
-  <si>
-    <t>7944.66666</t>
-  </si>
-  <si>
-    <t>262</t>
-  </si>
-  <si>
-    <t>135</t>
-  </si>
-  <si>
-    <t>136</t>
-  </si>
-  <si>
-    <t>128</t>
-  </si>
-  <si>
-    <t>129</t>
-  </si>
-  <si>
-    <t>125</t>
-  </si>
-  <si>
-    <t>126</t>
-  </si>
-  <si>
-    <t>296</t>
-  </si>
-  <si>
-    <t>7944.47905</t>
-  </si>
-  <si>
-    <t>298</t>
-  </si>
-  <si>
-    <t>7944.29396</t>
-  </si>
-  <si>
-    <t>264</t>
-  </si>
-  <si>
-    <t>266</t>
-  </si>
-  <si>
-    <t>137</t>
-  </si>
-  <si>
-    <t>138</t>
-  </si>
-  <si>
-    <t>130</t>
-  </si>
-  <si>
-    <t>131</t>
-  </si>
-  <si>
-    <t>18387.625</t>
-  </si>
-  <si>
-    <t>325</t>
-  </si>
-  <si>
-    <t>16915.82121</t>
-  </si>
-  <si>
-    <t>327</t>
-  </si>
-  <si>
-    <t>16924.82307</t>
-  </si>
-  <si>
-    <t>202</t>
-  </si>
-  <si>
-    <t>18386.78342</t>
-  </si>
-  <si>
-    <t>300</t>
-  </si>
-  <si>
-    <t>7944.11133</t>
-  </si>
-  <si>
-    <t>302</t>
-  </si>
-  <si>
-    <t>7943.93112</t>
-  </si>
-  <si>
-    <t>268</t>
-  </si>
-  <si>
-    <t>270</t>
-  </si>
-  <si>
-    <t>141</t>
-  </si>
-  <si>
-    <t>142</t>
-  </si>
-  <si>
-    <t>329</t>
-  </si>
-  <si>
-    <t>16933.71548</t>
-  </si>
-  <si>
-    <t>208</t>
-  </si>
-  <si>
-    <t>18386.8077</t>
-  </si>
-  <si>
-    <t>214</t>
-  </si>
-  <si>
-    <t>18386.78294</t>
-  </si>
-  <si>
-    <t>216</t>
-  </si>
-  <si>
-    <t>18386.79074</t>
-  </si>
-  <si>
-    <t>55162.875</t>
-  </si>
-  <si>
-    <t>121</t>
-  </si>
-  <si>
-    <t>55159.94917</t>
-  </si>
-  <si>
-    <t>101</t>
-  </si>
-  <si>
-    <t>55159.98837</t>
-  </si>
-  <si>
-    <t>55159.96071</t>
-  </si>
-  <si>
-    <t>304</t>
-  </si>
-  <si>
-    <t>7943.75328</t>
-  </si>
-  <si>
-    <t>306</t>
-  </si>
-  <si>
-    <t>7943.57777</t>
-  </si>
-  <si>
-    <t>272</t>
-  </si>
-  <si>
-    <t>218</t>
-  </si>
-  <si>
-    <t>18386.79839</t>
-  </si>
-  <si>
-    <t>308</t>
-  </si>
-  <si>
-    <t>7943.40454</t>
-  </si>
-  <si>
-    <t>274</t>
-  </si>
-  <si>
-    <t>143</t>
+    <t>60106.32358</t>
   </si>
 </sst>
 </file>
@@ -4627,7 +4432,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -4765,14 +4570,14 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>269</v>
+        <v>200</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>268</v>
+        <v>199</v>
       </c>
       <c r="BO23" s="121">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>5978.94273</v>
+        <v>8051.75552</v>
       </c>
       <c r="BP23" s="141">
         <f>BN23+AW23</f>
@@ -5320,7 +5125,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
@@ -5391,7 +5196,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -5479,7 +5284,7 @@
         <v>18386.775</v>
       </c>
       <c r="AS4" s="6" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
@@ -5488,7 +5293,7 @@
         <v>113</v>
       </c>
       <c r="AV4" t="s" s="1">
-        <v>232</v>
+        <v>155</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -5526,17 +5331,17 @@
       <c r="BJ4" s="6"/>
       <c r="BK4" s="6"/>
       <c r="BL4" s="28" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="BM4" t="s" s="1">
-        <v>248</v>
+        <v>198</v>
       </c>
       <c r="BN4" t="s" s="1">
-        <v>247</v>
+        <v>197</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>13833.80666</v>
+        <v>17539.73321</v>
       </c>
       <c r="BP4" s="34">
         <f>BN4+AW4</f>
@@ -5861,13 +5666,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -6068,7 +5873,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
@@ -6139,7 +5944,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -6227,16 +6032,16 @@
         <v>18386.775</v>
       </c>
       <c r="AS4" s="27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="AV4" s="23" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -6274,13 +6079,13 @@
       <c r="BJ4" s="28"/>
       <c r="BK4" s="28"/>
       <c r="BL4" s="33" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="BM4" s="23" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="BN4" s="23" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -6491,7 +6296,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="54" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="H7" s="55"/>
       <c r="I7" s="56">
@@ -6502,7 +6307,7 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="57" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="N7" s="58"/>
       <c r="O7" s="58"/>
@@ -6551,10 +6356,10 @@
       <c r="BF7" s="5"/>
       <c r="BG7" s="5"/>
       <c r="BH7" s="5" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="BI7" s="147" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="BJ7" s="5"/>
       <c r="BK7" s="5"/>
@@ -6573,7 +6378,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="54" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="H8" s="55"/>
       <c r="I8" s="56">
@@ -6593,7 +6398,7 @@
         <v>2</v>
       </c>
       <c r="P8" s="60" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
@@ -6639,10 +6444,10 @@
       <c r="BF8" s="5"/>
       <c r="BG8" s="5"/>
       <c r="BH8" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="BI8" s="147" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="BJ8" s="5"/>
       <c r="BK8" s="5"/>
@@ -6661,7 +6466,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="54" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="H9" s="55"/>
       <c r="I9" s="56">
@@ -6681,7 +6486,7 @@
         <v>2.5</v>
       </c>
       <c r="P9" s="20" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
@@ -6745,7 +6550,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="54" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="H10" s="55"/>
       <c r="I10" s="56">
@@ -6759,13 +6564,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="O10" s="20">
         <v>0.001</v>
       </c>
       <c r="P10" s="20" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="Q10" s="5"/>
       <c r="R10" s="5"/>
@@ -6829,7 +6634,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="54" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="H11" s="55"/>
       <c r="I11" s="61">
@@ -6963,10 +6768,10 @@
       <c r="BK12" s="5"/>
       <c r="BL12" s="5"/>
       <c r="BM12" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="BN12" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="BO12" s="5"/>
       <c r="BP12" s="6"/>
@@ -7036,7 +6841,7 @@
       <c r="BI13" s="5"/>
       <c r="BJ13" s="5"/>
       <c r="BK13" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="BL13" s="5">
         <v>12.5</v>
@@ -7117,7 +6922,7 @@
       <c r="BI14" s="5"/>
       <c r="BJ14" s="5"/>
       <c r="BK14" s="5" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="BL14" s="5">
         <v>487.4072</v>
@@ -7195,7 +7000,7 @@
       <c r="BI15" s="5"/>
       <c r="BJ15" s="5"/>
       <c r="BK15" s="5" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="BL15" s="5">
         <v>37.5</v>
@@ -7270,7 +7075,7 @@
       <c r="BI16" s="5"/>
       <c r="BJ16" s="5"/>
       <c r="BK16" s="5" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="BL16" s="5">
         <v>487.4072</v>
@@ -7578,13 +7383,13 @@
     </row>
     <row r="3" ht="46.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -7785,7 +7590,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
@@ -7805,14 +7610,14 @@
         <v>2</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="H4" s="22">
         <f>F4*G4</f>
         <v>500</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J4" s="22">
         <v>8</v>
@@ -7856,7 +7661,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -7944,16 +7749,16 @@
         <v>18386.775</v>
       </c>
       <c r="AS4" s="27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
+      <c r="AU4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AV4" t="s" s="1">
-        <v>232</v>
+      <c r="AV4" s="1" t="s">
+        <v>155</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -7991,17 +7796,17 @@
       <c r="BJ4" s="28"/>
       <c r="BK4" s="28"/>
       <c r="BL4" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="BM4" t="s" s="1">
-        <v>250</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>249</v>
+        <v>156</v>
+      </c>
+      <c r="BM4" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="BN4" s="1" t="s">
+        <v>184</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>18386.775</v>
+        <v>18386.80739</v>
       </c>
       <c r="BP4" s="34">
         <f>BN4+AW4</f>
@@ -8331,13 +8136,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -8538,15 +8343,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -8558,14 +8363,14 @@
         <v>2</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="H4" s="22">
         <f>F4*G4</f>
         <v>500</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J4" s="22">
         <v>8</v>
@@ -8609,7 +8414,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -8697,16 +8502,16 @@
         <v>18386.775</v>
       </c>
       <c r="AS4" s="27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="AV4" s="23" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -8744,13 +8549,13 @@
       <c r="BJ4" s="28"/>
       <c r="BK4" s="28"/>
       <c r="BL4" s="33" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="BM4" s="23" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="BN4" s="23" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -9091,13 +8896,13 @@
     </row>
     <row r="3" ht="46.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -9303,10 +9108,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -9369,7 +9174,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -9457,16 +9262,16 @@
         <v>18386.775</v>
       </c>
       <c r="AS4" s="27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
+      <c r="AU4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AV4" t="s" s="1">
-        <v>232</v>
+      <c r="AV4" s="1" t="s">
+        <v>155</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -9504,17 +9309,17 @@
       <c r="BJ4" s="28"/>
       <c r="BK4" s="28"/>
       <c r="BL4" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="BM4" t="s" s="1">
-        <v>267</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>266</v>
+        <v>156</v>
+      </c>
+      <c r="BM4" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="BN4" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>18386.775</v>
+        <v>18386.79818</v>
       </c>
       <c r="BP4" s="34">
         <f>BN4+AW4</f>
@@ -9524,7 +9329,7 @@
         <v>123562</v>
       </c>
     </row>
-    <row r="5" spans="1:69">
+    <row r="5" ht="15.75" spans="1:69">
       <c r="A5" s="5"/>
       <c r="B5" s="36"/>
       <c r="C5" s="36"/>
@@ -9851,13 +9656,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -10063,10 +9868,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
@@ -10217,16 +10022,16 @@
         <v>18386.775</v>
       </c>
       <c r="AS4" s="27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
       <c r="AU4" s="23" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="AV4" s="23" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -10264,13 +10069,13 @@
       <c r="BJ4" s="28"/>
       <c r="BK4" s="28"/>
       <c r="BL4" s="33" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="BM4" s="23" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="BN4" s="23" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -10481,7 +10286,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="54" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="H7" s="55"/>
       <c r="I7" s="56">
@@ -10492,7 +10297,7 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="57" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="N7" s="58"/>
       <c r="O7" s="58"/>
@@ -10541,10 +10346,10 @@
       <c r="BF7" s="5"/>
       <c r="BG7" s="5"/>
       <c r="BH7" s="5" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="BI7" s="147" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="BJ7" s="5"/>
       <c r="BK7" s="5"/>
@@ -10563,7 +10368,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="54" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="H8" s="55"/>
       <c r="I8" s="56">
@@ -10583,7 +10388,7 @@
         <v>2</v>
       </c>
       <c r="P8" s="60" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
@@ -10629,10 +10434,10 @@
       <c r="BF8" s="5"/>
       <c r="BG8" s="5"/>
       <c r="BH8" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="BI8" s="147" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="BJ8" s="5"/>
       <c r="BK8" s="5"/>
@@ -10651,7 +10456,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="54" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="H9" s="55"/>
       <c r="I9" s="56">
@@ -10671,7 +10476,7 @@
         <v>2.5</v>
       </c>
       <c r="P9" s="20" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
@@ -10735,7 +10540,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="54" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="H10" s="55"/>
       <c r="I10" s="56">
@@ -10749,13 +10554,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="O10" s="20">
         <v>0.001</v>
       </c>
       <c r="P10" s="20" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="Q10" s="5"/>
       <c r="R10" s="5"/>
@@ -10819,7 +10624,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="54" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="H11" s="55"/>
       <c r="I11" s="61">
@@ -10953,10 +10758,10 @@
       <c r="BK12" s="5"/>
       <c r="BL12" s="5"/>
       <c r="BM12" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="BN12" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="BO12" s="5"/>
       <c r="BP12" s="6"/>
@@ -11026,7 +10831,7 @@
       <c r="BI13" s="5"/>
       <c r="BJ13" s="5"/>
       <c r="BK13" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="BL13" s="5">
         <v>12.5</v>
@@ -11107,7 +10912,7 @@
       <c r="BI14" s="5"/>
       <c r="BJ14" s="5"/>
       <c r="BK14" s="5" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="BL14" s="5">
         <v>487.4072</v>
@@ -11185,7 +10990,7 @@
       <c r="BI15" s="5"/>
       <c r="BJ15" s="5"/>
       <c r="BK15" s="5" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="BL15" s="5">
         <v>37.5</v>
@@ -11260,7 +11065,7 @@
       <c r="BI16" s="5"/>
       <c r="BJ16" s="5"/>
       <c r="BK16" s="5" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="BL16" s="5">
         <v>487.4072</v>
@@ -11833,21 +11638,21 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -11904,7 +11709,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -11992,16 +11797,16 @@
         <v>55159.9</v>
       </c>
       <c r="AS4" s="6" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
+      <c r="AU4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AV4" t="s" s="1">
-        <v>255</v>
+      <c r="AV4" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -12039,17 +11844,17 @@
       <c r="BJ4" s="6"/>
       <c r="BK4" s="6"/>
       <c r="BL4" s="28" t="s">
-        <v>150</v>
-      </c>
-      <c r="BM4" t="s" s="1">
-        <v>257</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>256</v>
+        <v>156</v>
+      </c>
+      <c r="BM4" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="BN4" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>55159.9</v>
+        <v>55159.94877</v>
       </c>
       <c r="BP4" s="34">
         <f>BN4+AW4</f>
@@ -12373,13 +12178,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -12580,34 +12385,34 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="H4" s="22">
         <f>F4*G4</f>
         <v>750</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J4" s="22">
         <v>8</v>
@@ -12651,7 +12456,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -12739,16 +12544,16 @@
         <v>55159.9</v>
       </c>
       <c r="AS4" s="27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
+      <c r="AU4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AV4" t="s" s="1">
-        <v>255</v>
+      <c r="AV4" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -12786,17 +12591,17 @@
       <c r="BJ4" s="28"/>
       <c r="BK4" s="28"/>
       <c r="BL4" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="BM4" t="s" s="1">
-        <v>259</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>258</v>
+        <v>156</v>
+      </c>
+      <c r="BM4" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="BN4" s="1" t="s">
+        <v>194</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>55159.9</v>
+        <v>55159.9875</v>
       </c>
       <c r="BP4" s="34">
         <f>BN4+AW4</f>
@@ -13125,13 +12930,13 @@
     </row>
     <row r="3" ht="61.5" spans="1:69">
       <c r="A3" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>5</v>
@@ -13332,21 +13137,21 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:69">
+    <row r="4" spans="1:69">
       <c r="A4" s="20">
         <v>1</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F4" s="22">
         <v>3</v>
@@ -13403,7 +13208,7 @@
         <v>88363222</v>
       </c>
       <c r="U4" s="22">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="22">
         <f>IF(OR($C$2=1,$C$2=4),ROUND((((S4*U4)/100)/2),2),0)</f>
@@ -13491,16 +13296,16 @@
         <v>55159.9</v>
       </c>
       <c r="AS4" s="27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="AT4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AU4" t="s" s="1">
+      <c r="AU4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AV4" t="s" s="1">
-        <v>255</v>
+      <c r="AV4" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="AW4" s="28">
         <f>AM4</f>
@@ -13538,17 +13343,17 @@
       <c r="BJ4" s="28"/>
       <c r="BK4" s="28"/>
       <c r="BL4" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="BM4" t="s" s="1">
-        <v>260</v>
-      </c>
-      <c r="BN4" t="s" s="1">
-        <v>194</v>
+        <v>156</v>
+      </c>
+      <c r="BM4" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="BN4" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
-        <v>55159.9</v>
+        <v>55159.9601</v>
       </c>
       <c r="BP4" s="34">
         <f>BN4+AW4</f>
@@ -15767,7 +15572,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
@@ -15838,7 +15643,7 @@
         <v>88363222</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -18210,7 +18015,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
@@ -18281,7 +18086,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -18419,14 +18224,14 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>134</v>
+        <v>202</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>8572.52323</v>
+        <v>20068.08768</v>
       </c>
       <c r="BP23" s="106">
         <f>BN23+AW23</f>
@@ -20650,15 +20455,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
       <c r="B23" s="44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C23" s="44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D23" s="88" t="s">
         <v>12</v>
@@ -20721,7 +20526,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -23076,15 +22881,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
       <c r="B23" s="88" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C23" s="88" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D23" s="88" t="s">
         <v>12</v>
@@ -23103,7 +22908,7 @@
         <v>500</v>
       </c>
       <c r="I23" t="s" s="0">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J23" s="104">
         <v>2</v>
@@ -23147,7 +22952,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -23285,14 +23090,14 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>270</v>
+        <v>203</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>8482.8221</v>
+        <v>20046.0947</v>
       </c>
       <c r="BP23" s="106">
         <f>BN23+AW23</f>
@@ -25516,15 +25321,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
       <c r="B23" s="88" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C23" s="88" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D23" s="88" t="s">
         <v>12</v>
@@ -25543,7 +25348,7 @@
         <v>500</v>
       </c>
       <c r="I23" t="s" s="0">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J23" s="104">
         <v>2</v>
@@ -25587,7 +25392,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -27948,21 +27753,21 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
       <c r="B23" s="44" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C23" s="44" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D23" s="88" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="88" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F23" s="103">
         <v>3</v>
@@ -28019,7 +27824,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -28116,7 +27921,7 @@
         <v>113</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="AW23" s="104">
         <f>AM23</f>
@@ -28157,14 +27962,14 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>143</v>
+        <v>206</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>271</v>
+        <v>205</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>9181.28366</v>
+        <v>60106.32358</v>
       </c>
       <c r="BP23" s="106">
         <f>BN23+AW23</f>
@@ -30388,15 +30193,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
       <c r="B23" s="44" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C23" s="44" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D23" s="88" t="s">
         <v>12</v>
@@ -30459,7 +30264,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -30556,7 +30361,7 @@
         <v>113</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="AW23" s="104">
         <f>AM23</f>
@@ -30597,14 +30402,14 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>216</v>
+        <v>150</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>26398.17586</v>
+        <v>60307.28666</v>
       </c>
       <c r="BP23" s="106">
         <f>BN23+AW23</f>
@@ -32828,15 +32633,15 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:69">
+    <row r="23" spans="1:69">
       <c r="A23" s="88">
         <v>1</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D23" s="88" t="s">
         <v>12</v>
@@ -32855,7 +32660,7 @@
         <v>750</v>
       </c>
       <c r="I23" t="s" s="0">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J23" s="104">
         <v>2</v>
@@ -32899,7 +32704,7 @@
         <v>111</v>
       </c>
       <c r="U23" s="105">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V23" s="105">
         <f>IF(OR($C$21=1,$C$21=4),ROUND((((S23*U23)/100)/2),2),0)</f>
@@ -32996,7 +32801,7 @@
         <v>113</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="AW23" s="104">
         <f>AM23</f>
@@ -33037,14 +32842,14 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>25610.66503</v>
+        <v>60257.31958</v>
       </c>
       <c r="BP23" s="108">
         <f>BN23+AW23</f>

</xml_diff>

<commit_message>
Updated LOV select scripts and locator changes
Updated LOV select scripts and locator changes
</commit_message>
<xml_diff>
--- a/testdata/ImportGRN.xlsx
+++ b/testdata/ImportGRN.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2510" uniqueCount="219">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -665,6 +665,42 @@
   </si>
   <si>
     <t>60106.32358</t>
+  </si>
+  <si>
+    <t>519</t>
+  </si>
+  <si>
+    <t>17559.34092</t>
+  </si>
+  <si>
+    <t>556</t>
+  </si>
+  <si>
+    <t>8048.84496</t>
+  </si>
+  <si>
+    <t>521</t>
+  </si>
+  <si>
+    <t>17562.52051</t>
+  </si>
+  <si>
+    <t>558</t>
+  </si>
+  <si>
+    <t>8048.37204</t>
+  </si>
+  <si>
+    <t>560</t>
+  </si>
+  <si>
+    <t>8047.9025</t>
+  </si>
+  <si>
+    <t>530</t>
+  </si>
+  <si>
+    <t>20062.88319</t>
   </si>
 </sst>
 </file>
@@ -4570,10 +4606,10 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="BO23" s="121">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -5334,10 +5370,10 @@
         <v>156</v>
       </c>
       <c r="BM4" t="s" s="1">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="BN4" t="s" s="1">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="BO4" s="28">
         <f>ROUND((((AW4*AZ4)+(BN4*BM4))/(AW4+BN4)),5)</f>
@@ -18224,10 +18260,10 @@
         <v>119</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>202</v>
+        <v>218</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="BO23" s="104">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>